<commit_message>
Update Planeación - Armonización de Encuestas de Hogares.xlsx
</commit_message>
<xml_diff>
--- a/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
+++ b/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/dcor_iadb_org/Documents/Documents/GitHub/calculo_indicators_R/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2920" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5A44597-22A4-4F83-821C-B1BF7F2A35BD}"/>
+  <xr:revisionPtr revIDLastSave="2925" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81AEAA9F-C0AA-4AA7-80FD-935D0106705D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Encuestas Armonizadas" sheetId="2" state="hidden" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="507">
   <si>
     <t>Harmonized Household Survey Databases of LAC</t>
   </si>
@@ -1597,6 +1597,9 @@
   </si>
   <si>
     <t>m1</t>
+  </si>
+  <si>
+    <t>2023</t>
   </si>
 </sst>
 </file>
@@ -2592,34 +2595,25 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2652,6 +2646,15 @@
     <xf numFmtId="0" fontId="14" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2679,16 +2682,28 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2700,18 +2715,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="ANCLAS,REZONES Y SUS PARTES,DE FUNDICION,DE HIERRO O DE ACERO" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2721,7 +2724,38 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="45">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -5272,49 +5306,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}" name="Table13" displayName="Table13" ref="A1:AN89" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41" totalsRowBorderDxfId="40" headerRowCellStyle="Normal 2">
-  <autoFilter ref="A1:AN89" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}"/>
-  <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{6B064E87-3A0D-4584-8192-35267E66F273}" name="País" dataDxfId="39" dataCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{56390F1F-7512-4FEB-8AF3-898CDB1A9830}" name="Encuesta" dataDxfId="38"/>
-    <tableColumn id="38" xr3:uid="{76878665-537D-4B41-A64B-EA91CAA67E30}" name="access_right" dataDxfId="37" dataCellStyle="Normal 2"/>
-    <tableColumn id="3" xr3:uid="{6E24555E-9D4B-4EA9-B227-AC82DC996508}" name="Ronda armonizada BID" dataDxfId="36" dataCellStyle="Normal 2"/>
-    <tableColumn id="4" xr3:uid="{45B11BB2-5A64-4216-9E23-B09064B5C3D2}" name="1986" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{04A2DE59-1034-4485-AEBE-2132D54461E9}" name="1989" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{EAEE1B18-887D-43BC-8727-9C2CE724633C}" name="1990" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{2F33A639-9FAC-4DD3-9BFC-CA80A8657ECF}" name="1991" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{A1761052-3159-42ED-8624-97098C6DC00B}" name="1992" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{42773BA5-F2A0-4A78-A2F8-53E0EE22B9D1}" name="1993" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{67D3E1B3-E4EA-4C9C-9A36-8A6708B6D014}" name="1994" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{9EDB3DE7-CCC0-4F5E-AE35-F4128DD66F39}" name="1995" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{A93F6D39-B7E5-4461-A449-F7F40B9487C6}" name="1996" dataDxfId="27"/>
-    <tableColumn id="13" xr3:uid="{F2DE6F08-B56D-4265-AF23-0C514E64DE66}" name="1997" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{D6B69F96-5C92-432A-BAFD-FEE8EEAECCF7}" name="1998" dataDxfId="25"/>
-    <tableColumn id="15" xr3:uid="{224E7F10-B175-477F-B101-6E70FB191A01}" name="1999" dataDxfId="24"/>
-    <tableColumn id="16" xr3:uid="{15F72C33-3221-4279-A0CA-542684BB589E}" name="2000" dataDxfId="23"/>
-    <tableColumn id="17" xr3:uid="{BDE0486B-DE3F-4D08-9ACF-0616D1D50D4D}" name="2001" dataDxfId="22"/>
-    <tableColumn id="18" xr3:uid="{28FF96DB-7C31-4BFC-8548-98EF95161CFB}" name="2002" dataDxfId="21"/>
-    <tableColumn id="19" xr3:uid="{2FA8F5BF-F645-4E81-A847-003D0E90C20F}" name="2003" dataDxfId="20"/>
-    <tableColumn id="20" xr3:uid="{BCAB11DC-8BFA-42B6-9207-397B91E0B1C6}" name="2004" dataDxfId="19"/>
-    <tableColumn id="21" xr3:uid="{17C2EC16-AE6A-4666-B47F-466CE1B378D5}" name="2005" dataDxfId="18"/>
-    <tableColumn id="22" xr3:uid="{04F6B276-FCD1-401A-836E-177259B63A59}" name="2006" dataDxfId="17"/>
-    <tableColumn id="23" xr3:uid="{B8B96EF9-EDFC-44DA-BC31-74726BE33B55}" name="2007" dataDxfId="16"/>
-    <tableColumn id="24" xr3:uid="{E0460942-F274-4768-BF69-B887C868E5EC}" name="2008" dataDxfId="15"/>
-    <tableColumn id="25" xr3:uid="{AD6CFE48-D83D-4F93-9F8B-B2BBEF937BAB}" name="2009" dataDxfId="14"/>
-    <tableColumn id="26" xr3:uid="{7E598DF3-D7AE-4E66-AEB6-C288D8C67A98}" name="2010" dataDxfId="13"/>
-    <tableColumn id="27" xr3:uid="{0DA6D22D-AAA5-484F-B916-0AEAB0E1BA51}" name="2011" dataDxfId="12"/>
-    <tableColumn id="28" xr3:uid="{401D8801-8B1D-45B2-ABFD-F63694636C40}" name="2012" dataDxfId="11"/>
-    <tableColumn id="29" xr3:uid="{B2F8A0D3-26CD-4E4B-8FAB-2CEE94A0DA7A}" name="2013" dataDxfId="10"/>
-    <tableColumn id="30" xr3:uid="{AA7B0439-D20C-43DD-8146-5E5730473AB6}" name="2014" dataDxfId="9" dataCellStyle="Normal 2"/>
-    <tableColumn id="31" xr3:uid="{90B20A4D-DBF3-4729-AEBF-A464C2AB96ED}" name="2015" dataDxfId="8" dataCellStyle="Normal 2"/>
-    <tableColumn id="32" xr3:uid="{37632C06-0D2B-4432-A247-87237DD99DD7}" name="2016" dataDxfId="7"/>
-    <tableColumn id="33" xr3:uid="{0E571E7E-B684-4111-9B7B-D0D871EBC2BF}" name="2017" dataDxfId="6"/>
-    <tableColumn id="34" xr3:uid="{8F53FB35-C7B2-441A-BE88-62954F5D5B33}" name="2018" dataDxfId="5"/>
-    <tableColumn id="35" xr3:uid="{C8F8A85B-85AD-444C-92E1-1CA28B02F84B}" name="2019" dataDxfId="4"/>
-    <tableColumn id="36" xr3:uid="{1E2AD377-CC74-44E0-8152-9BA191ED06D8}" name="2020" dataDxfId="3"/>
-    <tableColumn id="37" xr3:uid="{B7A3A7EC-85D3-46A0-9981-6CA826A96680}" name="2021" dataDxfId="2" dataCellStyle="Normal 2"/>
-    <tableColumn id="40" xr3:uid="{537B0D14-850C-419A-B1CB-4E97FC19D51D}" name="2022" dataDxfId="1" dataCellStyle="Normal 2"/>
-    <tableColumn id="39" xr3:uid="{1D919B70-6E05-471A-A9D1-CD8C8D73D2BF}" name="Total" dataDxfId="0" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}" name="Table13" displayName="Table13" ref="A1:AO89" totalsRowShown="0" headerRowDxfId="44" headerRowBorderDxfId="43" tableBorderDxfId="42" totalsRowBorderDxfId="41" headerRowCellStyle="Normal 2">
+  <autoFilter ref="A1:AO89" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}"/>
+  <tableColumns count="41">
+    <tableColumn id="1" xr3:uid="{6B064E87-3A0D-4584-8192-35267E66F273}" name="País" dataDxfId="40" dataCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{56390F1F-7512-4FEB-8AF3-898CDB1A9830}" name="Encuesta" dataDxfId="39"/>
+    <tableColumn id="38" xr3:uid="{76878665-537D-4B41-A64B-EA91CAA67E30}" name="access_right" dataDxfId="38" dataCellStyle="Normal 2"/>
+    <tableColumn id="3" xr3:uid="{6E24555E-9D4B-4EA9-B227-AC82DC996508}" name="Ronda armonizada BID" dataDxfId="37" dataCellStyle="Normal 2"/>
+    <tableColumn id="4" xr3:uid="{45B11BB2-5A64-4216-9E23-B09064B5C3D2}" name="1986" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{04A2DE59-1034-4485-AEBE-2132D54461E9}" name="1989" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{EAEE1B18-887D-43BC-8727-9C2CE724633C}" name="1990" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{2F33A639-9FAC-4DD3-9BFC-CA80A8657ECF}" name="1991" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{A1761052-3159-42ED-8624-97098C6DC00B}" name="1992" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{42773BA5-F2A0-4A78-A2F8-53E0EE22B9D1}" name="1993" dataDxfId="31"/>
+    <tableColumn id="10" xr3:uid="{67D3E1B3-E4EA-4C9C-9A36-8A6708B6D014}" name="1994" dataDxfId="30"/>
+    <tableColumn id="11" xr3:uid="{9EDB3DE7-CCC0-4F5E-AE35-F4128DD66F39}" name="1995" dataDxfId="29"/>
+    <tableColumn id="12" xr3:uid="{A93F6D39-B7E5-4461-A449-F7F40B9487C6}" name="1996" dataDxfId="28"/>
+    <tableColumn id="13" xr3:uid="{F2DE6F08-B56D-4265-AF23-0C514E64DE66}" name="1997" dataDxfId="27"/>
+    <tableColumn id="14" xr3:uid="{D6B69F96-5C92-432A-BAFD-FEE8EEAECCF7}" name="1998" dataDxfId="26"/>
+    <tableColumn id="15" xr3:uid="{224E7F10-B175-477F-B101-6E70FB191A01}" name="1999" dataDxfId="25"/>
+    <tableColumn id="16" xr3:uid="{15F72C33-3221-4279-A0CA-542684BB589E}" name="2000" dataDxfId="24"/>
+    <tableColumn id="17" xr3:uid="{BDE0486B-DE3F-4D08-9ACF-0616D1D50D4D}" name="2001" dataDxfId="23"/>
+    <tableColumn id="18" xr3:uid="{28FF96DB-7C31-4BFC-8548-98EF95161CFB}" name="2002" dataDxfId="22"/>
+    <tableColumn id="19" xr3:uid="{2FA8F5BF-F645-4E81-A847-003D0E90C20F}" name="2003" dataDxfId="21"/>
+    <tableColumn id="20" xr3:uid="{BCAB11DC-8BFA-42B6-9207-397B91E0B1C6}" name="2004" dataDxfId="20"/>
+    <tableColumn id="21" xr3:uid="{17C2EC16-AE6A-4666-B47F-466CE1B378D5}" name="2005" dataDxfId="19"/>
+    <tableColumn id="22" xr3:uid="{04F6B276-FCD1-401A-836E-177259B63A59}" name="2006" dataDxfId="18"/>
+    <tableColumn id="23" xr3:uid="{B8B96EF9-EDFC-44DA-BC31-74726BE33B55}" name="2007" dataDxfId="17"/>
+    <tableColumn id="24" xr3:uid="{E0460942-F274-4768-BF69-B887C868E5EC}" name="2008" dataDxfId="16"/>
+    <tableColumn id="25" xr3:uid="{AD6CFE48-D83D-4F93-9F8B-B2BBEF937BAB}" name="2009" dataDxfId="15"/>
+    <tableColumn id="26" xr3:uid="{7E598DF3-D7AE-4E66-AEB6-C288D8C67A98}" name="2010" dataDxfId="14"/>
+    <tableColumn id="27" xr3:uid="{0DA6D22D-AAA5-484F-B916-0AEAB0E1BA51}" name="2011" dataDxfId="13"/>
+    <tableColumn id="28" xr3:uid="{401D8801-8B1D-45B2-ABFD-F63694636C40}" name="2012" dataDxfId="12"/>
+    <tableColumn id="29" xr3:uid="{B2F8A0D3-26CD-4E4B-8FAB-2CEE94A0DA7A}" name="2013" dataDxfId="11"/>
+    <tableColumn id="30" xr3:uid="{AA7B0439-D20C-43DD-8146-5E5730473AB6}" name="2014" dataDxfId="10" dataCellStyle="Normal 2"/>
+    <tableColumn id="31" xr3:uid="{90B20A4D-DBF3-4729-AEBF-A464C2AB96ED}" name="2015" dataDxfId="9" dataCellStyle="Normal 2"/>
+    <tableColumn id="32" xr3:uid="{37632C06-0D2B-4432-A247-87237DD99DD7}" name="2016" dataDxfId="8"/>
+    <tableColumn id="33" xr3:uid="{0E571E7E-B684-4111-9B7B-D0D871EBC2BF}" name="2017" dataDxfId="7"/>
+    <tableColumn id="34" xr3:uid="{8F53FB35-C7B2-441A-BE88-62954F5D5B33}" name="2018" dataDxfId="6"/>
+    <tableColumn id="35" xr3:uid="{C8F8A85B-85AD-444C-92E1-1CA28B02F84B}" name="2019" dataDxfId="5"/>
+    <tableColumn id="36" xr3:uid="{1E2AD377-CC74-44E0-8152-9BA191ED06D8}" name="2020" dataDxfId="4"/>
+    <tableColumn id="37" xr3:uid="{B7A3A7EC-85D3-46A0-9981-6CA826A96680}" name="2021" dataDxfId="3" dataCellStyle="Normal 2"/>
+    <tableColumn id="40" xr3:uid="{537B0D14-850C-419A-B1CB-4E97FC19D51D}" name="2022" dataDxfId="2" dataCellStyle="Normal 2"/>
+    <tableColumn id="41" xr3:uid="{045F6C2A-BE9D-402E-9DFC-1CC0BEE2F90C}" name="2023" dataDxfId="0" dataCellStyle="Normal 2"/>
+    <tableColumn id="39" xr3:uid="{1D919B70-6E05-471A-A9D1-CD8C8D73D2BF}" name="Total" dataDxfId="1" dataCellStyle="Normal 2">
       <calculatedColumnFormula>SUM(Table13[[#This Row],[1986]:[2021]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5633,44 +5668,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:75" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="B1" s="191" t="s">
+      <c r="B1" s="186" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="191"/>
-      <c r="D1" s="191"/>
-      <c r="E1" s="191"/>
-      <c r="F1" s="191"/>
-      <c r="G1" s="191"/>
-      <c r="H1" s="191"/>
-      <c r="I1" s="191"/>
-      <c r="J1" s="191"/>
-      <c r="K1" s="191"/>
-      <c r="L1" s="191"/>
-      <c r="M1" s="191"/>
-      <c r="N1" s="191"/>
-      <c r="O1" s="191"/>
-      <c r="P1" s="191"/>
-      <c r="Q1" s="191"/>
-      <c r="R1" s="191"/>
-      <c r="S1" s="191"/>
-      <c r="T1" s="191"/>
-      <c r="U1" s="191"/>
-      <c r="V1" s="191"/>
-      <c r="W1" s="191"/>
-      <c r="X1" s="191"/>
-      <c r="Y1" s="191"/>
-      <c r="Z1" s="191"/>
-      <c r="AA1" s="191"/>
-      <c r="AB1" s="191"/>
-      <c r="AC1" s="191"/>
-      <c r="AD1" s="191"/>
-      <c r="AE1" s="191"/>
-      <c r="AF1" s="191"/>
-      <c r="AG1" s="191"/>
-      <c r="AH1" s="191"/>
-      <c r="AI1" s="191"/>
-      <c r="AJ1" s="191"/>
-      <c r="AK1" s="191"/>
+      <c r="C1" s="186"/>
+      <c r="D1" s="186"/>
+      <c r="E1" s="186"/>
+      <c r="F1" s="186"/>
+      <c r="G1" s="186"/>
+      <c r="H1" s="186"/>
+      <c r="I1" s="186"/>
+      <c r="J1" s="186"/>
+      <c r="K1" s="186"/>
+      <c r="L1" s="186"/>
+      <c r="M1" s="186"/>
+      <c r="N1" s="186"/>
+      <c r="O1" s="186"/>
+      <c r="P1" s="186"/>
+      <c r="Q1" s="186"/>
+      <c r="R1" s="186"/>
+      <c r="S1" s="186"/>
+      <c r="T1" s="186"/>
+      <c r="U1" s="186"/>
+      <c r="V1" s="186"/>
+      <c r="W1" s="186"/>
+      <c r="X1" s="186"/>
+      <c r="Y1" s="186"/>
+      <c r="Z1" s="186"/>
+      <c r="AA1" s="186"/>
+      <c r="AB1" s="186"/>
+      <c r="AC1" s="186"/>
+      <c r="AD1" s="186"/>
+      <c r="AE1" s="186"/>
+      <c r="AF1" s="186"/>
+      <c r="AG1" s="186"/>
+      <c r="AH1" s="186"/>
+      <c r="AI1" s="186"/>
+      <c r="AJ1" s="186"/>
+      <c r="AK1" s="186"/>
       <c r="AL1" s="51"/>
       <c r="AM1" s="83"/>
       <c r="AN1" s="51"/>
@@ -5839,7 +5874,7 @@
       <c r="A3" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="186" t="s">
+      <c r="B3" s="188" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="57" t="s">
@@ -5933,7 +5968,7 @@
     </row>
     <row r="4" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="145"/>
-      <c r="B4" s="187"/>
+      <c r="B4" s="189"/>
       <c r="C4" s="57" t="s">
         <v>14</v>
       </c>
@@ -6169,7 +6204,7 @@
       <c r="A7" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="189" t="s">
+      <c r="B7" s="190" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="57" t="s">
@@ -6265,7 +6300,7 @@
     </row>
     <row r="8" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="145"/>
-      <c r="B8" s="189"/>
+      <c r="B8" s="190"/>
       <c r="C8" s="57" t="s">
         <v>26</v>
       </c>
@@ -6323,7 +6358,7 @@
     </row>
     <row r="9" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="145"/>
-      <c r="B9" s="189"/>
+      <c r="B9" s="190"/>
       <c r="C9" s="57" t="s">
         <v>27</v>
       </c>
@@ -6373,7 +6408,7 @@
     </row>
     <row r="10" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="145"/>
-      <c r="B10" s="189" t="s">
+      <c r="B10" s="190" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="39" t="s">
@@ -6467,7 +6502,7 @@
       <c r="A11" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="189"/>
+      <c r="B11" s="190"/>
       <c r="C11" s="39" t="s">
         <v>30</v>
       </c>
@@ -6703,7 +6738,7 @@
     </row>
     <row r="14" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="145"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="188" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="39" t="s">
@@ -6761,7 +6796,7 @@
     </row>
     <row r="15" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="145"/>
-      <c r="B15" s="188"/>
+      <c r="B15" s="191"/>
       <c r="C15" s="39" t="s">
         <v>39</v>
       </c>
@@ -6809,7 +6844,7 @@
     </row>
     <row r="16" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="145"/>
-      <c r="B16" s="188"/>
+      <c r="B16" s="191"/>
       <c r="C16" s="39" t="s">
         <v>40</v>
       </c>
@@ -6881,7 +6916,7 @@
       <c r="A17" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B17" s="187"/>
+      <c r="B17" s="189"/>
       <c r="C17" s="39" t="s">
         <v>41</v>
       </c>
@@ -6967,7 +7002,7 @@
     </row>
     <row r="18" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="145"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="188" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="41" t="s">
@@ -7057,7 +7092,7 @@
       <c r="A19" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B19" s="187"/>
+      <c r="B19" s="189"/>
       <c r="C19" s="57" t="s">
         <v>45</v>
       </c>
@@ -7135,7 +7170,7 @@
     </row>
     <row r="20" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="145"/>
-      <c r="B20" s="186" t="s">
+      <c r="B20" s="188" t="s">
         <v>48</v>
       </c>
       <c r="C20" s="57" t="s">
@@ -7225,7 +7260,7 @@
       <c r="A21" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B21" s="187"/>
+      <c r="B21" s="189"/>
       <c r="C21" s="57" t="s">
         <v>50</v>
       </c>
@@ -7289,7 +7324,7 @@
       <c r="A22" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B22" s="189" t="s">
+      <c r="B22" s="190" t="s">
         <v>53</v>
       </c>
       <c r="C22" s="57" t="s">
@@ -7409,7 +7444,7 @@
     </row>
     <row r="23" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="145"/>
-      <c r="B23" s="189"/>
+      <c r="B23" s="190"/>
       <c r="C23" s="57" t="s">
         <v>57</v>
       </c>
@@ -7463,7 +7498,7 @@
     </row>
     <row r="24" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="145"/>
-      <c r="B24" s="189" t="s">
+      <c r="B24" s="190" t="s">
         <v>58</v>
       </c>
       <c r="C24" s="57" t="s">
@@ -7519,7 +7554,7 @@
       <c r="A25" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="189"/>
+      <c r="B25" s="190"/>
       <c r="C25" s="57" t="s">
         <v>60</v>
       </c>
@@ -7601,7 +7636,7 @@
     </row>
     <row r="26" spans="1:42" ht="12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="145"/>
-      <c r="B26" s="189"/>
+      <c r="B26" s="190"/>
       <c r="C26" s="57" t="s">
         <v>62</v>
       </c>
@@ -7771,7 +7806,7 @@
       <c r="A28" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B28" s="186" t="s">
+      <c r="B28" s="188" t="s">
         <v>65</v>
       </c>
       <c r="C28" s="57" t="s">
@@ -7875,7 +7910,7 @@
     </row>
     <row r="29" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="145"/>
-      <c r="B29" s="187"/>
+      <c r="B29" s="189"/>
       <c r="C29" s="57" t="s">
         <v>67</v>
       </c>
@@ -8029,7 +8064,7 @@
     </row>
     <row r="31" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="145"/>
-      <c r="B31" s="186" t="s">
+      <c r="B31" s="188" t="s">
         <v>73</v>
       </c>
       <c r="C31" s="57" t="s">
@@ -8085,7 +8120,7 @@
       <c r="A32" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B32" s="187"/>
+      <c r="B32" s="189"/>
       <c r="C32" s="57" t="s">
         <v>74</v>
       </c>
@@ -8151,7 +8186,7 @@
     </row>
     <row r="33" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="145"/>
-      <c r="B33" s="186" t="s">
+      <c r="B33" s="188" t="s">
         <v>76</v>
       </c>
       <c r="C33" s="57" t="s">
@@ -8235,7 +8270,7 @@
       <c r="A34" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B34" s="187"/>
+      <c r="B34" s="189"/>
       <c r="C34" s="57" t="s">
         <v>44</v>
       </c>
@@ -8309,7 +8344,7 @@
     </row>
     <row r="35" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="145"/>
-      <c r="B35" s="186" t="s">
+      <c r="B35" s="188" t="s">
         <v>79</v>
       </c>
       <c r="C35" s="57" t="s">
@@ -8373,7 +8408,7 @@
     </row>
     <row r="36" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="145"/>
-      <c r="B36" s="188"/>
+      <c r="B36" s="191"/>
       <c r="C36" s="57" t="s">
         <v>26</v>
       </c>
@@ -8387,15 +8422,15 @@
       <c r="K36" s="80"/>
       <c r="L36" s="80"/>
       <c r="M36" s="80"/>
-      <c r="N36" s="192">
-        <v>1</v>
-      </c>
-      <c r="O36" s="192"/>
+      <c r="N36" s="187">
+        <v>1</v>
+      </c>
+      <c r="O36" s="187"/>
       <c r="P36" s="80"/>
-      <c r="Q36" s="192">
-        <v>1</v>
-      </c>
-      <c r="R36" s="192"/>
+      <c r="Q36" s="187">
+        <v>1</v>
+      </c>
+      <c r="R36" s="187"/>
       <c r="S36" s="80"/>
       <c r="T36" s="80"/>
       <c r="U36" s="80"/>
@@ -8425,7 +8460,7 @@
     </row>
     <row r="37" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="145"/>
-      <c r="B37" s="188"/>
+      <c r="B37" s="191"/>
       <c r="C37" s="57" t="s">
         <v>82</v>
       </c>
@@ -8509,7 +8544,7 @@
       <c r="A38" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B38" s="187"/>
+      <c r="B38" s="189"/>
       <c r="C38" s="57" t="s">
         <v>9</v>
       </c>
@@ -8573,7 +8608,7 @@
       <c r="A39" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B39" s="186" t="s">
+      <c r="B39" s="188" t="s">
         <v>83</v>
       </c>
       <c r="C39" s="57" t="s">
@@ -8679,7 +8714,7 @@
     </row>
     <row r="40" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="145"/>
-      <c r="B40" s="187"/>
+      <c r="B40" s="189"/>
       <c r="C40" s="57" t="s">
         <v>84</v>
       </c>
@@ -8969,7 +9004,7 @@
     </row>
     <row r="43" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="145"/>
-      <c r="B43" s="186" t="s">
+      <c r="B43" s="188" t="s">
         <v>87</v>
       </c>
       <c r="C43" s="57" t="s">
@@ -9071,7 +9106,7 @@
       <c r="A44" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B44" s="187"/>
+      <c r="B44" s="189"/>
       <c r="C44" s="41" t="s">
         <v>59</v>
       </c>
@@ -9583,43 +9618,43 @@
       </c>
     </row>
     <row r="58" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C58" s="190" t="s">
+      <c r="C58" s="192" t="s">
         <v>97</v>
       </c>
-      <c r="D58" s="190"/>
-      <c r="E58" s="190"/>
-      <c r="F58" s="190"/>
-      <c r="G58" s="190"/>
-      <c r="H58" s="190"/>
-      <c r="I58" s="190"/>
-      <c r="J58" s="190"/>
-      <c r="K58" s="190"/>
-      <c r="L58" s="190"/>
-      <c r="M58" s="190"/>
-      <c r="N58" s="190"/>
-      <c r="O58" s="190"/>
-      <c r="P58" s="190"/>
-      <c r="Q58" s="190"/>
-      <c r="R58" s="190"/>
-      <c r="S58" s="190"/>
-      <c r="T58" s="190"/>
-      <c r="U58" s="190"/>
-      <c r="V58" s="190"/>
-      <c r="W58" s="190"/>
-      <c r="X58" s="190"/>
-      <c r="Y58" s="190"/>
-      <c r="Z58" s="190"/>
-      <c r="AA58" s="190"/>
-      <c r="AB58" s="190"/>
-      <c r="AC58" s="190"/>
-      <c r="AD58" s="190"/>
-      <c r="AE58" s="190"/>
-      <c r="AF58" s="190"/>
-      <c r="AG58" s="190"/>
-      <c r="AH58" s="190"/>
-      <c r="AI58" s="190"/>
-      <c r="AJ58" s="190"/>
-      <c r="AK58" s="190"/>
+      <c r="D58" s="192"/>
+      <c r="E58" s="192"/>
+      <c r="F58" s="192"/>
+      <c r="G58" s="192"/>
+      <c r="H58" s="192"/>
+      <c r="I58" s="192"/>
+      <c r="J58" s="192"/>
+      <c r="K58" s="192"/>
+      <c r="L58" s="192"/>
+      <c r="M58" s="192"/>
+      <c r="N58" s="192"/>
+      <c r="O58" s="192"/>
+      <c r="P58" s="192"/>
+      <c r="Q58" s="192"/>
+      <c r="R58" s="192"/>
+      <c r="S58" s="192"/>
+      <c r="T58" s="192"/>
+      <c r="U58" s="192"/>
+      <c r="V58" s="192"/>
+      <c r="W58" s="192"/>
+      <c r="X58" s="192"/>
+      <c r="Y58" s="192"/>
+      <c r="Z58" s="192"/>
+      <c r="AA58" s="192"/>
+      <c r="AB58" s="192"/>
+      <c r="AC58" s="192"/>
+      <c r="AD58" s="192"/>
+      <c r="AE58" s="192"/>
+      <c r="AF58" s="192"/>
+      <c r="AG58" s="192"/>
+      <c r="AH58" s="192"/>
+      <c r="AI58" s="192"/>
+      <c r="AJ58" s="192"/>
+      <c r="AK58" s="192"/>
     </row>
     <row r="59" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C59" s="147" t="s">
@@ -9740,6 +9775,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C58:AK58"/>
     <mergeCell ref="B1:AK1"/>
     <mergeCell ref="Q36:R36"/>
     <mergeCell ref="B39:B40"/>
@@ -9756,8 +9793,6 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C58:AK58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" r:id="rId1"/>
@@ -12711,17 +12746,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC0F423-732A-4BB5-B708-202F80FAD9CB}">
-  <dimension ref="A1:AN89"/>
+  <dimension ref="A1:AO89"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="12" style="100" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.1796875" style="100" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="6" max="38" width="8.1796875" style="100" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.1796875" style="100" customWidth="1"/>
+    <col min="39" max="40" width="8.1796875" style="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" ht="24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:41" ht="24" x14ac:dyDescent="0.35">
       <c r="A1" s="174" t="s">
         <v>2</v>
       </c>
@@ -12839,11 +12874,14 @@
       <c r="AM1" s="179" t="s">
         <v>136</v>
       </c>
-      <c r="AN1" s="180" t="s">
+      <c r="AN1" s="179" t="s">
+        <v>506</v>
+      </c>
+      <c r="AO1" s="180" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A2" s="157" t="s">
         <v>8</v>
       </c>
@@ -12911,12 +12949,13 @@
       <c r="AK2" s="40"/>
       <c r="AL2" s="69"/>
       <c r="AM2" s="159"/>
-      <c r="AN2" s="158">
+      <c r="AN2" s="159"/>
+      <c r="AO2" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A3" s="157" t="s">
         <v>8</v>
       </c>
@@ -13002,12 +13041,13 @@
       <c r="AM3" s="159">
         <v>1</v>
       </c>
-      <c r="AN3" s="158">
+      <c r="AN3" s="159"/>
+      <c r="AO3" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A4" s="157" t="s">
         <v>8</v>
       </c>
@@ -13057,12 +13097,13 @@
       <c r="AK4" s="80"/>
       <c r="AL4" s="159"/>
       <c r="AM4" s="171"/>
-      <c r="AN4" s="160">
+      <c r="AN4" s="171"/>
+      <c r="AO4" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A5" s="157" t="s">
         <v>15</v>
       </c>
@@ -13134,12 +13175,13 @@
       <c r="AK5" s="40"/>
       <c r="AL5" s="69"/>
       <c r="AM5" s="159"/>
-      <c r="AN5" s="158">
+      <c r="AN5" s="159"/>
+      <c r="AO5" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A6" s="157" t="s">
         <v>20</v>
       </c>
@@ -13203,12 +13245,13 @@
       <c r="AK6" s="40"/>
       <c r="AL6" s="159"/>
       <c r="AM6" s="171"/>
-      <c r="AN6" s="160">
+      <c r="AN6" s="171"/>
+      <c r="AO6" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A7" s="157" t="s">
         <v>20</v>
       </c>
@@ -13266,12 +13309,13 @@
       <c r="AK7" s="80"/>
       <c r="AL7" s="69"/>
       <c r="AM7" s="159"/>
-      <c r="AN7" s="158">
+      <c r="AN7" s="159"/>
+      <c r="AO7" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A8" s="157" t="s">
         <v>20</v>
       </c>
@@ -13321,12 +13365,13 @@
       <c r="AK8" s="80"/>
       <c r="AL8" s="159"/>
       <c r="AM8" s="171"/>
-      <c r="AN8" s="160">
+      <c r="AN8" s="171"/>
+      <c r="AO8" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A9" s="157" t="s">
         <v>22</v>
       </c>
@@ -13380,12 +13425,13 @@
       <c r="AK9" s="40"/>
       <c r="AL9" s="69"/>
       <c r="AM9" s="159"/>
-      <c r="AN9" s="158">
+      <c r="AN9" s="159"/>
+      <c r="AO9" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A10" s="157" t="s">
         <v>22</v>
       </c>
@@ -13433,12 +13479,13 @@
       <c r="AK10" s="40"/>
       <c r="AL10" s="159"/>
       <c r="AM10" s="171"/>
-      <c r="AN10" s="160">
+      <c r="AN10" s="171"/>
+      <c r="AO10" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A11" s="157" t="s">
         <v>22</v>
       </c>
@@ -13486,12 +13533,13 @@
       <c r="AK11" s="40"/>
       <c r="AL11" s="159"/>
       <c r="AM11" s="171"/>
-      <c r="AN11" s="160">
+      <c r="AN11" s="171"/>
+      <c r="AO11" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A12" s="157" t="s">
         <v>22</v>
       </c>
@@ -13539,12 +13587,13 @@
       <c r="AK12" s="40"/>
       <c r="AL12" s="159"/>
       <c r="AM12" s="171"/>
-      <c r="AN12" s="160">
+      <c r="AN12" s="171"/>
+      <c r="AO12" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A13" s="157" t="s">
         <v>22</v>
       </c>
@@ -13592,12 +13641,13 @@
       <c r="AK13" s="40"/>
       <c r="AL13" s="69"/>
       <c r="AM13" s="159"/>
-      <c r="AN13" s="158">
+      <c r="AN13" s="159"/>
+      <c r="AO13" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A14" s="157" t="s">
         <v>22</v>
       </c>
@@ -13667,12 +13717,13 @@
         <v>1</v>
       </c>
       <c r="AM14" s="159"/>
-      <c r="AN14" s="158">
+      <c r="AN14" s="159"/>
+      <c r="AO14" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A15" s="157" t="s">
         <v>22</v>
       </c>
@@ -13736,12 +13787,13 @@
       <c r="AK15" s="40"/>
       <c r="AL15" s="159"/>
       <c r="AM15" s="171"/>
-      <c r="AN15" s="160">
+      <c r="AN15" s="171"/>
+      <c r="AO15" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A16" s="157" t="s">
         <v>28</v>
       </c>
@@ -13833,12 +13885,13 @@
       <c r="AK16" s="80"/>
       <c r="AL16" s="69"/>
       <c r="AM16" s="159"/>
-      <c r="AN16" s="158">
+      <c r="AN16" s="159"/>
+      <c r="AO16" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A17" s="157" t="s">
         <v>28</v>
       </c>
@@ -13900,12 +13953,13 @@
       <c r="AM17" s="159">
         <v>1</v>
       </c>
-      <c r="AN17" s="158">
+      <c r="AN17" s="159"/>
+      <c r="AO17" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A18" s="157" t="s">
         <v>32</v>
       </c>
@@ -13979,12 +14033,13 @@
       <c r="AK18" s="80"/>
       <c r="AL18" s="69"/>
       <c r="AM18" s="159"/>
-      <c r="AN18" s="158">
+      <c r="AN18" s="159"/>
+      <c r="AO18" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A19" s="157" t="s">
         <v>32</v>
       </c>
@@ -14034,12 +14089,13 @@
       <c r="AK19" s="80"/>
       <c r="AL19" s="159"/>
       <c r="AM19" s="171"/>
-      <c r="AN19" s="160">
+      <c r="AN19" s="171"/>
+      <c r="AO19" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A20" s="157" t="s">
         <v>34</v>
       </c>
@@ -14103,12 +14159,13 @@
       <c r="AK20" s="40"/>
       <c r="AL20" s="69"/>
       <c r="AM20" s="159"/>
-      <c r="AN20" s="158">
+      <c r="AN20" s="159"/>
+      <c r="AO20" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A21" s="157" t="s">
         <v>34</v>
       </c>
@@ -14164,12 +14221,13 @@
       </c>
       <c r="AL21" s="159"/>
       <c r="AM21" s="171"/>
-      <c r="AN21" s="160">
+      <c r="AN21" s="171"/>
+      <c r="AO21" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A22" s="157" t="s">
         <v>38</v>
       </c>
@@ -14239,12 +14297,13 @@
       <c r="AK22" s="40"/>
       <c r="AL22" s="69"/>
       <c r="AM22" s="159"/>
-      <c r="AN22" s="158">
+      <c r="AN22" s="159"/>
+      <c r="AO22" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A23" s="157" t="s">
         <v>38</v>
       </c>
@@ -14302,12 +14361,13 @@
       <c r="AK23" s="40"/>
       <c r="AL23" s="69"/>
       <c r="AM23" s="159"/>
-      <c r="AN23" s="158">
+      <c r="AN23" s="159"/>
+      <c r="AO23" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A24" s="157" t="s">
         <v>38</v>
       </c>
@@ -14385,12 +14445,13 @@
         <v>1</v>
       </c>
       <c r="AM24" s="159"/>
-      <c r="AN24" s="158">
+      <c r="AN24" s="159"/>
+      <c r="AO24" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A25" s="157" t="s">
         <v>38</v>
       </c>
@@ -14440,12 +14501,13 @@
       </c>
       <c r="AL25" s="159"/>
       <c r="AM25" s="171"/>
-      <c r="AN25" s="160">
+      <c r="AN25" s="171"/>
+      <c r="AO25" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A26" s="157" t="s">
         <v>43</v>
       </c>
@@ -14533,12 +14595,13 @@
       <c r="AK26" s="40"/>
       <c r="AL26" s="69"/>
       <c r="AM26" s="159"/>
-      <c r="AN26" s="158">
+      <c r="AN26" s="159"/>
+      <c r="AO26" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A27" s="157" t="s">
         <v>43</v>
       </c>
@@ -14612,12 +14675,13 @@
       <c r="AM27" s="159">
         <v>1</v>
       </c>
-      <c r="AN27" s="158">
+      <c r="AN27" s="159"/>
+      <c r="AO27" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A28" s="157" t="s">
         <v>48</v>
       </c>
@@ -14667,12 +14731,13 @@
       <c r="AK28" s="80"/>
       <c r="AL28" s="159"/>
       <c r="AM28" s="171"/>
-      <c r="AN28" s="160">
+      <c r="AN28" s="171"/>
+      <c r="AO28" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A29" s="157" t="s">
         <v>48</v>
       </c>
@@ -14722,12 +14787,13 @@
       <c r="AK29" s="80"/>
       <c r="AL29" s="159"/>
       <c r="AM29" s="171"/>
-      <c r="AN29" s="160">
+      <c r="AN29" s="171"/>
+      <c r="AO29" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A30" s="157" t="s">
         <v>48</v>
       </c>
@@ -14777,12 +14843,13 @@
       <c r="AK30" s="80"/>
       <c r="AL30" s="159"/>
       <c r="AM30" s="171"/>
-      <c r="AN30" s="160">
+      <c r="AN30" s="171"/>
+      <c r="AO30" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A31" s="157" t="s">
         <v>48</v>
       </c>
@@ -14864,12 +14931,13 @@
       <c r="AK31" s="80"/>
       <c r="AL31" s="69"/>
       <c r="AM31" s="159"/>
-      <c r="AN31" s="158">
+      <c r="AN31" s="159"/>
+      <c r="AO31" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A32" s="157" t="s">
         <v>48</v>
       </c>
@@ -14927,12 +14995,13 @@
         <v>1</v>
       </c>
       <c r="AM32" s="159"/>
-      <c r="AN32" s="158">
+      <c r="AN32" s="159"/>
+      <c r="AO32" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A33" s="157" t="s">
         <v>53</v>
       </c>
@@ -15002,12 +15071,13 @@
       <c r="AK33" s="80"/>
       <c r="AL33" s="159"/>
       <c r="AM33" s="171"/>
-      <c r="AN33" s="160">
+      <c r="AN33" s="171"/>
+      <c r="AO33" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A34" s="157" t="s">
         <v>53</v>
       </c>
@@ -15095,12 +15165,15 @@
       <c r="AM34" s="159">
         <v>1</v>
       </c>
-      <c r="AN34" s="158">
+      <c r="AN34" s="159">
+        <v>1</v>
+      </c>
+      <c r="AO34" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A35" s="157" t="s">
         <v>58</v>
       </c>
@@ -15150,12 +15223,13 @@
       <c r="AK35" s="40"/>
       <c r="AL35" s="159"/>
       <c r="AM35" s="171"/>
-      <c r="AN35" s="160">
+      <c r="AN35" s="171"/>
+      <c r="AO35" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A36" s="157" t="s">
         <v>58</v>
       </c>
@@ -15203,12 +15277,13 @@
       <c r="AK36" s="40"/>
       <c r="AL36" s="159"/>
       <c r="AM36" s="171"/>
-      <c r="AN36" s="160">
+      <c r="AN36" s="171"/>
+      <c r="AO36" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A37" s="157" t="s">
         <v>58</v>
       </c>
@@ -15256,12 +15331,13 @@
       <c r="AK37" s="40"/>
       <c r="AL37" s="159"/>
       <c r="AM37" s="171"/>
-      <c r="AN37" s="160">
+      <c r="AN37" s="171"/>
+      <c r="AO37" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A38" s="157" t="s">
         <v>58</v>
       </c>
@@ -15309,12 +15385,13 @@
       <c r="AK38" s="40"/>
       <c r="AL38" s="159"/>
       <c r="AM38" s="171"/>
-      <c r="AN38" s="160">
+      <c r="AN38" s="171"/>
+      <c r="AO38" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A39" s="157" t="s">
         <v>58</v>
       </c>
@@ -15374,12 +15451,13 @@
         <v>1</v>
       </c>
       <c r="AM39" s="159"/>
-      <c r="AN39" s="158">
+      <c r="AN39" s="159"/>
+      <c r="AO39" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A40" s="181" t="s">
         <v>58</v>
       </c>
@@ -15427,12 +15505,13 @@
       <c r="AM40" s="184">
         <v>1</v>
       </c>
-      <c r="AN40" s="185">
+      <c r="AN40" s="184"/>
+      <c r="AO40" s="185">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A41" s="157" t="s">
         <v>58</v>
       </c>
@@ -15482,12 +15561,13 @@
       <c r="AK41" s="80"/>
       <c r="AL41" s="159"/>
       <c r="AM41" s="171"/>
-      <c r="AN41" s="160">
+      <c r="AN41" s="171"/>
+      <c r="AO41" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A42" s="157" t="s">
         <v>58</v>
       </c>
@@ -15537,12 +15617,13 @@
       <c r="AK42" s="80"/>
       <c r="AL42" s="159"/>
       <c r="AM42" s="171"/>
-      <c r="AN42" s="160">
+      <c r="AN42" s="171"/>
+      <c r="AO42" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A43" s="157" t="s">
         <v>63</v>
       </c>
@@ -15614,12 +15695,13 @@
       <c r="AK43" s="80"/>
       <c r="AL43" s="69"/>
       <c r="AM43" s="159"/>
-      <c r="AN43" s="158">
+      <c r="AN43" s="159"/>
+      <c r="AO43" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A44" s="157" t="s">
         <v>63</v>
       </c>
@@ -15669,12 +15751,13 @@
       <c r="AK44" s="80"/>
       <c r="AL44" s="159"/>
       <c r="AM44" s="171"/>
-      <c r="AN44" s="160">
+      <c r="AN44" s="171"/>
+      <c r="AO44" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A45" s="157" t="s">
         <v>63</v>
       </c>
@@ -15728,12 +15811,13 @@
       <c r="AK45" s="80"/>
       <c r="AL45" s="159"/>
       <c r="AM45" s="171"/>
-      <c r="AN45" s="160">
+      <c r="AN45" s="171"/>
+      <c r="AO45" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A46" s="157" t="s">
         <v>63</v>
       </c>
@@ -15791,12 +15875,13 @@
       <c r="AK46" s="80"/>
       <c r="AL46" s="159"/>
       <c r="AM46" s="171"/>
-      <c r="AN46" s="160">
+      <c r="AN46" s="171"/>
+      <c r="AO46" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A47" s="157" t="s">
         <v>63</v>
       </c>
@@ -15854,12 +15939,15 @@
       <c r="AK47" s="80"/>
       <c r="AL47" s="159"/>
       <c r="AM47" s="171"/>
-      <c r="AN47" s="160">
+      <c r="AN47" s="171">
+        <v>1</v>
+      </c>
+      <c r="AO47" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A48" s="157" t="s">
         <v>154</v>
       </c>
@@ -15907,12 +15995,13 @@
       <c r="AK48" s="80"/>
       <c r="AL48" s="159"/>
       <c r="AM48" s="171"/>
-      <c r="AN48" s="160">
+      <c r="AN48" s="171"/>
+      <c r="AO48" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A49" s="157" t="s">
         <v>65</v>
       </c>
@@ -15964,12 +16053,13 @@
       </c>
       <c r="AL49" s="159"/>
       <c r="AM49" s="171"/>
-      <c r="AN49" s="160">
+      <c r="AN49" s="171"/>
+      <c r="AO49" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A50" s="157" t="s">
         <v>65</v>
       </c>
@@ -16059,12 +16149,13 @@
       <c r="AK50" s="40"/>
       <c r="AL50" s="69"/>
       <c r="AM50" s="159"/>
-      <c r="AN50" s="158">
+      <c r="AN50" s="159"/>
+      <c r="AO50" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A51" s="157" t="s">
         <v>65</v>
       </c>
@@ -16120,12 +16211,13 @@
       <c r="AK51" s="40"/>
       <c r="AL51" s="69"/>
       <c r="AM51" s="159"/>
-      <c r="AN51" s="158">
+      <c r="AN51" s="159"/>
+      <c r="AO51" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A52" s="157" t="s">
         <v>68</v>
       </c>
@@ -16183,12 +16275,13 @@
       <c r="AK52" s="40"/>
       <c r="AL52" s="159"/>
       <c r="AM52" s="171"/>
-      <c r="AN52" s="160">
+      <c r="AN52" s="171"/>
+      <c r="AO52" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A53" s="157" t="s">
         <v>68</v>
       </c>
@@ -16236,12 +16329,13 @@
       <c r="AK53" s="40"/>
       <c r="AL53" s="159"/>
       <c r="AM53" s="171"/>
-      <c r="AN53" s="160">
+      <c r="AN53" s="171"/>
+      <c r="AO53" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A54" s="157" t="s">
         <v>68</v>
       </c>
@@ -16289,12 +16383,13 @@
       <c r="AK54" s="40"/>
       <c r="AL54" s="159"/>
       <c r="AM54" s="171"/>
-      <c r="AN54" s="160">
+      <c r="AN54" s="171"/>
+      <c r="AO54" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A55" s="157" t="s">
         <v>68</v>
       </c>
@@ -16356,12 +16451,13 @@
       </c>
       <c r="AL55" s="69"/>
       <c r="AM55" s="159"/>
-      <c r="AN55" s="158">
+      <c r="AN55" s="159"/>
+      <c r="AO55" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A56" s="157" t="s">
         <v>73</v>
       </c>
@@ -16417,12 +16513,13 @@
       <c r="AK56" s="40"/>
       <c r="AL56" s="69"/>
       <c r="AM56" s="159"/>
-      <c r="AN56" s="158">
+      <c r="AN56" s="159"/>
+      <c r="AO56" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A57" s="157" t="s">
         <v>73</v>
       </c>
@@ -16474,12 +16571,13 @@
       <c r="AK57" s="40"/>
       <c r="AL57" s="159"/>
       <c r="AM57" s="171"/>
-      <c r="AN57" s="160">
+      <c r="AN57" s="171"/>
+      <c r="AO57" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A58" s="157" t="s">
         <v>73</v>
       </c>
@@ -16533,12 +16631,13 @@
       <c r="AK58" s="40"/>
       <c r="AL58" s="69"/>
       <c r="AM58" s="159"/>
-      <c r="AN58" s="158">
+      <c r="AN58" s="159"/>
+      <c r="AO58" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A59" s="157" t="s">
         <v>73</v>
       </c>
@@ -16588,12 +16687,13 @@
       <c r="AK59" s="40"/>
       <c r="AL59" s="159"/>
       <c r="AM59" s="171"/>
-      <c r="AN59" s="160">
+      <c r="AN59" s="171"/>
+      <c r="AO59" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A60" s="157" t="s">
         <v>76</v>
       </c>
@@ -16675,12 +16775,13 @@
       <c r="AK60" s="40"/>
       <c r="AL60" s="69"/>
       <c r="AM60" s="159"/>
-      <c r="AN60" s="158">
+      <c r="AN60" s="159"/>
+      <c r="AO60" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A61" s="157" t="s">
         <v>76</v>
       </c>
@@ -16748,12 +16849,13 @@
       <c r="AM61" s="159">
         <v>1</v>
       </c>
-      <c r="AN61" s="158">
+      <c r="AN61" s="159"/>
+      <c r="AO61" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A62" s="157" t="s">
         <v>79</v>
       </c>
@@ -16801,12 +16903,13 @@
       <c r="AK62" s="40"/>
       <c r="AL62" s="159"/>
       <c r="AM62" s="171"/>
-      <c r="AN62" s="160">
+      <c r="AN62" s="171"/>
+      <c r="AO62" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A63" s="157" t="s">
         <v>79</v>
       </c>
@@ -16854,12 +16957,13 @@
       <c r="AK63" s="40"/>
       <c r="AL63" s="159"/>
       <c r="AM63" s="171"/>
-      <c r="AN63" s="160">
+      <c r="AN63" s="171"/>
+      <c r="AO63" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A64" s="157" t="s">
         <v>79</v>
       </c>
@@ -16907,12 +17011,13 @@
       <c r="AK64" s="40"/>
       <c r="AL64" s="159"/>
       <c r="AM64" s="171"/>
-      <c r="AN64" s="160">
+      <c r="AN64" s="171"/>
+      <c r="AO64" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A65" s="157" t="s">
         <v>79</v>
       </c>
@@ -16960,12 +17065,13 @@
       <c r="AK65" s="40"/>
       <c r="AL65" s="159"/>
       <c r="AM65" s="171"/>
-      <c r="AN65" s="160">
+      <c r="AN65" s="171"/>
+      <c r="AO65" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A66" s="157" t="s">
         <v>79</v>
       </c>
@@ -17013,12 +17119,13 @@
       <c r="AK66" s="40"/>
       <c r="AL66" s="159"/>
       <c r="AM66" s="171"/>
-      <c r="AN66" s="160">
+      <c r="AN66" s="171"/>
+      <c r="AO66" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A67" s="157" t="s">
         <v>79</v>
       </c>
@@ -17066,12 +17173,13 @@
       <c r="AK67" s="40"/>
       <c r="AL67" s="69"/>
       <c r="AM67" s="159"/>
-      <c r="AN67" s="158">
+      <c r="AN67" s="159"/>
+      <c r="AO67" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A68" s="157" t="s">
         <v>79</v>
       </c>
@@ -17119,12 +17227,13 @@
       <c r="AK68" s="40"/>
       <c r="AL68" s="159"/>
       <c r="AM68" s="171"/>
-      <c r="AN68" s="160">
+      <c r="AN68" s="171"/>
+      <c r="AO68" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A69" s="157" t="s">
         <v>79</v>
       </c>
@@ -17172,12 +17281,13 @@
       <c r="AK69" s="40"/>
       <c r="AL69" s="159"/>
       <c r="AM69" s="171"/>
-      <c r="AN69" s="160">
+      <c r="AN69" s="171"/>
+      <c r="AO69" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A70" s="157" t="s">
         <v>79</v>
       </c>
@@ -17225,12 +17335,13 @@
       <c r="AK70" s="80"/>
       <c r="AL70" s="159"/>
       <c r="AM70" s="171"/>
-      <c r="AN70" s="160">
+      <c r="AN70" s="171"/>
+      <c r="AO70" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A71" s="157" t="s">
         <v>79</v>
       </c>
@@ -17280,12 +17391,13 @@
       <c r="AK71" s="80"/>
       <c r="AL71" s="159"/>
       <c r="AM71" s="171"/>
-      <c r="AN71" s="160">
+      <c r="AN71" s="171"/>
+      <c r="AO71" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A72" s="157" t="s">
         <v>79</v>
       </c>
@@ -17335,12 +17447,13 @@
       <c r="AK72" s="80"/>
       <c r="AL72" s="159"/>
       <c r="AM72" s="171"/>
-      <c r="AN72" s="160">
+      <c r="AN72" s="171"/>
+      <c r="AO72" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A73" s="157" t="s">
         <v>79</v>
       </c>
@@ -17388,12 +17501,13 @@
       <c r="AK73" s="80"/>
       <c r="AL73" s="159"/>
       <c r="AM73" s="171"/>
-      <c r="AN73" s="160">
+      <c r="AN73" s="171"/>
+      <c r="AO73" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A74" s="157" t="s">
         <v>79</v>
       </c>
@@ -17463,12 +17577,13 @@
       <c r="AK74" s="80"/>
       <c r="AL74" s="69"/>
       <c r="AM74" s="159"/>
-      <c r="AN74" s="158">
+      <c r="AN74" s="159"/>
+      <c r="AO74" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A75" s="157" t="s">
         <v>79</v>
       </c>
@@ -17522,12 +17637,13 @@
       <c r="AM75" s="159">
         <v>1</v>
       </c>
-      <c r="AN75" s="158">
+      <c r="AN75" s="159"/>
+      <c r="AO75" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A76" s="157" t="s">
         <v>83</v>
       </c>
@@ -17577,12 +17693,13 @@
       <c r="AK76" s="80"/>
       <c r="AL76" s="69"/>
       <c r="AM76" s="159"/>
-      <c r="AN76" s="158">
+      <c r="AN76" s="159"/>
+      <c r="AO76" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A77" s="157" t="s">
         <v>83</v>
       </c>
@@ -17640,12 +17757,13 @@
       <c r="AK77" s="40"/>
       <c r="AL77" s="69"/>
       <c r="AM77" s="159"/>
-      <c r="AN77" s="158">
+      <c r="AN77" s="159"/>
+      <c r="AO77" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A78" s="157" t="s">
         <v>83</v>
       </c>
@@ -17729,12 +17847,13 @@
         <v>1</v>
       </c>
       <c r="AM78" s="171"/>
-      <c r="AN78" s="160">
+      <c r="AN78" s="171"/>
+      <c r="AO78" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A79" s="157" t="s">
         <v>85</v>
       </c>
@@ -17836,12 +17955,13 @@
       <c r="AM79" s="159">
         <v>1</v>
       </c>
-      <c r="AN79" s="158">
+      <c r="AN79" s="159"/>
+      <c r="AO79" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>27</v>
       </c>
     </row>
-    <row r="80" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A80" s="157" t="s">
         <v>86</v>
       </c>
@@ -17899,12 +18019,13 @@
         <v>1</v>
       </c>
       <c r="AM80" s="171"/>
-      <c r="AN80" s="160">
+      <c r="AN80" s="171"/>
+      <c r="AO80" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A81" s="157" t="s">
         <v>86</v>
       </c>
@@ -18004,12 +18125,13 @@
       <c r="AM81" s="159">
         <v>1</v>
       </c>
-      <c r="AN81" s="158">
+      <c r="AN81" s="159"/>
+      <c r="AO81" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A82" s="157" t="s">
         <v>87</v>
       </c>
@@ -18107,12 +18229,13 @@
       <c r="AK82" s="80"/>
       <c r="AL82" s="69"/>
       <c r="AM82" s="159"/>
-      <c r="AN82" s="158">
+      <c r="AN82" s="159"/>
+      <c r="AO82" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A83" s="157" t="s">
         <v>87</v>
       </c>
@@ -18168,12 +18291,13 @@
         <v>1</v>
       </c>
       <c r="AM83" s="159"/>
-      <c r="AN83" s="158">
+      <c r="AN83" s="159"/>
+      <c r="AO83" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A84" s="157" t="s">
         <v>88</v>
       </c>
@@ -18255,12 +18379,13 @@
       <c r="AK84" s="40"/>
       <c r="AL84" s="69"/>
       <c r="AM84" s="159"/>
-      <c r="AN84" s="158">
+      <c r="AN84" s="159"/>
+      <c r="AO84" s="158">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>17</v>
       </c>
     </row>
-    <row r="85" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A85" s="164" t="s">
         <v>89</v>
       </c>
@@ -18310,12 +18435,13 @@
       <c r="AK85" s="165"/>
       <c r="AL85" s="163"/>
       <c r="AM85" s="171"/>
-      <c r="AN85" s="160">
+      <c r="AN85" s="171"/>
+      <c r="AO85" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A86" s="164" t="s">
         <v>89</v>
       </c>
@@ -18365,12 +18491,13 @@
       <c r="AM86" s="171">
         <v>1</v>
       </c>
-      <c r="AN86" s="160">
+      <c r="AN86" s="171"/>
+      <c r="AO86" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A87" s="164" t="s">
         <v>170</v>
       </c>
@@ -18424,12 +18551,13 @@
       <c r="AK87" s="165"/>
       <c r="AL87" s="163"/>
       <c r="AM87" s="171"/>
-      <c r="AN87" s="160">
+      <c r="AN87" s="171"/>
+      <c r="AO87" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A88" s="164" t="s">
         <v>170</v>
       </c>
@@ -18479,12 +18607,13 @@
         <v>1</v>
       </c>
       <c r="AM88" s="171"/>
-      <c r="AN88" s="160">
+      <c r="AN88" s="171"/>
+      <c r="AO88" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A89" s="167" t="s">
         <v>90</v>
       </c>
@@ -18492,7 +18621,7 @@
       <c r="C89" s="169"/>
       <c r="D89" s="170"/>
       <c r="E89" s="160">
-        <f t="shared" ref="E89:AN89" si="0">SUM(E2:E87)</f>
+        <f t="shared" ref="E89:AO89" si="0">SUM(E2:E87)</f>
         <v>1</v>
       </c>
       <c r="F89" s="160">
@@ -18631,7 +18760,8 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="AN89" s="160">
+      <c r="AN89" s="160"/>
+      <c r="AO89" s="160">
         <f t="shared" si="0"/>
         <v>557</v>
       </c>
@@ -18761,34 +18891,34 @@
       <c r="AG2" s="132"/>
     </row>
     <row r="3" spans="1:33" s="130" customFormat="1" ht="78" x14ac:dyDescent="0.35">
-      <c r="A3" s="198" t="s">
+      <c r="A3" s="195" t="s">
         <v>359</v>
       </c>
-      <c r="B3" s="198" t="s">
+      <c r="B3" s="195" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="200" t="s">
+      <c r="C3" s="197" t="s">
         <v>360</v>
       </c>
       <c r="D3" s="131" t="s">
         <v>361</v>
       </c>
-      <c r="E3" s="200" t="s">
+      <c r="E3" s="197" t="s">
         <v>362</v>
       </c>
-      <c r="F3" s="202" t="s">
+      <c r="F3" s="199" t="s">
         <v>363</v>
       </c>
-      <c r="G3" s="204" t="s">
+      <c r="G3" s="201" t="s">
         <v>364</v>
       </c>
-      <c r="H3" s="202" t="s">
+      <c r="H3" s="199" t="s">
         <v>365</v>
       </c>
-      <c r="I3" s="202" t="s">
+      <c r="I3" s="199" t="s">
         <v>366</v>
       </c>
-      <c r="J3" s="202"/>
+      <c r="J3" s="199"/>
       <c r="K3" s="128" t="s">
         <v>367</v>
       </c>
@@ -18801,57 +18931,57 @@
       <c r="N3" s="127" t="s">
         <v>370</v>
       </c>
-      <c r="O3" s="195" t="s">
+      <c r="O3" s="205" t="s">
         <v>371</v>
       </c>
-      <c r="P3" s="195"/>
-      <c r="Q3" s="195" t="s">
+      <c r="P3" s="205"/>
+      <c r="Q3" s="205" t="s">
         <v>372</v>
       </c>
-      <c r="R3" s="195"/>
-      <c r="S3" s="195" t="s">
+      <c r="R3" s="205"/>
+      <c r="S3" s="205" t="s">
         <v>373</v>
       </c>
-      <c r="T3" s="195"/>
-      <c r="U3" s="194" t="s">
+      <c r="T3" s="205"/>
+      <c r="U3" s="204" t="s">
         <v>374</v>
       </c>
-      <c r="V3" s="194"/>
-      <c r="W3" s="194" t="s">
+      <c r="V3" s="204"/>
+      <c r="W3" s="204" t="s">
         <v>375</v>
       </c>
-      <c r="X3" s="194"/>
-      <c r="Y3" s="194" t="s">
+      <c r="X3" s="204"/>
+      <c r="Y3" s="204" t="s">
         <v>376</v>
       </c>
-      <c r="Z3" s="194"/>
-      <c r="AA3" s="194" t="s">
+      <c r="Z3" s="204"/>
+      <c r="AA3" s="204" t="s">
         <v>377</v>
       </c>
-      <c r="AB3" s="194"/>
-      <c r="AC3" s="194" t="s">
+      <c r="AB3" s="204"/>
+      <c r="AC3" s="204" t="s">
         <v>378</v>
       </c>
-      <c r="AD3" s="194"/>
-      <c r="AE3" s="196" t="s">
+      <c r="AD3" s="204"/>
+      <c r="AE3" s="193" t="s">
         <v>379</v>
       </c>
-      <c r="AF3" s="197"/>
+      <c r="AF3" s="194"/>
       <c r="AG3" s="125" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="4" spans="1:33" s="124" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="199"/>
-      <c r="B4" s="199"/>
-      <c r="C4" s="201"/>
+      <c r="A4" s="196"/>
+      <c r="B4" s="196"/>
+      <c r="C4" s="198"/>
       <c r="D4" s="129"/>
-      <c r="E4" s="201"/>
-      <c r="F4" s="203"/>
-      <c r="G4" s="205"/>
-      <c r="H4" s="203"/>
-      <c r="I4" s="203"/>
-      <c r="J4" s="203"/>
+      <c r="E4" s="198"/>
+      <c r="F4" s="200"/>
+      <c r="G4" s="202"/>
+      <c r="H4" s="200"/>
+      <c r="I4" s="200"/>
+      <c r="J4" s="200"/>
       <c r="K4" s="128"/>
       <c r="L4" s="128"/>
       <c r="M4" s="128"/>
@@ -19935,7 +20065,7 @@
       <c r="E25" s="104" t="s">
         <v>454</v>
       </c>
-      <c r="I25" s="193"/>
+      <c r="I25" s="203"/>
       <c r="J25" s="57"/>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.35">
@@ -19945,7 +20075,7 @@
       <c r="E26" s="103" t="s">
         <v>455</v>
       </c>
-      <c r="I26" s="193"/>
+      <c r="I26" s="203"/>
       <c r="J26" s="57"/>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.35">
@@ -19955,7 +20085,7 @@
       <c r="E27" s="104" t="s">
         <v>457</v>
       </c>
-      <c r="I27" s="193"/>
+      <c r="I27" s="203"/>
       <c r="J27" s="57"/>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.35">
@@ -19965,7 +20095,7 @@
       <c r="E28" s="104" t="s">
         <v>458</v>
       </c>
-      <c r="I28" s="193"/>
+      <c r="I28" s="203"/>
       <c r="J28" s="57"/>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.35">
@@ -19999,6 +20129,15 @@
     <filterColumn colId="28" showButton="0"/>
   </autoFilter>
   <mergeCells count="19">
+    <mergeCell ref="I25:I28"/>
+    <mergeCell ref="AC3:AD3"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="Y3:Z3"/>
+    <mergeCell ref="AA3:AB3"/>
     <mergeCell ref="AE3:AF3"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -20009,15 +20148,6 @@
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="I25:I28"/>
-    <mergeCell ref="AC3:AD3"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="W3:X3"/>
-    <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="AA3:AB3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -20566,18 +20696,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="215" t="s">
+      <c r="B1" s="222" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="215"/>
-      <c r="D1" s="215"/>
-      <c r="E1" s="215"/>
-      <c r="F1" s="215"/>
-      <c r="G1" s="215"/>
-      <c r="H1" s="215"/>
-      <c r="I1" s="215"/>
-      <c r="J1" s="215"/>
-      <c r="K1" s="215"/>
+      <c r="C1" s="222"/>
+      <c r="D1" s="222"/>
+      <c r="E1" s="222"/>
+      <c r="F1" s="222"/>
+      <c r="G1" s="222"/>
+      <c r="H1" s="222"/>
+      <c r="I1" s="222"/>
+      <c r="J1" s="222"/>
+      <c r="K1" s="222"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" spans="2:12" ht="24" x14ac:dyDescent="0.35">
@@ -20603,7 +20733,7 @@
       <c r="L2" s="44"/>
     </row>
     <row r="3" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="216" t="s">
+      <c r="B3" s="218" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="97" t="s">
@@ -20620,7 +20750,7 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="217"/>
+      <c r="B4" s="215"/>
       <c r="C4" s="97" t="s">
         <v>14</v>
       </c>
@@ -20635,7 +20765,7 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="217"/>
+      <c r="B5" s="215"/>
       <c r="C5" s="97" t="s">
         <v>257</v>
       </c>
@@ -20650,7 +20780,7 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="218"/>
+      <c r="B6" s="219"/>
       <c r="C6" s="97" t="s">
         <v>259</v>
       </c>
@@ -20682,7 +20812,7 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="217" t="s">
+      <c r="B8" s="215" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="94" t="s">
@@ -20699,7 +20829,7 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="217"/>
+      <c r="B9" s="215"/>
       <c r="C9" s="93" t="s">
         <v>67</v>
       </c>
@@ -20714,7 +20844,7 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="219" t="s">
+      <c r="B10" s="223" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="98" t="s">
@@ -20731,7 +20861,7 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="220"/>
+      <c r="B11" s="224"/>
       <c r="C11" s="98" t="s">
         <v>26</v>
       </c>
@@ -20746,7 +20876,7 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="220"/>
+      <c r="B12" s="224"/>
       <c r="C12" s="98" t="s">
         <v>27</v>
       </c>
@@ -20761,7 +20891,7 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="221"/>
+      <c r="B13" s="225"/>
       <c r="C13" s="98" t="s">
         <v>267</v>
       </c>
@@ -20776,7 +20906,7 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="216" t="s">
+      <c r="B14" s="218" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="60" t="s">
@@ -20793,7 +20923,7 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="217"/>
+      <c r="B15" s="215"/>
       <c r="C15" s="60" t="s">
         <v>29</v>
       </c>
@@ -20808,7 +20938,7 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="217"/>
+      <c r="B16" s="215"/>
       <c r="C16" s="60" t="s">
         <v>271</v>
       </c>
@@ -20823,7 +20953,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="218"/>
+      <c r="B17" s="219"/>
       <c r="C17" s="61" t="s">
         <v>267</v>
       </c>
@@ -20838,7 +20968,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="223" t="s">
+      <c r="B18" s="216" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="59" t="s">
@@ -20855,7 +20985,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="224"/>
+      <c r="B19" s="217"/>
       <c r="C19" s="2" t="s">
         <v>67</v>
       </c>
@@ -20870,7 +21000,7 @@
       </c>
     </row>
     <row r="20" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="217" t="s">
+      <c r="B20" s="215" t="s">
         <v>34</v>
       </c>
       <c r="C20" s="62" t="s">
@@ -20887,7 +21017,7 @@
       </c>
     </row>
     <row r="21" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="217"/>
+      <c r="B21" s="215"/>
       <c r="C21" s="60" t="s">
         <v>27</v>
       </c>
@@ -20902,7 +21032,7 @@
       </c>
     </row>
     <row r="22" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="217"/>
+      <c r="B22" s="215"/>
       <c r="C22" s="60" t="s">
         <v>277</v>
       </c>
@@ -20917,7 +21047,7 @@
       </c>
     </row>
     <row r="23" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="217"/>
+      <c r="B23" s="215"/>
       <c r="C23" s="61" t="s">
         <v>279</v>
       </c>
@@ -20932,7 +21062,7 @@
       </c>
     </row>
     <row r="24" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="219" t="s">
+      <c r="B24" s="223" t="s">
         <v>38</v>
       </c>
       <c r="C24" s="63" t="s">
@@ -20949,7 +21079,7 @@
       </c>
     </row>
     <row r="25" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="220"/>
+      <c r="B25" s="224"/>
       <c r="C25" s="63" t="s">
         <v>39</v>
       </c>
@@ -20964,7 +21094,7 @@
       </c>
     </row>
     <row r="26" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="220"/>
+      <c r="B26" s="224"/>
       <c r="C26" s="63" t="s">
         <v>40</v>
       </c>
@@ -20979,7 +21109,7 @@
       </c>
     </row>
     <row r="27" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="220"/>
+      <c r="B27" s="224"/>
       <c r="C27" s="63" t="s">
         <v>41</v>
       </c>
@@ -20994,7 +21124,7 @@
       </c>
     </row>
     <row r="28" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="220"/>
+      <c r="B28" s="224"/>
       <c r="C28" s="63" t="s">
         <v>285</v>
       </c>
@@ -21009,7 +21139,7 @@
       </c>
     </row>
     <row r="29" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="220"/>
+      <c r="B29" s="224"/>
       <c r="C29" s="63" t="s">
         <v>267</v>
       </c>
@@ -21024,7 +21154,7 @@
       </c>
     </row>
     <row r="30" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="221"/>
+      <c r="B30" s="225"/>
       <c r="C30" s="63" t="s">
         <v>279</v>
       </c>
@@ -21039,7 +21169,7 @@
       </c>
     </row>
     <row r="31" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="217" t="s">
+      <c r="B31" s="215" t="s">
         <v>43</v>
       </c>
       <c r="C31" s="12" t="s">
@@ -21056,7 +21186,7 @@
       </c>
     </row>
     <row r="32" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="217"/>
+      <c r="B32" s="215"/>
       <c r="C32" s="97" t="s">
         <v>45</v>
       </c>
@@ -21071,7 +21201,7 @@
       </c>
     </row>
     <row r="33" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="217"/>
+      <c r="B33" s="215"/>
       <c r="C33" s="97" t="s">
         <v>40</v>
       </c>
@@ -21086,7 +21216,7 @@
       </c>
     </row>
     <row r="34" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="217"/>
+      <c r="B34" s="215"/>
       <c r="C34" s="93" t="s">
         <v>259</v>
       </c>
@@ -21101,7 +21231,7 @@
       </c>
     </row>
     <row r="35" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="225" t="s">
+      <c r="B35" s="220" t="s">
         <v>48</v>
       </c>
       <c r="C35" s="98" t="s">
@@ -21118,7 +21248,7 @@
       </c>
     </row>
     <row r="36" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="225"/>
+      <c r="B36" s="220"/>
       <c r="C36" s="98" t="s">
         <v>49</v>
       </c>
@@ -21133,7 +21263,7 @@
       </c>
     </row>
     <row r="37" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="225"/>
+      <c r="B37" s="220"/>
       <c r="C37" s="98" t="s">
         <v>293</v>
       </c>
@@ -21148,7 +21278,7 @@
       </c>
     </row>
     <row r="38" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="225"/>
+      <c r="B38" s="220"/>
       <c r="C38" s="98" t="s">
         <v>267</v>
       </c>
@@ -21163,7 +21293,7 @@
       </c>
     </row>
     <row r="39" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="218" t="s">
+      <c r="B39" s="219" t="s">
         <v>53</v>
       </c>
       <c r="C39" s="94" t="s">
@@ -21180,7 +21310,7 @@
       </c>
     </row>
     <row r="40" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="216"/>
+      <c r="B40" s="218"/>
       <c r="C40" s="93" t="s">
         <v>57</v>
       </c>
@@ -21195,7 +21325,7 @@
       </c>
     </row>
     <row r="41" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="219" t="s">
+      <c r="B41" s="223" t="s">
         <v>58</v>
       </c>
       <c r="C41" s="98" t="s">
@@ -21212,7 +21342,7 @@
       </c>
     </row>
     <row r="42" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="220"/>
+      <c r="B42" s="224"/>
       <c r="C42" s="98" t="s">
         <v>60</v>
       </c>
@@ -21227,7 +21357,7 @@
       </c>
     </row>
     <row r="43" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="220"/>
+      <c r="B43" s="224"/>
       <c r="C43" s="98" t="s">
         <v>62</v>
       </c>
@@ -21242,7 +21372,7 @@
       </c>
     </row>
     <row r="44" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="220"/>
+      <c r="B44" s="224"/>
       <c r="C44" s="98" t="s">
         <v>300</v>
       </c>
@@ -21257,7 +21387,7 @@
       </c>
     </row>
     <row r="45" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B45" s="221"/>
+      <c r="B45" s="225"/>
       <c r="C45" s="98" t="s">
         <v>267</v>
       </c>
@@ -21272,7 +21402,7 @@
       </c>
     </row>
     <row r="46" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B46" s="216" t="s">
+      <c r="B46" s="218" t="s">
         <v>170</v>
       </c>
       <c r="C46" s="64" t="s">
@@ -21289,7 +21419,7 @@
       </c>
     </row>
     <row r="47" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B47" s="217"/>
+      <c r="B47" s="215"/>
       <c r="C47" s="64" t="s">
         <v>259</v>
       </c>
@@ -21304,7 +21434,7 @@
       </c>
     </row>
     <row r="48" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B48" s="217"/>
+      <c r="B48" s="215"/>
       <c r="C48" s="64" t="s">
         <v>267</v>
       </c>
@@ -21319,7 +21449,7 @@
       </c>
     </row>
     <row r="49" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="218"/>
+      <c r="B49" s="219"/>
       <c r="C49" s="64" t="s">
         <v>16</v>
       </c>
@@ -21334,7 +21464,7 @@
       </c>
     </row>
     <row r="50" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="216" t="s">
+      <c r="B50" s="218" t="s">
         <v>63</v>
       </c>
       <c r="C50" s="64" t="s">
@@ -21351,7 +21481,7 @@
       </c>
     </row>
     <row r="51" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="217"/>
+      <c r="B51" s="215"/>
       <c r="C51" s="64" t="s">
         <v>59</v>
       </c>
@@ -21366,7 +21496,7 @@
       </c>
     </row>
     <row r="52" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="218"/>
+      <c r="B52" s="219"/>
       <c r="C52" s="64" t="s">
         <v>267</v>
       </c>
@@ -21381,7 +21511,7 @@
       </c>
     </row>
     <row r="53" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B53" s="220" t="s">
+      <c r="B53" s="224" t="s">
         <v>154</v>
       </c>
       <c r="C53" s="96" t="s">
@@ -21398,7 +21528,7 @@
       </c>
     </row>
     <row r="54" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="220"/>
+      <c r="B54" s="224"/>
       <c r="C54" s="98" t="s">
         <v>155</v>
       </c>
@@ -21413,7 +21543,7 @@
       </c>
     </row>
     <row r="55" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B55" s="220"/>
+      <c r="B55" s="224"/>
       <c r="C55" s="95" t="s">
         <v>267</v>
       </c>
@@ -21428,7 +21558,7 @@
       </c>
     </row>
     <row r="56" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B56" s="216" t="s">
+      <c r="B56" s="218" t="s">
         <v>65</v>
       </c>
       <c r="C56" s="97" t="s">
@@ -21445,7 +21575,7 @@
       </c>
     </row>
     <row r="57" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B57" s="217"/>
+      <c r="B57" s="215"/>
       <c r="C57" s="97" t="s">
         <v>67</v>
       </c>
@@ -21460,7 +21590,7 @@
       </c>
     </row>
     <row r="58" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="218"/>
+      <c r="B58" s="219"/>
       <c r="C58" s="97" t="s">
         <v>259</v>
       </c>
@@ -21475,7 +21605,7 @@
       </c>
     </row>
     <row r="59" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B59" s="219" t="s">
+      <c r="B59" s="223" t="s">
         <v>68</v>
       </c>
       <c r="C59" s="98" t="s">
@@ -21492,7 +21622,7 @@
       </c>
     </row>
     <row r="60" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B60" s="220"/>
+      <c r="B60" s="224"/>
       <c r="C60" s="98" t="s">
         <v>27</v>
       </c>
@@ -21507,7 +21637,7 @@
       </c>
     </row>
     <row r="61" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="220"/>
+      <c r="B61" s="224"/>
       <c r="C61" s="98" t="s">
         <v>316</v>
       </c>
@@ -21522,7 +21652,7 @@
       </c>
     </row>
     <row r="62" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="220"/>
+      <c r="B62" s="224"/>
       <c r="C62" s="98" t="s">
         <v>318</v>
       </c>
@@ -21537,7 +21667,7 @@
       </c>
     </row>
     <row r="63" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="220"/>
+      <c r="B63" s="224"/>
       <c r="C63" s="98" t="s">
         <v>320</v>
       </c>
@@ -21552,7 +21682,7 @@
       </c>
     </row>
     <row r="64" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="220"/>
+      <c r="B64" s="224"/>
       <c r="C64" s="98" t="s">
         <v>322</v>
       </c>
@@ -21567,7 +21697,7 @@
       </c>
     </row>
     <row r="65" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B65" s="221"/>
+      <c r="B65" s="225"/>
       <c r="C65" s="98" t="s">
         <v>324</v>
       </c>
@@ -21582,7 +21712,7 @@
       </c>
     </row>
     <row r="66" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B66" s="216" t="s">
+      <c r="B66" s="218" t="s">
         <v>73</v>
       </c>
       <c r="C66" s="94" t="s">
@@ -21599,7 +21729,7 @@
       </c>
     </row>
     <row r="67" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="217"/>
+      <c r="B67" s="215"/>
       <c r="C67" s="97" t="s">
         <v>74</v>
       </c>
@@ -21614,7 +21744,7 @@
       </c>
     </row>
     <row r="68" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="217"/>
+      <c r="B68" s="215"/>
       <c r="C68" s="97" t="s">
         <v>327</v>
       </c>
@@ -21629,7 +21759,7 @@
       </c>
     </row>
     <row r="69" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B69" s="218"/>
+      <c r="B69" s="219"/>
       <c r="C69" s="93" t="s">
         <v>267</v>
       </c>
@@ -21644,7 +21774,7 @@
       </c>
     </row>
     <row r="70" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B70" s="219" t="s">
+      <c r="B70" s="223" t="s">
         <v>76</v>
       </c>
       <c r="C70" s="98" t="s">
@@ -21661,7 +21791,7 @@
       </c>
     </row>
     <row r="71" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B71" s="220"/>
+      <c r="B71" s="224"/>
       <c r="C71" s="98" t="s">
         <v>44</v>
       </c>
@@ -21676,7 +21806,7 @@
       </c>
     </row>
     <row r="72" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B72" s="220"/>
+      <c r="B72" s="224"/>
       <c r="C72" s="98" t="s">
         <v>332</v>
       </c>
@@ -21691,7 +21821,7 @@
       </c>
     </row>
     <row r="73" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B73" s="220"/>
+      <c r="B73" s="224"/>
       <c r="C73" s="98" t="s">
         <v>334</v>
       </c>
@@ -21706,7 +21836,7 @@
       </c>
     </row>
     <row r="74" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="221"/>
+      <c r="B74" s="225"/>
       <c r="C74" s="98" t="s">
         <v>82</v>
       </c>
@@ -21721,7 +21851,7 @@
       </c>
     </row>
     <row r="75" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B75" s="218" t="s">
+      <c r="B75" s="219" t="s">
         <v>79</v>
       </c>
       <c r="C75" s="94" t="s">
@@ -21738,7 +21868,7 @@
       </c>
     </row>
     <row r="76" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B76" s="222"/>
+      <c r="B76" s="221"/>
       <c r="C76" s="97" t="s">
         <v>26</v>
       </c>
@@ -21753,7 +21883,7 @@
       </c>
     </row>
     <row r="77" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B77" s="216"/>
+      <c r="B77" s="218"/>
       <c r="C77" s="93" t="s">
         <v>9</v>
       </c>
@@ -21768,7 +21898,7 @@
       </c>
     </row>
     <row r="78" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B78" s="216"/>
+      <c r="B78" s="218"/>
       <c r="C78" s="93" t="s">
         <v>82</v>
       </c>
@@ -21783,7 +21913,7 @@
       </c>
     </row>
     <row r="79" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B79" s="219" t="s">
+      <c r="B79" s="223" t="s">
         <v>83</v>
       </c>
       <c r="C79" s="98" t="s">
@@ -21800,7 +21930,7 @@
       </c>
     </row>
     <row r="80" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B80" s="220"/>
+      <c r="B80" s="224"/>
       <c r="C80" s="98" t="s">
         <v>84</v>
       </c>
@@ -21815,7 +21945,7 @@
       </c>
     </row>
     <row r="81" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="220"/>
+      <c r="B81" s="224"/>
       <c r="C81" s="98" t="s">
         <v>342</v>
       </c>
@@ -21830,7 +21960,7 @@
       </c>
     </row>
     <row r="82" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B82" s="221"/>
+      <c r="B82" s="225"/>
       <c r="C82" s="98" t="s">
         <v>267</v>
       </c>
@@ -21845,7 +21975,7 @@
       </c>
     </row>
     <row r="83" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B83" s="217" t="s">
+      <c r="B83" s="215" t="s">
         <v>85</v>
       </c>
       <c r="C83" s="94" t="s">
@@ -21862,7 +21992,7 @@
       </c>
     </row>
     <row r="84" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B84" s="217"/>
+      <c r="B84" s="215"/>
       <c r="C84" s="93" t="s">
         <v>345</v>
       </c>
@@ -21877,7 +22007,7 @@
       </c>
     </row>
     <row r="85" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B85" s="223" t="s">
+      <c r="B85" s="216" t="s">
         <v>89</v>
       </c>
       <c r="C85" s="98" t="s">
@@ -21894,7 +22024,7 @@
       </c>
     </row>
     <row r="86" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B86" s="224"/>
+      <c r="B86" s="217"/>
       <c r="C86" s="2" t="s">
         <v>67</v>
       </c>
@@ -21909,7 +22039,7 @@
       </c>
     </row>
     <row r="87" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B87" s="217" t="s">
+      <c r="B87" s="215" t="s">
         <v>88</v>
       </c>
       <c r="C87" s="94" t="s">
@@ -21926,7 +22056,7 @@
       </c>
     </row>
     <row r="88" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="217"/>
+      <c r="B88" s="215"/>
       <c r="C88" s="97" t="s">
         <v>349</v>
       </c>
@@ -21941,7 +22071,7 @@
       </c>
     </row>
     <row r="89" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B89" s="217"/>
+      <c r="B89" s="215"/>
       <c r="C89" s="97" t="s">
         <v>259</v>
       </c>
@@ -21956,7 +22086,7 @@
       </c>
     </row>
     <row r="90" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B90" s="217"/>
+      <c r="B90" s="215"/>
       <c r="C90" s="93" t="s">
         <v>67</v>
       </c>
@@ -21988,7 +22118,7 @@
       </c>
     </row>
     <row r="92" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B92" s="222" t="s">
+      <c r="B92" s="221" t="s">
         <v>87</v>
       </c>
       <c r="C92" s="94" t="s">
@@ -22005,7 +22135,7 @@
       </c>
     </row>
     <row r="93" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="222"/>
+      <c r="B93" s="221"/>
       <c r="C93" s="94" t="s">
         <v>59</v>
       </c>
@@ -22021,15 +22151,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B35:B38"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B87:B90"/>
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="B66:B69"/>
     <mergeCell ref="B70:B74"/>
@@ -22046,6 +22167,15 @@
     <mergeCell ref="B24:B30"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B87:B90"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
@@ -22053,6 +22183,53 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="c84b764c-50f3-4666-981f-a21c15460b9f">
+      <UserInfo>
+        <DisplayName>Sanchez Avalos, Roberto</DisplayName>
+        <AccountId>7</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Maria Reyes Retana Torre</DisplayName>
+        <AccountId>546</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Natalia Tosi</DisplayName>
+        <AccountId>929</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oliveri, Maria Laura</DisplayName>
+        <AccountId>1153</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Eric Torres</DisplayName>
+        <AccountId>474</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cdc7663a-08f0-4737-9e8c-148ce897a09c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100498A226200FBA747BF499A3F16BD9306" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a802e24b83766cc1d8af855be1bd7937">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f" xmlns:ns3="c84b764c-50f3-4666-981f-a21c15460b9f" xmlns:ns4="cdc7663a-08f0-4737-9e8c-148ce897a09c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6e8a154215ca5c893126bc8f6b108500" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f"/>
@@ -22300,54 +22477,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{283029C9-A5AB-4AAC-9B8A-368CAB8C733A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c84b764c-50f3-4666-981f-a21c15460b9f"/>
+    <ds:schemaRef ds:uri="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f"/>
+    <ds:schemaRef ds:uri="cdc7663a-08f0-4737-9e8c-148ce897a09c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="c84b764c-50f3-4666-981f-a21c15460b9f">
-      <UserInfo>
-        <DisplayName>Sanchez Avalos, Roberto</DisplayName>
-        <AccountId>7</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Maria Reyes Retana Torre</DisplayName>
-        <AccountId>546</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Natalia Tosi</DisplayName>
-        <AccountId>929</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oliveri, Maria Laura</DisplayName>
-        <AccountId>1153</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Eric Torres</DisplayName>
-        <AccountId>474</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cdc7663a-08f0-4737-9e8c-148ce897a09c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5341BEEE-99C0-4ED9-8E19-6F685D668845}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8D9694B-F156-44C8-A40A-23B2416BDA15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22365,24 +22515,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5341BEEE-99C0-4ED9-8E19-6F685D668845}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{283029C9-A5AB-4AAC-9B8A-368CAB8C733A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c84b764c-50f3-4666-981f-a21c15460b9f"/>
-    <ds:schemaRef ds:uri="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f"/>
-    <ds:schemaRef ds:uri="cdc7663a-08f0-4737-9e8c-148ce897a09c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix conditional check for restricted access
Updated the restriction check to use isTRUE to correctly handle missing values (public as default). Also updated the Excel input file since some public surveys were listed as restricted.
</commit_message>
<xml_diff>
--- a/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
+++ b/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/dcor_iadb_org/Documents/Documents/GitHub/calculo_indicators_R/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/matiasi_iadb_org/Documents/Documents/Github/calculo_indicators_R/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3044" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDDD835A-FF03-4E4D-942B-5CC5601DEF85}"/>
+  <xr:revisionPtr revIDLastSave="3050" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A67BFB29-5B16-4AC6-99FB-B5C3FD593252}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34290" yWindow="3550" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Encuestas Armonizadas" sheetId="2" state="hidden" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId8"/>
+    <pivotCache cacheId="7" r:id="rId8"/>
   </pivotCaches>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
@@ -2058,7 +2058,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="235">
+  <cellXfs count="226">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2607,25 +2607,25 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2725,33 +2725,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5121,7 +5094,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{963ADC1E-6961-40E2-8B9B-709AC1AD34EB}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{963ADC1E-6961-40E2-8B9B-709AC1AD34EB}" name="PivotTable4" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:U32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -5723,59 +5696,59 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BW61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" style="52" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" style="55" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="55" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" style="55" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" style="55" customWidth="1"/>
     <col min="4" max="4" width="11" style="55" bestFit="1" customWidth="1"/>
-    <col min="5" max="39" width="4.26953125" style="52" customWidth="1"/>
-    <col min="40" max="40" width="12.26953125" style="52" customWidth="1"/>
-    <col min="41" max="41" width="17.7265625" style="52" customWidth="1"/>
-    <col min="42" max="42" width="14.453125" style="52" customWidth="1"/>
+    <col min="5" max="39" width="4.28515625" style="52" customWidth="1"/>
+    <col min="40" max="40" width="12.28515625" style="52" customWidth="1"/>
+    <col min="41" max="41" width="17.7109375" style="52" customWidth="1"/>
+    <col min="42" max="42" width="14.42578125" style="52" customWidth="1"/>
     <col min="43" max="45" width="9" style="53"/>
     <col min="46" max="16384" width="9" style="55"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:75" ht="14.5" x14ac:dyDescent="0.3">
-      <c r="B1" s="186" t="s">
+    <row r="1" spans="1:75" ht="15" x14ac:dyDescent="0.2">
+      <c r="B1" s="191" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="186"/>
-      <c r="D1" s="186"/>
-      <c r="E1" s="186"/>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
-      <c r="I1" s="186"/>
-      <c r="J1" s="186"/>
-      <c r="K1" s="186"/>
-      <c r="L1" s="186"/>
-      <c r="M1" s="186"/>
-      <c r="N1" s="186"/>
-      <c r="O1" s="186"/>
-      <c r="P1" s="186"/>
-      <c r="Q1" s="186"/>
-      <c r="R1" s="186"/>
-      <c r="S1" s="186"/>
-      <c r="T1" s="186"/>
-      <c r="U1" s="186"/>
-      <c r="V1" s="186"/>
-      <c r="W1" s="186"/>
-      <c r="X1" s="186"/>
-      <c r="Y1" s="186"/>
-      <c r="Z1" s="186"/>
-      <c r="AA1" s="186"/>
-      <c r="AB1" s="186"/>
-      <c r="AC1" s="186"/>
-      <c r="AD1" s="186"/>
-      <c r="AE1" s="186"/>
-      <c r="AF1" s="186"/>
-      <c r="AG1" s="186"/>
-      <c r="AH1" s="186"/>
-      <c r="AI1" s="186"/>
-      <c r="AJ1" s="186"/>
-      <c r="AK1" s="186"/>
+      <c r="C1" s="191"/>
+      <c r="D1" s="191"/>
+      <c r="E1" s="191"/>
+      <c r="F1" s="191"/>
+      <c r="G1" s="191"/>
+      <c r="H1" s="191"/>
+      <c r="I1" s="191"/>
+      <c r="J1" s="191"/>
+      <c r="K1" s="191"/>
+      <c r="L1" s="191"/>
+      <c r="M1" s="191"/>
+      <c r="N1" s="191"/>
+      <c r="O1" s="191"/>
+      <c r="P1" s="191"/>
+      <c r="Q1" s="191"/>
+      <c r="R1" s="191"/>
+      <c r="S1" s="191"/>
+      <c r="T1" s="191"/>
+      <c r="U1" s="191"/>
+      <c r="V1" s="191"/>
+      <c r="W1" s="191"/>
+      <c r="X1" s="191"/>
+      <c r="Y1" s="191"/>
+      <c r="Z1" s="191"/>
+      <c r="AA1" s="191"/>
+      <c r="AB1" s="191"/>
+      <c r="AC1" s="191"/>
+      <c r="AD1" s="191"/>
+      <c r="AE1" s="191"/>
+      <c r="AF1" s="191"/>
+      <c r="AG1" s="191"/>
+      <c r="AH1" s="191"/>
+      <c r="AI1" s="191"/>
+      <c r="AJ1" s="191"/>
+      <c r="AK1" s="191"/>
       <c r="AL1" s="51"/>
       <c r="AM1" s="83"/>
       <c r="AN1" s="51"/>
@@ -5812,7 +5785,7 @@
       <c r="BV1" s="54"/>
       <c r="BW1" s="54"/>
     </row>
-    <row r="2" spans="1:75" ht="55.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:75" ht="55.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="145" t="s">
         <v>1</v>
       </c>
@@ -5940,11 +5913,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="188" t="s">
+      <c r="B3" s="186" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="57" t="s">
@@ -6036,9 +6009,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="145"/>
-      <c r="B4" s="189"/>
+      <c r="B4" s="187"/>
       <c r="C4" s="57" t="s">
         <v>14</v>
       </c>
@@ -6106,7 +6079,7 @@
       <c r="AO4" s="40"/>
       <c r="AP4" s="76"/>
     </row>
-    <row r="5" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="145" t="b">
         <v>1</v>
       </c>
@@ -6188,7 +6161,7 @@
       </c>
       <c r="AP5" s="76"/>
     </row>
-    <row r="6" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="145" t="b">
         <v>1</v>
       </c>
@@ -6270,11 +6243,11 @@
       </c>
       <c r="AP6" s="79"/>
     </row>
-    <row r="7" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="190" t="s">
+      <c r="B7" s="189" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="57" t="s">
@@ -6368,9 +6341,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="145"/>
-      <c r="B8" s="190"/>
+      <c r="B8" s="189"/>
       <c r="C8" s="57" t="s">
         <v>26</v>
       </c>
@@ -6426,9 +6399,9 @@
       <c r="AO8" s="40"/>
       <c r="AP8" s="76"/>
     </row>
-    <row r="9" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="145"/>
-      <c r="B9" s="190"/>
+      <c r="B9" s="189"/>
       <c r="C9" s="57" t="s">
         <v>27</v>
       </c>
@@ -6476,9 +6449,9 @@
       <c r="AO9" s="40"/>
       <c r="AP9" s="76"/>
     </row>
-    <row r="10" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="145"/>
-      <c r="B10" s="190" t="s">
+      <c r="B10" s="189" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="39" t="s">
@@ -6568,11 +6541,11 @@
       <c r="AO10" s="80"/>
       <c r="AP10" s="79"/>
     </row>
-    <row r="11" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="190"/>
+      <c r="B11" s="189"/>
       <c r="C11" s="39" t="s">
         <v>30</v>
       </c>
@@ -6636,7 +6609,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:75" ht="12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:75" ht="12" x14ac:dyDescent="0.2">
       <c r="A12" s="145" t="b">
         <v>1</v>
       </c>
@@ -6720,7 +6693,7 @@
       </c>
       <c r="AP12" s="79"/>
     </row>
-    <row r="13" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:75" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="145" t="b">
         <v>1</v>
       </c>
@@ -6806,9 +6779,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="145"/>
-      <c r="B14" s="188" t="s">
+      <c r="B14" s="186" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="39" t="s">
@@ -6864,9 +6837,9 @@
       <c r="AO14" s="40"/>
       <c r="AP14" s="76"/>
     </row>
-    <row r="15" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="145"/>
-      <c r="B15" s="191"/>
+      <c r="B15" s="188"/>
       <c r="C15" s="39" t="s">
         <v>39</v>
       </c>
@@ -6912,9 +6885,9 @@
       <c r="AO15" s="40"/>
       <c r="AP15" s="76"/>
     </row>
-    <row r="16" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="145"/>
-      <c r="B16" s="191"/>
+      <c r="B16" s="188"/>
       <c r="C16" s="39" t="s">
         <v>40</v>
       </c>
@@ -6982,11 +6955,11 @@
       <c r="AO16" s="40"/>
       <c r="AP16" s="76"/>
     </row>
-    <row r="17" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B17" s="189"/>
+      <c r="B17" s="187"/>
       <c r="C17" s="39" t="s">
         <v>41</v>
       </c>
@@ -7070,9 +7043,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="145"/>
-      <c r="B18" s="188" t="s">
+      <c r="B18" s="186" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="41" t="s">
@@ -7158,11 +7131,11 @@
       <c r="AO18" s="40"/>
       <c r="AP18" s="76"/>
     </row>
-    <row r="19" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B19" s="189"/>
+      <c r="B19" s="187"/>
       <c r="C19" s="57" t="s">
         <v>45</v>
       </c>
@@ -7238,9 +7211,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="145"/>
-      <c r="B20" s="188" t="s">
+      <c r="B20" s="186" t="s">
         <v>48</v>
       </c>
       <c r="C20" s="57" t="s">
@@ -7326,11 +7299,11 @@
       <c r="AO20" s="80"/>
       <c r="AP20" s="79"/>
     </row>
-    <row r="21" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B21" s="189"/>
+      <c r="B21" s="187"/>
       <c r="C21" s="57" t="s">
         <v>50</v>
       </c>
@@ -7390,11 +7363,11 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B22" s="190" t="s">
+      <c r="B22" s="189" t="s">
         <v>53</v>
       </c>
       <c r="C22" s="57" t="s">
@@ -7512,9 +7485,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="145"/>
-      <c r="B23" s="190"/>
+      <c r="B23" s="189"/>
       <c r="C23" s="57" t="s">
         <v>57</v>
       </c>
@@ -7566,9 +7539,9 @@
       <c r="AO23" s="80"/>
       <c r="AP23" s="79"/>
     </row>
-    <row r="24" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="145"/>
-      <c r="B24" s="190" t="s">
+      <c r="B24" s="189" t="s">
         <v>58</v>
       </c>
       <c r="C24" s="57" t="s">
@@ -7620,11 +7593,11 @@
       <c r="AO24" s="40"/>
       <c r="AP24" s="76"/>
     </row>
-    <row r="25" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="190"/>
+      <c r="B25" s="189"/>
       <c r="C25" s="57" t="s">
         <v>60</v>
       </c>
@@ -7704,9 +7677,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:42" ht="12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:42" ht="12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="145"/>
-      <c r="B26" s="190"/>
+      <c r="B26" s="189"/>
       <c r="C26" s="57" t="s">
         <v>62</v>
       </c>
@@ -7752,7 +7725,7 @@
       <c r="AO26" s="40"/>
       <c r="AP26" s="76"/>
     </row>
-    <row r="27" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="145" t="b">
         <v>1</v>
       </c>
@@ -7872,11 +7845,11 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:42" ht="10.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:42" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B28" s="188" t="s">
+      <c r="B28" s="186" t="s">
         <v>65</v>
       </c>
       <c r="C28" s="57" t="s">
@@ -7978,9 +7951,9 @@
       </c>
       <c r="AP28" s="76"/>
     </row>
-    <row r="29" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="145"/>
-      <c r="B29" s="189"/>
+      <c r="B29" s="187"/>
       <c r="C29" s="57" t="s">
         <v>67</v>
       </c>
@@ -8042,7 +8015,7 @@
       <c r="AO29" s="40"/>
       <c r="AP29" s="76"/>
     </row>
-    <row r="30" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="145" t="b">
         <v>1</v>
       </c>
@@ -8132,9 +8105,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="145"/>
-      <c r="B31" s="188" t="s">
+      <c r="B31" s="186" t="s">
         <v>73</v>
       </c>
       <c r="C31" s="57" t="s">
@@ -8186,11 +8159,11 @@
       <c r="AO31" s="40"/>
       <c r="AP31" s="76"/>
     </row>
-    <row r="32" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B32" s="189"/>
+      <c r="B32" s="187"/>
       <c r="C32" s="57" t="s">
         <v>74</v>
       </c>
@@ -8254,9 +8227,9 @@
       </c>
       <c r="AP32" s="76"/>
     </row>
-    <row r="33" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="145"/>
-      <c r="B33" s="188" t="s">
+      <c r="B33" s="186" t="s">
         <v>76</v>
       </c>
       <c r="C33" s="57" t="s">
@@ -8336,11 +8309,11 @@
       <c r="AO33" s="40"/>
       <c r="AP33" s="76"/>
     </row>
-    <row r="34" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B34" s="189"/>
+      <c r="B34" s="187"/>
       <c r="C34" s="57" t="s">
         <v>44</v>
       </c>
@@ -8412,9 +8385,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="145"/>
-      <c r="B35" s="188" t="s">
+      <c r="B35" s="186" t="s">
         <v>79</v>
       </c>
       <c r="C35" s="57" t="s">
@@ -8476,9 +8449,9 @@
       </c>
       <c r="AP35" s="76"/>
     </row>
-    <row r="36" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="145"/>
-      <c r="B36" s="191"/>
+      <c r="B36" s="188"/>
       <c r="C36" s="57" t="s">
         <v>26</v>
       </c>
@@ -8492,15 +8465,15 @@
       <c r="K36" s="80"/>
       <c r="L36" s="80"/>
       <c r="M36" s="80"/>
-      <c r="N36" s="187">
-        <v>1</v>
-      </c>
-      <c r="O36" s="187"/>
+      <c r="N36" s="192">
+        <v>1</v>
+      </c>
+      <c r="O36" s="192"/>
       <c r="P36" s="80"/>
-      <c r="Q36" s="187">
-        <v>1</v>
-      </c>
-      <c r="R36" s="187"/>
+      <c r="Q36" s="192">
+        <v>1</v>
+      </c>
+      <c r="R36" s="192"/>
       <c r="S36" s="80"/>
       <c r="T36" s="80"/>
       <c r="U36" s="80"/>
@@ -8528,9 +8501,9 @@
       </c>
       <c r="AP36" s="76"/>
     </row>
-    <row r="37" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="145"/>
-      <c r="B37" s="191"/>
+      <c r="B37" s="188"/>
       <c r="C37" s="57" t="s">
         <v>82</v>
       </c>
@@ -8610,11 +8583,11 @@
       </c>
       <c r="AP37" s="79"/>
     </row>
-    <row r="38" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B38" s="189"/>
+      <c r="B38" s="187"/>
       <c r="C38" s="57" t="s">
         <v>9</v>
       </c>
@@ -8674,11 +8647,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B39" s="188" t="s">
+      <c r="B39" s="186" t="s">
         <v>83</v>
       </c>
       <c r="C39" s="57" t="s">
@@ -8782,9 +8755,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="145"/>
-      <c r="B40" s="189"/>
+      <c r="B40" s="187"/>
       <c r="C40" s="57" t="s">
         <v>84</v>
       </c>
@@ -8838,7 +8811,7 @@
       </c>
       <c r="AP40" s="79"/>
     </row>
-    <row r="41" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="145" t="b">
         <v>1</v>
       </c>
@@ -8950,7 +8923,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="145" t="b">
         <v>1</v>
       </c>
@@ -9072,9 +9045,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="145"/>
-      <c r="B43" s="188" t="s">
+      <c r="B43" s="186" t="s">
         <v>87</v>
       </c>
       <c r="C43" s="57" t="s">
@@ -9172,11 +9145,11 @@
       <c r="AO43" s="80"/>
       <c r="AP43" s="79"/>
     </row>
-    <row r="44" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B44" s="189"/>
+      <c r="B44" s="187"/>
       <c r="C44" s="41" t="s">
         <v>59</v>
       </c>
@@ -9244,7 +9217,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="145"/>
       <c r="B45" s="86" t="s">
         <v>88</v>
@@ -9290,7 +9263,7 @@
       <c r="AO45" s="40"/>
       <c r="AP45" s="76"/>
     </row>
-    <row r="46" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="145"/>
       <c r="B46" s="86" t="s">
         <v>89</v>
@@ -9336,7 +9309,7 @@
       <c r="AO46" s="40"/>
       <c r="AP46" s="76"/>
     </row>
-    <row r="47" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C47" s="55" t="s">
         <v>90</v>
       </c>
@@ -9482,7 +9455,7 @@
       </c>
       <c r="AP47" s="1"/>
     </row>
-    <row r="48" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:42" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C48" s="55" t="s">
         <v>91</v>
       </c>
@@ -9627,7 +9600,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="49" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AE49" s="156" t="s">
         <v>92</v>
       </c>
@@ -9649,7 +9622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AK51" s="149">
         <v>1</v>
       </c>
@@ -9657,7 +9630,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AK52" s="77">
         <v>1</v>
       </c>
@@ -9667,7 +9640,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AK53" s="82">
         <v>1</v>
       </c>
@@ -9677,7 +9650,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="54" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AK54" s="78">
         <v>1</v>
       </c>
@@ -9687,46 +9660,46 @@
         <v>96</v>
       </c>
     </row>
-    <row r="58" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C58" s="192" t="s">
+    <row r="58" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C58" s="190" t="s">
         <v>97</v>
       </c>
-      <c r="D58" s="192"/>
-      <c r="E58" s="192"/>
-      <c r="F58" s="192"/>
-      <c r="G58" s="192"/>
-      <c r="H58" s="192"/>
-      <c r="I58" s="192"/>
-      <c r="J58" s="192"/>
-      <c r="K58" s="192"/>
-      <c r="L58" s="192"/>
-      <c r="M58" s="192"/>
-      <c r="N58" s="192"/>
-      <c r="O58" s="192"/>
-      <c r="P58" s="192"/>
-      <c r="Q58" s="192"/>
-      <c r="R58" s="192"/>
-      <c r="S58" s="192"/>
-      <c r="T58" s="192"/>
-      <c r="U58" s="192"/>
-      <c r="V58" s="192"/>
-      <c r="W58" s="192"/>
-      <c r="X58" s="192"/>
-      <c r="Y58" s="192"/>
-      <c r="Z58" s="192"/>
-      <c r="AA58" s="192"/>
-      <c r="AB58" s="192"/>
-      <c r="AC58" s="192"/>
-      <c r="AD58" s="192"/>
-      <c r="AE58" s="192"/>
-      <c r="AF58" s="192"/>
-      <c r="AG58" s="192"/>
-      <c r="AH58" s="192"/>
-      <c r="AI58" s="192"/>
-      <c r="AJ58" s="192"/>
-      <c r="AK58" s="192"/>
-    </row>
-    <row r="59" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D58" s="190"/>
+      <c r="E58" s="190"/>
+      <c r="F58" s="190"/>
+      <c r="G58" s="190"/>
+      <c r="H58" s="190"/>
+      <c r="I58" s="190"/>
+      <c r="J58" s="190"/>
+      <c r="K58" s="190"/>
+      <c r="L58" s="190"/>
+      <c r="M58" s="190"/>
+      <c r="N58" s="190"/>
+      <c r="O58" s="190"/>
+      <c r="P58" s="190"/>
+      <c r="Q58" s="190"/>
+      <c r="R58" s="190"/>
+      <c r="S58" s="190"/>
+      <c r="T58" s="190"/>
+      <c r="U58" s="190"/>
+      <c r="V58" s="190"/>
+      <c r="W58" s="190"/>
+      <c r="X58" s="190"/>
+      <c r="Y58" s="190"/>
+      <c r="Z58" s="190"/>
+      <c r="AA58" s="190"/>
+      <c r="AB58" s="190"/>
+      <c r="AC58" s="190"/>
+      <c r="AD58" s="190"/>
+      <c r="AE58" s="190"/>
+      <c r="AF58" s="190"/>
+      <c r="AG58" s="190"/>
+      <c r="AH58" s="190"/>
+      <c r="AI58" s="190"/>
+      <c r="AJ58" s="190"/>
+      <c r="AK58" s="190"/>
+    </row>
+    <row r="59" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C59" s="147" t="s">
         <v>98</v>
       </c>
@@ -9765,7 +9738,7 @@
       <c r="AJ59" s="146"/>
       <c r="AK59" s="146"/>
     </row>
-    <row r="60" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C60" s="147" t="s">
         <v>99</v>
       </c>
@@ -9804,7 +9777,7 @@
       <c r="AJ60" s="146"/>
       <c r="AK60" s="146"/>
     </row>
-    <row r="61" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C61" s="147" t="s">
         <v>100</v>
       </c>
@@ -9845,8 +9818,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C58:AK58"/>
     <mergeCell ref="B1:AK1"/>
     <mergeCell ref="Q36:R36"/>
     <mergeCell ref="B39:B40"/>
@@ -9863,6 +9834,8 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C58:AK58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" r:id="rId1"/>
@@ -9872,13 +9845,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B92816-9A9B-481E-B050-65BD5C8E1CB2}">
   <dimension ref="A3:V32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="21" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="21" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>461</v>
       </c>
@@ -9943,7 +9916,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="104" t="s">
         <v>484</v>
       </c>
@@ -10012,7 +9985,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="173" t="s">
         <v>15</v>
       </c>
@@ -10050,7 +10023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="173" t="s">
         <v>22</v>
       </c>
@@ -10106,7 +10079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="173" t="s">
         <v>32</v>
       </c>
@@ -10150,7 +10123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="173" t="s">
         <v>48</v>
       </c>
@@ -10212,7 +10185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="173" t="s">
         <v>58</v>
       </c>
@@ -10262,7 +10235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="173" t="s">
         <v>63</v>
       </c>
@@ -10318,7 +10291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="173" t="s">
         <v>65</v>
       </c>
@@ -10365,7 +10338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="173" t="s">
         <v>73</v>
       </c>
@@ -10388,7 +10361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="173" t="s">
         <v>83</v>
       </c>
@@ -10450,7 +10423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="173" t="s">
         <v>85</v>
       </c>
@@ -10515,7 +10488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="173" t="s">
         <v>88</v>
       </c>
@@ -10559,7 +10532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="173" t="s">
         <v>87</v>
       </c>
@@ -10618,7 +10591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="104" t="s">
         <v>483</v>
       </c>
@@ -10687,7 +10660,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="173" t="s">
         <v>8</v>
       </c>
@@ -10756,7 +10729,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="173" t="s">
         <v>20</v>
       </c>
@@ -10777,7 +10750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="173" t="s">
         <v>28</v>
       </c>
@@ -10843,7 +10816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="173" t="s">
         <v>34</v>
       </c>
@@ -10876,7 +10849,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="173" t="s">
         <v>38</v>
       </c>
@@ -10942,7 +10915,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="173" t="s">
         <v>43</v>
       </c>
@@ -11011,7 +10984,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="173" t="s">
         <v>53</v>
       </c>
@@ -11080,7 +11053,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="173" t="s">
         <v>170</v>
       </c>
@@ -11101,7 +11074,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="173" t="s">
         <v>154</v>
       </c>
@@ -11113,7 +11086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="173" t="s">
         <v>68</v>
       </c>
@@ -11152,7 +11125,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="173" t="s">
         <v>76</v>
       </c>
@@ -11215,7 +11188,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="173" t="s">
         <v>79</v>
       </c>
@@ -11281,7 +11254,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="173" t="s">
         <v>89</v>
       </c>
@@ -11293,7 +11266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="173" t="s">
         <v>86</v>
       </c>
@@ -11362,7 +11335,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="104" t="s">
         <v>478</v>
       </c>
@@ -11435,9 +11408,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA588299-A923-4948-B338-1E6680648B04}">
   <dimension ref="A1:V27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>461</v>
       </c>
@@ -11502,7 +11475,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>484</v>
       </c>
@@ -11543,7 +11516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>484</v>
       </c>
@@ -11602,7 +11575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>484</v>
       </c>
@@ -11649,7 +11622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>484</v>
       </c>
@@ -11714,7 +11687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>484</v>
       </c>
@@ -11767,7 +11740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>484</v>
       </c>
@@ -11826,7 +11799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>484</v>
       </c>
@@ -11876,7 +11849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>484</v>
       </c>
@@ -11902,7 +11875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>484</v>
       </c>
@@ -11967,7 +11940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>484</v>
       </c>
@@ -12035,7 +12008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>484</v>
       </c>
@@ -12082,7 +12055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>484</v>
       </c>
@@ -12144,7 +12117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>483</v>
       </c>
@@ -12212,7 +12185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>483</v>
       </c>
@@ -12232,7 +12205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>483</v>
       </c>
@@ -12297,7 +12270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>483</v>
       </c>
@@ -12329,7 +12302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>483</v>
       </c>
@@ -12394,7 +12367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>483</v>
       </c>
@@ -12462,7 +12435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>483</v>
       </c>
@@ -12530,7 +12503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>483</v>
       </c>
@@ -12550,7 +12523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>483</v>
       </c>
@@ -12561,7 +12534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>483</v>
       </c>
@@ -12599,7 +12572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>483</v>
       </c>
@@ -12661,7 +12634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>483</v>
       </c>
@@ -12726,7 +12699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>483</v>
       </c>
@@ -12737,7 +12710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>483</v>
       </c>
@@ -12817,16 +12790,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC0F423-732A-4BB5-B708-202F80FAD9CB}">
   <dimension ref="A1:AP96"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12" style="100" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1796875" style="100" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="38" width="8.1796875" style="100" bestFit="1" customWidth="1"/>
-    <col min="39" max="40" width="8.1796875" style="100" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="100" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="38" width="8.140625" style="100" bestFit="1" customWidth="1"/>
+    <col min="39" max="40" width="8.140625" style="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" ht="36" x14ac:dyDescent="0.25">
       <c r="A1" s="174" t="s">
         <v>2</v>
       </c>
@@ -12954,7 +12927,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" s="157" t="s">
         <v>8</v>
       </c>
@@ -13029,7 +13002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" s="157" t="s">
         <v>8</v>
       </c>
@@ -13126,7 +13099,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" s="157" t="s">
         <v>8</v>
       </c>
@@ -13183,7 +13156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" s="157" t="s">
         <v>15</v>
       </c>
@@ -13276,7 +13249,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" s="157" t="s">
         <v>20</v>
       </c>
@@ -13347,7 +13320,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" s="157" t="s">
         <v>20</v>
       </c>
@@ -13412,7 +13385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" s="157" t="s">
         <v>20</v>
       </c>
@@ -13469,7 +13442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" s="157" t="s">
         <v>22</v>
       </c>
@@ -13530,7 +13503,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" s="157" t="s">
         <v>22</v>
       </c>
@@ -13585,7 +13558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" s="157" t="s">
         <v>22</v>
       </c>
@@ -13640,7 +13613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" s="157" t="s">
         <v>22</v>
       </c>
@@ -13695,7 +13668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A13" s="157" t="s">
         <v>22</v>
       </c>
@@ -13750,7 +13723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" s="157" t="s">
         <v>22</v>
       </c>
@@ -13805,7 +13778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" s="157" t="s">
         <v>22</v>
       </c>
@@ -13882,7 +13855,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A16" s="157" t="s">
         <v>22</v>
       </c>
@@ -13955,7 +13928,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A17" s="157" t="s">
         <v>28</v>
       </c>
@@ -14054,7 +14027,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A18" s="157" t="s">
         <v>28</v>
       </c>
@@ -14127,7 +14100,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A19" s="157" t="s">
         <v>32</v>
       </c>
@@ -14208,7 +14181,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A20" s="157" t="s">
         <v>32</v>
       </c>
@@ -14265,64 +14238,64 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.35">
-      <c r="A21" s="226" t="s">
+    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A21" s="157" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="227" t="s">
+      <c r="B21" s="57" t="s">
         <v>510</v>
       </c>
       <c r="C21" s="162" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D21" s="69" t="s">
-        <v>145</v>
-      </c>
-      <c r="E21" s="230"/>
-      <c r="F21" s="230"/>
-      <c r="G21" s="230"/>
-      <c r="H21" s="230"/>
-      <c r="I21" s="230"/>
-      <c r="J21" s="230"/>
-      <c r="K21" s="230"/>
-      <c r="L21" s="230"/>
-      <c r="M21" s="230"/>
-      <c r="N21" s="230"/>
-      <c r="O21" s="230"/>
-      <c r="P21" s="230"/>
-      <c r="Q21" s="230"/>
-      <c r="R21" s="230"/>
-      <c r="S21" s="230"/>
-      <c r="T21" s="230"/>
-      <c r="U21" s="230"/>
-      <c r="V21" s="230"/>
-      <c r="W21" s="230"/>
-      <c r="X21" s="230"/>
-      <c r="Y21" s="230"/>
-      <c r="Z21" s="230"/>
-      <c r="AA21" s="230"/>
-      <c r="AB21" s="230"/>
+        <v>17</v>
+      </c>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="80"/>
+      <c r="J21" s="80"/>
+      <c r="K21" s="80"/>
+      <c r="L21" s="80"/>
+      <c r="M21" s="80"/>
+      <c r="N21" s="80"/>
+      <c r="O21" s="80"/>
+      <c r="P21" s="80"/>
+      <c r="Q21" s="80"/>
+      <c r="R21" s="80"/>
+      <c r="S21" s="80"/>
+      <c r="T21" s="80"/>
+      <c r="U21" s="80"/>
+      <c r="V21" s="80"/>
+      <c r="W21" s="80"/>
+      <c r="X21" s="80"/>
+      <c r="Y21" s="80"/>
+      <c r="Z21" s="80"/>
+      <c r="AA21" s="80"/>
+      <c r="AB21" s="80"/>
       <c r="AC21" s="80"/>
       <c r="AD21" s="80"/>
-      <c r="AE21" s="230"/>
-      <c r="AF21" s="230"/>
+      <c r="AE21" s="80"/>
+      <c r="AF21" s="80"/>
       <c r="AG21" s="80"/>
       <c r="AH21" s="80"/>
       <c r="AI21" s="80"/>
       <c r="AJ21" s="80"/>
       <c r="AK21" s="80"/>
-      <c r="AL21" s="231"/>
-      <c r="AM21" s="232"/>
-      <c r="AN21" s="232"/>
-      <c r="AO21" s="232">
-        <v>1</v>
-      </c>
-      <c r="AP21" s="233">
+      <c r="AL21" s="159"/>
+      <c r="AM21" s="171"/>
+      <c r="AN21" s="171"/>
+      <c r="AO21" s="171">
+        <v>1</v>
+      </c>
+      <c r="AP21" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A22" s="157" t="s">
         <v>34</v>
       </c>
@@ -14393,7 +14366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A23" s="157" t="s">
         <v>34</v>
       </c>
@@ -14458,7 +14431,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A24" s="157" t="s">
         <v>38</v>
       </c>
@@ -14535,7 +14508,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A25" s="157" t="s">
         <v>38</v>
       </c>
@@ -14600,7 +14573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A26" s="157" t="s">
         <v>38</v>
       </c>
@@ -14691,7 +14664,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A27" s="157" t="s">
         <v>38</v>
       </c>
@@ -14748,7 +14721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A28" s="157" t="s">
         <v>43</v>
       </c>
@@ -14843,7 +14816,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A29" s="157" t="s">
         <v>43</v>
       </c>
@@ -14928,7 +14901,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A30" s="157" t="s">
         <v>48</v>
       </c>
@@ -14985,7 +14958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A31" s="157" t="s">
         <v>48</v>
       </c>
@@ -15042,7 +15015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A32" s="157" t="s">
         <v>48</v>
       </c>
@@ -15099,7 +15072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A33" s="157" t="s">
         <v>48</v>
       </c>
@@ -15188,7 +15161,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A34" s="157" t="s">
         <v>48</v>
       </c>
@@ -15196,7 +15169,7 @@
         <v>50</v>
       </c>
       <c r="C34" s="69" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D34" s="69" t="s">
         <v>51</v>
@@ -15259,7 +15232,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A35" s="157" t="s">
         <v>53</v>
       </c>
@@ -15336,7 +15309,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A36" s="157" t="s">
         <v>53</v>
       </c>
@@ -15435,7 +15408,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A37" s="157" t="s">
         <v>58</v>
       </c>
@@ -15492,62 +15465,62 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A38" s="157" t="s">
         <v>58</v>
       </c>
       <c r="B38" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="228"/>
-      <c r="D38" s="229" t="s">
+      <c r="C38" s="163"/>
+      <c r="D38" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="E38" s="230"/>
-      <c r="F38" s="230"/>
-      <c r="G38" s="230"/>
-      <c r="H38" s="230"/>
-      <c r="I38" s="230"/>
-      <c r="J38" s="230"/>
-      <c r="K38" s="230"/>
-      <c r="L38" s="230"/>
-      <c r="M38" s="230"/>
-      <c r="N38" s="230"/>
-      <c r="O38" s="234"/>
-      <c r="P38" s="234"/>
-      <c r="Q38" s="230"/>
-      <c r="R38" s="234"/>
-      <c r="S38" s="234"/>
-      <c r="T38" s="234"/>
-      <c r="U38" s="234"/>
-      <c r="V38" s="234"/>
-      <c r="W38" s="230"/>
-      <c r="X38" s="234"/>
-      <c r="Y38" s="234"/>
-      <c r="Z38" s="234"/>
-      <c r="AA38" s="234"/>
-      <c r="AB38" s="230"/>
+      <c r="E38" s="80"/>
+      <c r="F38" s="80"/>
+      <c r="G38" s="80"/>
+      <c r="H38" s="80"/>
+      <c r="I38" s="80"/>
+      <c r="J38" s="80"/>
+      <c r="K38" s="80"/>
+      <c r="L38" s="80"/>
+      <c r="M38" s="80"/>
+      <c r="N38" s="80"/>
+      <c r="O38" s="40"/>
+      <c r="P38" s="40"/>
+      <c r="Q38" s="80"/>
+      <c r="R38" s="40"/>
+      <c r="S38" s="40"/>
+      <c r="T38" s="40"/>
+      <c r="U38" s="40"/>
+      <c r="V38" s="40"/>
+      <c r="W38" s="80"/>
+      <c r="X38" s="40"/>
+      <c r="Y38" s="40"/>
+      <c r="Z38" s="40"/>
+      <c r="AA38" s="40"/>
+      <c r="AB38" s="80"/>
       <c r="AC38" s="80"/>
       <c r="AD38" s="40"/>
-      <c r="AE38" s="230"/>
-      <c r="AF38" s="230"/>
+      <c r="AE38" s="80"/>
+      <c r="AF38" s="80"/>
       <c r="AG38" s="40"/>
       <c r="AH38" s="40"/>
       <c r="AI38" s="40"/>
       <c r="AJ38" s="40"/>
       <c r="AK38" s="40"/>
-      <c r="AL38" s="231"/>
-      <c r="AM38" s="232"/>
-      <c r="AN38" s="232">
-        <v>1</v>
-      </c>
-      <c r="AO38" s="232"/>
-      <c r="AP38" s="233">
+      <c r="AL38" s="159"/>
+      <c r="AM38" s="171"/>
+      <c r="AN38" s="171">
+        <v>1</v>
+      </c>
+      <c r="AO38" s="171"/>
+      <c r="AP38" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A39" s="157" t="s">
         <v>58</v>
       </c>
@@ -15602,7 +15575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A40" s="157" t="s">
         <v>58</v>
       </c>
@@ -15657,7 +15630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A41" s="157" t="s">
         <v>58</v>
       </c>
@@ -15712,7 +15685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A42" s="157" t="s">
         <v>58</v>
       </c>
@@ -15779,7 +15752,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A43" s="157" t="s">
         <v>58</v>
       </c>
@@ -15834,7 +15807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A44" s="181" t="s">
         <v>58</v>
       </c>
@@ -15889,7 +15862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A45" s="157" t="s">
         <v>58</v>
       </c>
@@ -15946,7 +15919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A46" s="157" t="s">
         <v>58</v>
       </c>
@@ -16003,7 +15976,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A47" s="157" t="s">
         <v>63</v>
       </c>
@@ -16082,7 +16055,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A48" s="157" t="s">
         <v>63</v>
       </c>
@@ -16139,7 +16112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A49" s="157" t="s">
         <v>63</v>
       </c>
@@ -16200,7 +16173,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A50" s="157" t="s">
         <v>63</v>
       </c>
@@ -16265,7 +16238,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A51" s="157" t="s">
         <v>63</v>
       </c>
@@ -16336,7 +16309,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A52" s="157" t="s">
         <v>154</v>
       </c>
@@ -16391,7 +16364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A53" s="157" t="s">
         <v>65</v>
       </c>
@@ -16450,7 +16423,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A54" s="157" t="s">
         <v>65</v>
       </c>
@@ -16547,7 +16520,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A55" s="157" t="s">
         <v>65</v>
       </c>
@@ -16610,7 +16583,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A56" s="157" t="s">
         <v>68</v>
       </c>
@@ -16675,7 +16648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A57" s="157" t="s">
         <v>68</v>
       </c>
@@ -16730,7 +16703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A58" s="157" t="s">
         <v>68</v>
       </c>
@@ -16785,7 +16758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A59" s="157" t="s">
         <v>68</v>
       </c>
@@ -16858,7 +16831,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A60" s="157" t="s">
         <v>73</v>
       </c>
@@ -16921,7 +16894,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A61" s="157" t="s">
         <v>73</v>
       </c>
@@ -16980,7 +16953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A62" s="157" t="s">
         <v>73</v>
       </c>
@@ -17041,7 +17014,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A63" s="157" t="s">
         <v>73</v>
       </c>
@@ -17098,7 +17071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A64" s="157" t="s">
         <v>76</v>
       </c>
@@ -17187,7 +17160,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="65" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A65" s="157" t="s">
         <v>76</v>
       </c>
@@ -17195,7 +17168,7 @@
         <v>44</v>
       </c>
       <c r="C65" s="69" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D65" s="69" t="s">
         <v>78</v>
@@ -17262,121 +17235,121 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:42" x14ac:dyDescent="0.35">
-      <c r="A66" s="226" t="s">
+    <row r="66" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A66" s="157" t="s">
         <v>76</v>
       </c>
       <c r="B66" s="57" t="s">
         <v>332</v>
       </c>
       <c r="C66" s="69" t="s">
-        <v>140</v>
-      </c>
-      <c r="D66" s="229" t="s">
+        <v>138</v>
+      </c>
+      <c r="D66" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="E66" s="230"/>
-      <c r="F66" s="230"/>
-      <c r="G66" s="230"/>
-      <c r="H66" s="230"/>
-      <c r="I66" s="230"/>
-      <c r="J66" s="230"/>
-      <c r="K66" s="230"/>
-      <c r="L66" s="230"/>
-      <c r="M66" s="230"/>
-      <c r="N66" s="230"/>
-      <c r="O66" s="230"/>
-      <c r="P66" s="230"/>
-      <c r="Q66" s="230"/>
-      <c r="R66" s="230"/>
-      <c r="S66" s="230"/>
-      <c r="T66" s="230"/>
-      <c r="U66" s="230"/>
-      <c r="V66" s="230"/>
-      <c r="W66" s="230"/>
-      <c r="X66" s="230"/>
-      <c r="Y66" s="230"/>
-      <c r="Z66" s="230"/>
-      <c r="AA66" s="230"/>
-      <c r="AB66" s="230"/>
+      <c r="E66" s="80"/>
+      <c r="F66" s="80"/>
+      <c r="G66" s="80"/>
+      <c r="H66" s="80"/>
+      <c r="I66" s="80"/>
+      <c r="J66" s="80"/>
+      <c r="K66" s="80"/>
+      <c r="L66" s="80"/>
+      <c r="M66" s="80"/>
+      <c r="N66" s="80"/>
+      <c r="O66" s="80"/>
+      <c r="P66" s="80"/>
+      <c r="Q66" s="80"/>
+      <c r="R66" s="80"/>
+      <c r="S66" s="80"/>
+      <c r="T66" s="80"/>
+      <c r="U66" s="80"/>
+      <c r="V66" s="80"/>
+      <c r="W66" s="80"/>
+      <c r="X66" s="80"/>
+      <c r="Y66" s="80"/>
+      <c r="Z66" s="80"/>
+      <c r="AA66" s="80"/>
+      <c r="AB66" s="80"/>
       <c r="AC66" s="80"/>
       <c r="AD66" s="40"/>
-      <c r="AE66" s="230"/>
-      <c r="AF66" s="230"/>
+      <c r="AE66" s="80"/>
+      <c r="AF66" s="80"/>
       <c r="AG66" s="40"/>
       <c r="AH66" s="40"/>
       <c r="AI66" s="40"/>
       <c r="AJ66" s="40"/>
       <c r="AK66" s="40"/>
-      <c r="AL66" s="231"/>
-      <c r="AM66" s="232"/>
-      <c r="AN66" s="232">
-        <v>1</v>
-      </c>
-      <c r="AO66" s="232"/>
-      <c r="AP66" s="233">
+      <c r="AL66" s="159"/>
+      <c r="AM66" s="171"/>
+      <c r="AN66" s="171">
+        <v>1</v>
+      </c>
+      <c r="AO66" s="171"/>
+      <c r="AP66" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:42" x14ac:dyDescent="0.35">
-      <c r="A67" s="226" t="s">
+    <row r="67" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A67" s="157" t="s">
         <v>76</v>
       </c>
       <c r="B67" s="57" t="s">
         <v>332</v>
       </c>
       <c r="C67" s="69" t="s">
-        <v>140</v>
-      </c>
-      <c r="D67" s="229" t="s">
+        <v>138</v>
+      </c>
+      <c r="D67" s="69" t="s">
         <v>137</v>
       </c>
-      <c r="E67" s="230"/>
-      <c r="F67" s="230"/>
-      <c r="G67" s="230"/>
-      <c r="H67" s="230"/>
-      <c r="I67" s="230"/>
-      <c r="J67" s="230"/>
-      <c r="K67" s="230"/>
-      <c r="L67" s="230"/>
-      <c r="M67" s="230"/>
-      <c r="N67" s="230"/>
-      <c r="O67" s="230"/>
-      <c r="P67" s="230"/>
-      <c r="Q67" s="230"/>
-      <c r="R67" s="230"/>
-      <c r="S67" s="230"/>
-      <c r="T67" s="230"/>
-      <c r="U67" s="230"/>
-      <c r="V67" s="230"/>
-      <c r="W67" s="230"/>
-      <c r="X67" s="230"/>
-      <c r="Y67" s="230"/>
-      <c r="Z67" s="230"/>
-      <c r="AA67" s="230"/>
-      <c r="AB67" s="230"/>
+      <c r="E67" s="80"/>
+      <c r="F67" s="80"/>
+      <c r="G67" s="80"/>
+      <c r="H67" s="80"/>
+      <c r="I67" s="80"/>
+      <c r="J67" s="80"/>
+      <c r="K67" s="80"/>
+      <c r="L67" s="80"/>
+      <c r="M67" s="80"/>
+      <c r="N67" s="80"/>
+      <c r="O67" s="80"/>
+      <c r="P67" s="80"/>
+      <c r="Q67" s="80"/>
+      <c r="R67" s="80"/>
+      <c r="S67" s="80"/>
+      <c r="T67" s="80"/>
+      <c r="U67" s="80"/>
+      <c r="V67" s="80"/>
+      <c r="W67" s="80"/>
+      <c r="X67" s="80"/>
+      <c r="Y67" s="80"/>
+      <c r="Z67" s="80"/>
+      <c r="AA67" s="80"/>
+      <c r="AB67" s="80"/>
       <c r="AC67" s="80"/>
       <c r="AD67" s="40"/>
-      <c r="AE67" s="230"/>
-      <c r="AF67" s="230"/>
+      <c r="AE67" s="80"/>
+      <c r="AF67" s="80"/>
       <c r="AG67" s="40"/>
       <c r="AH67" s="40"/>
       <c r="AI67" s="40"/>
       <c r="AJ67" s="40"/>
       <c r="AK67" s="40"/>
-      <c r="AL67" s="231"/>
-      <c r="AM67" s="232"/>
-      <c r="AN67" s="232"/>
-      <c r="AO67" s="232">
-        <v>1</v>
-      </c>
-      <c r="AP67" s="233">
+      <c r="AL67" s="159"/>
+      <c r="AM67" s="171"/>
+      <c r="AN67" s="171"/>
+      <c r="AO67" s="171">
+        <v>1</v>
+      </c>
+      <c r="AP67" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A68" s="157" t="s">
         <v>79</v>
       </c>
@@ -17431,7 +17404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A69" s="157" t="s">
         <v>79</v>
       </c>
@@ -17486,7 +17459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A70" s="157" t="s">
         <v>79</v>
       </c>
@@ -17541,7 +17514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A71" s="157" t="s">
         <v>79</v>
       </c>
@@ -17596,7 +17569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A72" s="157" t="s">
         <v>79</v>
       </c>
@@ -17651,7 +17624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A73" s="157" t="s">
         <v>79</v>
       </c>
@@ -17706,7 +17679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A74" s="157" t="s">
         <v>79</v>
       </c>
@@ -17761,7 +17734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A75" s="157" t="s">
         <v>79</v>
       </c>
@@ -17816,7 +17789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A76" s="157" t="s">
         <v>79</v>
       </c>
@@ -17871,7 +17844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A77" s="157" t="s">
         <v>79</v>
       </c>
@@ -17928,7 +17901,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A78" s="157" t="s">
         <v>79</v>
       </c>
@@ -17985,7 +17958,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A79" s="157" t="s">
         <v>79</v>
       </c>
@@ -18040,7 +18013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A80" s="157" t="s">
         <v>79</v>
       </c>
@@ -18117,7 +18090,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A81" s="157" t="s">
         <v>79</v>
       </c>
@@ -18182,7 +18155,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A82" s="157" t="s">
         <v>83</v>
       </c>
@@ -18239,7 +18212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A83" s="157" t="s">
         <v>83</v>
       </c>
@@ -18304,7 +18277,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A84" s="157" t="s">
         <v>83</v>
       </c>
@@ -18401,7 +18374,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="85" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A85" s="157" t="s">
         <v>85</v>
       </c>
@@ -18514,7 +18487,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="86" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A86" s="157" t="s">
         <v>86</v>
       </c>
@@ -18579,7 +18552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A87" s="157" t="s">
         <v>86</v>
       </c>
@@ -18690,7 +18663,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A88" s="157" t="s">
         <v>87</v>
       </c>
@@ -18795,7 +18768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A89" s="157" t="s">
         <v>87</v>
       </c>
@@ -18856,7 +18829,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A90" s="157" t="s">
         <v>87</v>
       </c>
@@ -18866,37 +18839,37 @@
       <c r="C90" s="69" t="s">
         <v>140</v>
       </c>
-      <c r="D90" s="229" t="s">
+      <c r="D90" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="E90" s="234"/>
-      <c r="F90" s="234"/>
-      <c r="G90" s="234"/>
-      <c r="H90" s="234"/>
-      <c r="I90" s="234"/>
-      <c r="J90" s="234"/>
-      <c r="K90" s="234"/>
-      <c r="L90" s="234"/>
-      <c r="M90" s="234"/>
-      <c r="N90" s="234"/>
-      <c r="O90" s="234"/>
-      <c r="P90" s="234"/>
-      <c r="Q90" s="234"/>
-      <c r="R90" s="234"/>
-      <c r="S90" s="234"/>
-      <c r="T90" s="234"/>
-      <c r="U90" s="234"/>
-      <c r="V90" s="234"/>
-      <c r="W90" s="234"/>
-      <c r="X90" s="234"/>
-      <c r="Y90" s="234"/>
-      <c r="Z90" s="234"/>
-      <c r="AA90" s="234"/>
-      <c r="AB90" s="234"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
+      <c r="G90" s="40"/>
+      <c r="H90" s="40"/>
+      <c r="I90" s="40"/>
+      <c r="J90" s="40"/>
+      <c r="K90" s="40"/>
+      <c r="L90" s="40"/>
+      <c r="M90" s="40"/>
+      <c r="N90" s="40"/>
+      <c r="O90" s="40"/>
+      <c r="P90" s="40"/>
+      <c r="Q90" s="40"/>
+      <c r="R90" s="40"/>
+      <c r="S90" s="40"/>
+      <c r="T90" s="40"/>
+      <c r="U90" s="40"/>
+      <c r="V90" s="40"/>
+      <c r="W90" s="40"/>
+      <c r="X90" s="40"/>
+      <c r="Y90" s="40"/>
+      <c r="Z90" s="40"/>
+      <c r="AA90" s="40"/>
+      <c r="AB90" s="40"/>
       <c r="AC90" s="40"/>
       <c r="AD90" s="40"/>
-      <c r="AE90" s="230"/>
-      <c r="AF90" s="230"/>
+      <c r="AE90" s="80"/>
+      <c r="AF90" s="80"/>
       <c r="AG90" s="40"/>
       <c r="AH90" s="40"/>
       <c r="AI90" s="40"/>
@@ -18904,20 +18877,20 @@
       <c r="AK90" s="40">
         <v>1</v>
       </c>
-      <c r="AL90" s="231">
-        <v>1</v>
-      </c>
-      <c r="AM90" s="232"/>
-      <c r="AN90" s="232"/>
-      <c r="AO90" s="232">
-        <v>1</v>
-      </c>
-      <c r="AP90" s="233">
+      <c r="AL90" s="159">
+        <v>1</v>
+      </c>
+      <c r="AM90" s="171"/>
+      <c r="AN90" s="171"/>
+      <c r="AO90" s="171">
+        <v>1</v>
+      </c>
+      <c r="AP90" s="160">
         <f>SUM(Table13[[#This Row],[1986]:[2021]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A91" s="157" t="s">
         <v>88</v>
       </c>
@@ -19006,7 +18979,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="92" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A92" s="164" t="s">
         <v>89</v>
       </c>
@@ -19063,7 +19036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A93" s="164" t="s">
         <v>89</v>
       </c>
@@ -19120,7 +19093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A94" s="164" t="s">
         <v>170</v>
       </c>
@@ -19181,7 +19154,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A95" s="164" t="s">
         <v>170</v>
       </c>
@@ -19238,7 +19211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A96" s="167" t="s">
         <v>90</v>
       </c>
@@ -19405,41 +19378,41 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE2CF519-9585-4EA6-8BEA-E1E089CD8A6E}">
   <dimension ref="A1:AG34"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="67" customWidth="1"/>
-    <col min="2" max="3" width="10.26953125" style="72" customWidth="1"/>
-    <col min="4" max="4" width="18.26953125" customWidth="1"/>
-    <col min="5" max="5" width="25.26953125" style="67" customWidth="1"/>
-    <col min="6" max="6" width="23.453125" style="100" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" style="100" customWidth="1"/>
+    <col min="2" max="3" width="10.28515625" style="72" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" style="67" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" style="100" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="100" customWidth="1"/>
     <col min="8" max="8" width="28" style="100" customWidth="1"/>
-    <col min="9" max="9" width="14.453125" style="100" customWidth="1"/>
-    <col min="10" max="10" width="34.7265625" style="101" customWidth="1"/>
-    <col min="11" max="12" width="18.453125" style="100" customWidth="1"/>
-    <col min="13" max="13" width="34.7265625" style="100" customWidth="1"/>
-    <col min="14" max="14" width="18.453125" style="100" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.453125" style="100" customWidth="1"/>
-    <col min="16" max="16" width="5.26953125" style="100" customWidth="1"/>
-    <col min="17" max="18" width="6.453125" style="100" customWidth="1"/>
-    <col min="19" max="19" width="4.453125" style="100" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.453125" style="100" customWidth="1"/>
-    <col min="21" max="21" width="5.7265625" style="100" customWidth="1"/>
-    <col min="22" max="22" width="4.453125" style="100" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.453125" style="100" customWidth="1"/>
-    <col min="24" max="24" width="4.453125" style="100" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="3.453125" style="100" customWidth="1"/>
-    <col min="26" max="26" width="7.453125" style="100" customWidth="1"/>
-    <col min="27" max="27" width="3.453125" style="100" customWidth="1"/>
-    <col min="28" max="28" width="4.453125" style="100" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="3.7265625" style="100" customWidth="1"/>
-    <col min="30" max="30" width="6.453125" style="100" customWidth="1"/>
-    <col min="31" max="31" width="4.453125" style="100" customWidth="1"/>
-    <col min="32" max="32" width="13.7265625" style="100" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="100" customWidth="1"/>
+    <col min="10" max="10" width="34.7109375" style="101" customWidth="1"/>
+    <col min="11" max="12" width="18.42578125" style="100" customWidth="1"/>
+    <col min="13" max="13" width="34.7109375" style="100" customWidth="1"/>
+    <col min="14" max="14" width="18.42578125" style="100" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" style="100" customWidth="1"/>
+    <col min="16" max="16" width="5.28515625" style="100" customWidth="1"/>
+    <col min="17" max="18" width="6.42578125" style="100" customWidth="1"/>
+    <col min="19" max="19" width="4.42578125" style="100" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.42578125" style="100" customWidth="1"/>
+    <col min="21" max="21" width="5.7109375" style="100" customWidth="1"/>
+    <col min="22" max="22" width="4.42578125" style="100" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.42578125" style="100" customWidth="1"/>
+    <col min="24" max="24" width="4.42578125" style="100" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="3.42578125" style="100" customWidth="1"/>
+    <col min="26" max="26" width="7.42578125" style="100" customWidth="1"/>
+    <col min="27" max="27" width="3.42578125" style="100" customWidth="1"/>
+    <col min="28" max="28" width="4.42578125" style="100" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="3.7109375" style="100" customWidth="1"/>
+    <col min="30" max="30" width="6.42578125" style="100" customWidth="1"/>
+    <col min="31" max="31" width="4.42578125" style="100" customWidth="1"/>
+    <col min="32" max="32" width="13.7109375" style="100" customWidth="1"/>
     <col min="33" max="33" width="39" style="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="140" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:33" s="140" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="143"/>
       <c r="B1" s="144"/>
       <c r="C1" s="144"/>
@@ -19473,7 +19446,7 @@
       <c r="AF1" s="141"/>
       <c r="AG1" s="141"/>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="137"/>
       <c r="B2" s="139"/>
       <c r="C2" s="139"/>
@@ -19516,7 +19489,7 @@
       <c r="AF2" s="133"/>
       <c r="AG2" s="132"/>
     </row>
-    <row r="3" spans="1:33" s="130" customFormat="1" ht="78" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" s="130" customFormat="1" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A3" s="195" t="s">
         <v>359</v>
       </c>
@@ -19597,7 +19570,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="4" spans="1:33" s="124" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" s="124" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="196"/>
       <c r="B4" s="196"/>
       <c r="C4" s="198"/>
@@ -19668,7 +19641,7 @@
       </c>
       <c r="AG4" s="125"/>
     </row>
-    <row r="5" spans="1:33" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="113" t="s">
         <v>38</v>
       </c>
@@ -19737,7 +19710,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="6" spans="1:33" s="72" customFormat="1" ht="78" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" s="72" customFormat="1" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A6" s="113" t="s">
         <v>8</v>
       </c>
@@ -19800,7 +19773,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="7" spans="1:33" s="72" customFormat="1" ht="120" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" s="72" customFormat="1" ht="144" x14ac:dyDescent="0.25">
       <c r="A7" s="113" t="s">
         <v>83</v>
       </c>
@@ -19863,7 +19836,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="8" spans="1:33" s="74" customFormat="1" ht="94.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:33" s="74" customFormat="1" ht="94.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="113" t="s">
         <v>86</v>
       </c>
@@ -19935,7 +19908,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="9" spans="1:33" s="72" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:33" s="72" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="110" t="s">
         <v>58</v>
       </c>
@@ -19978,7 +19951,7 @@
       <c r="AF9" s="68"/>
       <c r="AG9" s="68"/>
     </row>
-    <row r="10" spans="1:33" s="73" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" s="73" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="122" t="s">
         <v>43</v>
       </c>
@@ -20035,7 +20008,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="11" spans="1:33" s="72" customFormat="1" ht="65" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" s="72" customFormat="1" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A11" s="110" t="s">
         <v>28</v>
       </c>
@@ -20086,7 +20059,7 @@
       <c r="AF11" s="68"/>
       <c r="AG11" s="68"/>
     </row>
-    <row r="12" spans="1:33" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="113" t="s">
         <v>53</v>
       </c>
@@ -20155,7 +20128,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="13" spans="1:33" s="74" customFormat="1" ht="55.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" s="74" customFormat="1" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="113" t="s">
         <v>85</v>
       </c>
@@ -20214,7 +20187,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="110" t="s">
         <v>48</v>
       </c>
@@ -20259,7 +20232,7 @@
       <c r="AF14" s="108"/>
       <c r="AG14" s="108"/>
     </row>
-    <row r="15" spans="1:33" s="72" customFormat="1" ht="115.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" s="72" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" s="113" t="s">
         <v>22</v>
       </c>
@@ -20320,7 +20293,7 @@
       </c>
       <c r="AG15" s="68"/>
     </row>
-    <row r="16" spans="1:33" s="74" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:33" s="74" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="114" t="s">
         <v>170</v>
       </c>
@@ -20367,7 +20340,7 @@
       <c r="AF16" s="75"/>
       <c r="AG16" s="75"/>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" s="110" t="s">
         <v>73</v>
       </c>
@@ -20408,7 +20381,7 @@
       <c r="AF17" s="108"/>
       <c r="AG17" s="108"/>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" s="110" t="s">
         <v>76</v>
       </c>
@@ -20449,7 +20422,7 @@
       <c r="AF18" s="108"/>
       <c r="AG18" s="108"/>
     </row>
-    <row r="19" spans="1:33" ht="52" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:33" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="113" t="s">
         <v>79</v>
       </c>
@@ -20512,7 +20485,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" s="110" t="s">
         <v>89</v>
       </c>
@@ -20549,7 +20522,7 @@
       <c r="AF20" s="108"/>
       <c r="AG20" s="108"/>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" s="109" t="s">
         <v>87</v>
       </c>
@@ -20592,7 +20565,7 @@
       <c r="AF21" s="108"/>
       <c r="AG21" s="108"/>
     </row>
-    <row r="22" spans="1:33" s="72" customFormat="1" ht="31.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:33" s="72" customFormat="1" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A22" s="107" t="s">
         <v>63</v>
       </c>
@@ -20663,7 +20636,7 @@
       <c r="AF22" s="68"/>
       <c r="AG22" s="68"/>
     </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" s="70" t="s">
         <v>449</v>
       </c>
@@ -20677,7 +20650,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" s="70" t="s">
         <v>452</v>
       </c>
@@ -20694,7 +20667,7 @@
       <c r="I25" s="203"/>
       <c r="J25" s="57"/>
     </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
       <c r="D26" s="104" t="s">
         <v>453</v>
       </c>
@@ -20704,7 +20677,7 @@
       <c r="I26" s="203"/>
       <c r="J26" s="57"/>
     </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="D27" s="104" t="s">
         <v>456</v>
       </c>
@@ -20714,7 +20687,7 @@
       <c r="I27" s="203"/>
       <c r="J27" s="57"/>
     </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
       <c r="D28" s="104" t="s">
         <v>456</v>
       </c>
@@ -20724,7 +20697,7 @@
       <c r="I28" s="203"/>
       <c r="J28" s="57"/>
     </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
       <c r="D29" s="104" t="s">
         <v>456</v>
       </c>
@@ -20732,12 +20705,12 @@
         <v>459</v>
       </c>
     </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
       <c r="B31" s="102" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="72">
         <f>16*3/3</f>
         <v>16</v>
@@ -20783,17 +20756,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="10.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.453125" style="29" customWidth="1"/>
-    <col min="3" max="3" width="42.26953125" style="26" customWidth="1"/>
-    <col min="4" max="4" width="22.7265625" style="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.7265625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" style="29" customWidth="1"/>
+    <col min="3" max="3" width="42.28515625" style="26" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="28" customWidth="1"/>
     <col min="6" max="16384" width="9" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
         <v>171</v>
       </c>
@@ -20802,14 +20775,14 @@
       <c r="D1" s="22"/>
       <c r="E1" s="23"/>
     </row>
-    <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="34"/>
       <c r="B2" s="24"/>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
       <c r="E2" s="23"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="25"/>
       <c r="B3" s="25" t="s">
         <v>172</v>
@@ -20822,7 +20795,7 @@
       </c>
       <c r="E3" s="23"/>
     </row>
-    <row r="4" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="91" t="s">
         <v>8</v>
       </c>
@@ -20837,7 +20810,7 @@
       </c>
       <c r="E4" s="28"/>
     </row>
-    <row r="5" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="92"/>
       <c r="B5" s="90"/>
       <c r="C5" s="90" t="s">
@@ -20848,7 +20821,7 @@
       </c>
       <c r="E5" s="28"/>
     </row>
-    <row r="6" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="91" t="s">
         <v>22</v>
       </c>
@@ -20863,7 +20836,7 @@
       </c>
       <c r="E6" s="28"/>
     </row>
-    <row r="7" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="27"/>
       <c r="C7" s="26" t="s">
         <v>183</v>
@@ -20873,7 +20846,7 @@
       </c>
       <c r="E7" s="28"/>
     </row>
-    <row r="8" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="92"/>
       <c r="B8" s="90"/>
       <c r="C8" s="90" t="s">
@@ -20884,7 +20857,7 @@
       </c>
       <c r="E8" s="28"/>
     </row>
-    <row r="9" spans="1:5" s="26" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" s="26" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="213" t="s">
         <v>28</v>
       </c>
@@ -20899,7 +20872,7 @@
       </c>
       <c r="E9" s="28"/>
     </row>
-    <row r="10" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="214"/>
       <c r="B10" s="212"/>
       <c r="C10" s="26" t="s">
@@ -20910,7 +20883,7 @@
       </c>
       <c r="E10" s="28"/>
     </row>
-    <row r="11" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="65" t="s">
         <v>34</v>
       </c>
@@ -20925,7 +20898,7 @@
       </c>
       <c r="E11" s="28"/>
     </row>
-    <row r="12" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="91" t="s">
         <v>38</v>
       </c>
@@ -20940,7 +20913,7 @@
       </c>
       <c r="E12" s="28"/>
     </row>
-    <row r="13" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="27"/>
       <c r="B13" s="209"/>
       <c r="C13" s="26" t="s">
@@ -20951,7 +20924,7 @@
       </c>
       <c r="E13" s="28"/>
     </row>
-    <row r="14" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="92"/>
       <c r="B14" s="210"/>
       <c r="C14" s="90" t="s">
@@ -20962,7 +20935,7 @@
       </c>
       <c r="E14" s="28"/>
     </row>
-    <row r="15" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="91" t="s">
         <v>43</v>
       </c>
@@ -20977,7 +20950,7 @@
       </c>
       <c r="E15" s="28"/>
     </row>
-    <row r="16" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="27"/>
       <c r="B16" s="87"/>
       <c r="C16" s="31" t="s">
@@ -20988,7 +20961,7 @@
       </c>
       <c r="E16" s="32"/>
     </row>
-    <row r="17" spans="1:5" s="26" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" s="26" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="213" t="s">
         <v>48</v>
       </c>
@@ -21003,7 +20976,7 @@
       </c>
       <c r="E17" s="32"/>
     </row>
-    <row r="18" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="214"/>
       <c r="B18" s="212"/>
       <c r="C18" s="30" t="s">
@@ -21014,7 +20987,7 @@
       </c>
       <c r="E18" s="28"/>
     </row>
-    <row r="19" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="65" t="s">
         <v>53</v>
       </c>
@@ -21029,7 +21002,7 @@
       </c>
       <c r="E19" s="28"/>
     </row>
-    <row r="20" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="91" t="s">
         <v>58</v>
       </c>
@@ -21044,7 +21017,7 @@
       </c>
       <c r="E20" s="28"/>
     </row>
-    <row r="21" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="27"/>
       <c r="C21" s="26" t="s">
         <v>216</v>
@@ -21054,7 +21027,7 @@
       </c>
       <c r="E21" s="28"/>
     </row>
-    <row r="22" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="92"/>
       <c r="C22" s="26" t="s">
         <v>218</v>
@@ -21064,7 +21037,7 @@
       </c>
       <c r="E22" s="28"/>
     </row>
-    <row r="23" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="65" t="s">
         <v>63</v>
       </c>
@@ -21079,7 +21052,7 @@
       </c>
       <c r="E23" s="28"/>
     </row>
-    <row r="24" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
         <v>65</v>
       </c>
@@ -21094,7 +21067,7 @@
       </c>
       <c r="E24" s="28"/>
     </row>
-    <row r="25" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="65" t="s">
         <v>68</v>
       </c>
@@ -21109,7 +21082,7 @@
       </c>
       <c r="E25" s="28"/>
     </row>
-    <row r="26" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="91" t="s">
         <v>73</v>
       </c>
@@ -21124,7 +21097,7 @@
       </c>
       <c r="E26" s="28"/>
     </row>
-    <row r="27" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="92"/>
       <c r="B27" s="90"/>
       <c r="C27" s="88" t="s">
@@ -21135,7 +21108,7 @@
       </c>
       <c r="E27" s="32"/>
     </row>
-    <row r="28" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="91" t="s">
         <v>76</v>
       </c>
@@ -21150,7 +21123,7 @@
       </c>
       <c r="E28" s="32"/>
     </row>
-    <row r="29" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="92"/>
       <c r="B29" s="90"/>
       <c r="C29" s="90" t="s">
@@ -21161,7 +21134,7 @@
       </c>
       <c r="E29" s="28"/>
     </row>
-    <row r="30" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="91" t="s">
         <v>79</v>
       </c>
@@ -21176,7 +21149,7 @@
       </c>
       <c r="E30" s="28"/>
     </row>
-    <row r="31" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="27"/>
       <c r="B31" s="209"/>
       <c r="C31" s="26" t="s">
@@ -21187,7 +21160,7 @@
       </c>
       <c r="E31" s="28"/>
     </row>
-    <row r="32" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="27"/>
       <c r="B32" s="209"/>
       <c r="C32" s="26" t="s">
@@ -21198,7 +21171,7 @@
       </c>
       <c r="E32" s="28"/>
     </row>
-    <row r="33" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="92"/>
       <c r="B33" s="210"/>
       <c r="C33" s="90" t="s">
@@ -21209,7 +21182,7 @@
       </c>
       <c r="E33" s="28"/>
     </row>
-    <row r="34" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="65" t="s">
         <v>83</v>
       </c>
@@ -21224,7 +21197,7 @@
       </c>
       <c r="E34" s="28"/>
     </row>
-    <row r="35" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="65" t="s">
         <v>85</v>
       </c>
@@ -21239,7 +21212,7 @@
       </c>
       <c r="E35" s="28"/>
     </row>
-    <row r="36" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="27" t="s">
         <v>86</v>
       </c>
@@ -21254,7 +21227,7 @@
       </c>
       <c r="E36" s="28"/>
     </row>
-    <row r="37" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="206" t="s">
         <v>87</v>
       </c>
@@ -21269,7 +21242,7 @@
       </c>
       <c r="E37" s="28"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="207"/>
       <c r="B38" s="50" t="s">
         <v>249</v>
@@ -21281,7 +21254,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="27"/>
       <c r="B39" s="27"/>
       <c r="E39" s="28"/>
@@ -21304,24 +21277,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:L93"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.25" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="2.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.26953125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.26953125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="8.26953125" style="3" customWidth="1"/>
-    <col min="12" max="12" width="11.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="2.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="4.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="222" t="s">
         <v>251</v>
       </c>
@@ -21336,7 +21309,7 @@
       <c r="K1" s="222"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="2:12" ht="24" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" ht="36" x14ac:dyDescent="0.25">
       <c r="B2" s="59" t="s">
         <v>2</v>
       </c>
@@ -21358,7 +21331,7 @@
       <c r="K2" s="44"/>
       <c r="L2" s="44"/>
     </row>
-    <row r="3" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="218" t="s">
         <v>8</v>
       </c>
@@ -21375,7 +21348,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="215"/>
       <c r="C4" s="97" t="s">
         <v>14</v>
@@ -21390,7 +21363,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="215"/>
       <c r="C5" s="97" t="s">
         <v>257</v>
@@ -21405,7 +21378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="219"/>
       <c r="C6" s="97" t="s">
         <v>259</v>
@@ -21420,7 +21393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="98" t="s">
         <v>15</v>
       </c>
@@ -21437,7 +21410,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="215" t="s">
         <v>20</v>
       </c>
@@ -21454,7 +21427,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="215"/>
       <c r="C9" s="93" t="s">
         <v>67</v>
@@ -21469,7 +21442,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="223" t="s">
         <v>22</v>
       </c>
@@ -21486,7 +21459,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="224"/>
       <c r="C11" s="98" t="s">
         <v>26</v>
@@ -21501,7 +21474,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="224"/>
       <c r="C12" s="98" t="s">
         <v>27</v>
@@ -21516,7 +21489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="225"/>
       <c r="C13" s="98" t="s">
         <v>267</v>
@@ -21531,7 +21504,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="218" t="s">
         <v>28</v>
       </c>
@@ -21548,7 +21521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="215"/>
       <c r="C15" s="60" t="s">
         <v>29</v>
@@ -21563,7 +21536,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="215"/>
       <c r="C16" s="60" t="s">
         <v>271</v>
@@ -21578,7 +21551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="219"/>
       <c r="C17" s="61" t="s">
         <v>267</v>
@@ -21593,7 +21566,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="216" t="s">
         <v>32</v>
       </c>
@@ -21610,7 +21583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="217"/>
       <c r="C19" s="2" t="s">
         <v>67</v>
@@ -21625,7 +21598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="215" t="s">
         <v>34</v>
       </c>
@@ -21642,7 +21615,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="215"/>
       <c r="C21" s="60" t="s">
         <v>27</v>
@@ -21657,7 +21630,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="215"/>
       <c r="C22" s="60" t="s">
         <v>277</v>
@@ -21672,7 +21645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="215"/>
       <c r="C23" s="61" t="s">
         <v>279</v>
@@ -21687,7 +21660,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="223" t="s">
         <v>38</v>
       </c>
@@ -21704,7 +21677,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="224"/>
       <c r="C25" s="63" t="s">
         <v>39</v>
@@ -21719,7 +21692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="224"/>
       <c r="C26" s="63" t="s">
         <v>40</v>
@@ -21734,7 +21707,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="224"/>
       <c r="C27" s="63" t="s">
         <v>41</v>
@@ -21749,7 +21722,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="224"/>
       <c r="C28" s="63" t="s">
         <v>285</v>
@@ -21764,7 +21737,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="224"/>
       <c r="C29" s="63" t="s">
         <v>267</v>
@@ -21779,7 +21752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="225"/>
       <c r="C30" s="63" t="s">
         <v>279</v>
@@ -21794,7 +21767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="215" t="s">
         <v>43</v>
       </c>
@@ -21811,7 +21784,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="215"/>
       <c r="C32" s="97" t="s">
         <v>45</v>
@@ -21826,7 +21799,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="215"/>
       <c r="C33" s="97" t="s">
         <v>40</v>
@@ -21841,7 +21814,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="215"/>
       <c r="C34" s="93" t="s">
         <v>259</v>
@@ -21856,7 +21829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="220" t="s">
         <v>48</v>
       </c>
@@ -21873,7 +21846,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="220"/>
       <c r="C36" s="98" t="s">
         <v>49</v>
@@ -21888,7 +21861,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="220"/>
       <c r="C37" s="98" t="s">
         <v>293</v>
@@ -21903,7 +21876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="220"/>
       <c r="C38" s="98" t="s">
         <v>267</v>
@@ -21918,7 +21891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="219" t="s">
         <v>53</v>
       </c>
@@ -21935,7 +21908,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="218"/>
       <c r="C40" s="93" t="s">
         <v>57</v>
@@ -21950,7 +21923,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="223" t="s">
         <v>58</v>
       </c>
@@ -21967,7 +21940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="224"/>
       <c r="C42" s="98" t="s">
         <v>60</v>
@@ -21982,7 +21955,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="224"/>
       <c r="C43" s="98" t="s">
         <v>62</v>
@@ -21997,7 +21970,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="224"/>
       <c r="C44" s="98" t="s">
         <v>300</v>
@@ -22012,7 +21985,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="225"/>
       <c r="C45" s="98" t="s">
         <v>267</v>
@@ -22027,7 +22000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="218" t="s">
         <v>170</v>
       </c>
@@ -22044,7 +22017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="215"/>
       <c r="C47" s="64" t="s">
         <v>259</v>
@@ -22059,7 +22032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="215"/>
       <c r="C48" s="64" t="s">
         <v>267</v>
@@ -22074,7 +22047,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="219"/>
       <c r="C49" s="64" t="s">
         <v>16</v>
@@ -22089,7 +22062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="218" t="s">
         <v>63</v>
       </c>
@@ -22106,7 +22079,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="215"/>
       <c r="C51" s="64" t="s">
         <v>59</v>
@@ -22121,7 +22094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="219"/>
       <c r="C52" s="64" t="s">
         <v>267</v>
@@ -22136,7 +22109,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="224" t="s">
         <v>154</v>
       </c>
@@ -22153,7 +22126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="224"/>
       <c r="C54" s="98" t="s">
         <v>155</v>
@@ -22168,7 +22141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="224"/>
       <c r="C55" s="95" t="s">
         <v>267</v>
@@ -22183,7 +22156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="218" t="s">
         <v>65</v>
       </c>
@@ -22200,7 +22173,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="215"/>
       <c r="C57" s="97" t="s">
         <v>67</v>
@@ -22215,7 +22188,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="58" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="219"/>
       <c r="C58" s="97" t="s">
         <v>259</v>
@@ -22230,7 +22203,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="223" t="s">
         <v>68</v>
       </c>
@@ -22247,7 +22220,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="60" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="224"/>
       <c r="C60" s="98" t="s">
         <v>27</v>
@@ -22262,7 +22235,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="224"/>
       <c r="C61" s="98" t="s">
         <v>316</v>
@@ -22277,7 +22250,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="62" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="224"/>
       <c r="C62" s="98" t="s">
         <v>318</v>
@@ -22292,7 +22265,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="224"/>
       <c r="C63" s="98" t="s">
         <v>320</v>
@@ -22307,7 +22280,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="224"/>
       <c r="C64" s="98" t="s">
         <v>322</v>
@@ -22322,7 +22295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="225"/>
       <c r="C65" s="98" t="s">
         <v>324</v>
@@ -22337,7 +22310,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="218" t="s">
         <v>73</v>
       </c>
@@ -22354,7 +22327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="215"/>
       <c r="C67" s="97" t="s">
         <v>74</v>
@@ -22369,7 +22342,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="215"/>
       <c r="C68" s="97" t="s">
         <v>327</v>
@@ -22384,7 +22357,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="219"/>
       <c r="C69" s="93" t="s">
         <v>267</v>
@@ -22399,7 +22372,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="223" t="s">
         <v>76</v>
       </c>
@@ -22416,7 +22389,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="224"/>
       <c r="C71" s="98" t="s">
         <v>44</v>
@@ -22431,7 +22404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="224"/>
       <c r="C72" s="98" t="s">
         <v>332</v>
@@ -22446,7 +22419,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="224"/>
       <c r="C73" s="98" t="s">
         <v>334</v>
@@ -22461,7 +22434,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="225"/>
       <c r="C74" s="98" t="s">
         <v>82</v>
@@ -22476,7 +22449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="219" t="s">
         <v>79</v>
       </c>
@@ -22493,7 +22466,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="221"/>
       <c r="C76" s="97" t="s">
         <v>26</v>
@@ -22508,7 +22481,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="218"/>
       <c r="C77" s="93" t="s">
         <v>9</v>
@@ -22523,7 +22496,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="218"/>
       <c r="C78" s="93" t="s">
         <v>82</v>
@@ -22538,7 +22511,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="79" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="223" t="s">
         <v>83</v>
       </c>
@@ -22555,7 +22528,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="80" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="224"/>
       <c r="C80" s="98" t="s">
         <v>84</v>
@@ -22570,7 +22543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="224"/>
       <c r="C81" s="98" t="s">
         <v>342</v>
@@ -22585,7 +22558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="225"/>
       <c r="C82" s="98" t="s">
         <v>267</v>
@@ -22600,7 +22573,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="83" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="215" t="s">
         <v>85</v>
       </c>
@@ -22617,7 +22590,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="215"/>
       <c r="C84" s="93" t="s">
         <v>345</v>
@@ -22632,7 +22605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="216" t="s">
         <v>89</v>
       </c>
@@ -22649,7 +22622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="217"/>
       <c r="C86" s="2" t="s">
         <v>67</v>
@@ -22664,7 +22637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="215" t="s">
         <v>88</v>
       </c>
@@ -22681,7 +22654,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="215"/>
       <c r="C88" s="97" t="s">
         <v>349</v>
@@ -22696,7 +22669,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="215"/>
       <c r="C89" s="97" t="s">
         <v>259</v>
@@ -22711,7 +22684,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="215"/>
       <c r="C90" s="93" t="s">
         <v>67</v>
@@ -22726,7 +22699,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="98" t="s">
         <v>86</v>
       </c>
@@ -22743,7 +22716,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="92" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="221" t="s">
         <v>87</v>
       </c>
@@ -22760,7 +22733,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="93" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="221"/>
       <c r="C93" s="94" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Add escolar and no escolar age groups to education vars
Introduced 'edad_escolar' and 'edad_no_escolar' variables in var_EDU.R for more granular age groupings. Updated functions.R to handle these new variables in groupings. Modified idef.csv to use the new age group variables in relevant indicators.
</commit_message>
<xml_diff>
--- a/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
+++ b/Inputs/Planeación - Armonización de Encuestas de Hogares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/matiasi_iadb_org/Documents/Documents/Github/calculo_indicators_R/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3050" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A67BFB29-5B16-4AC6-99FB-B5C3FD593252}"/>
+  <xr:revisionPtr revIDLastSave="3052" documentId="13_ncr:1_{8AF7F83F-6557-4E4A-89D0-13E0BF5AF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D5A1775-7191-40D9-9C69-27E4A30D34F0}"/>
   <bookViews>
-    <workbookView xWindow="34290" yWindow="3550" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24090" yWindow="4110" windowWidth="19125" windowHeight="10035" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Encuestas Armonizadas" sheetId="2" state="hidden" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId8"/>
+    <pivotCache cacheId="23" r:id="rId8"/>
   </pivotCaches>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
@@ -2607,25 +2607,34 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2658,15 +2667,6 @@
     <xf numFmtId="0" fontId="14" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2694,28 +2694,16 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2725,6 +2713,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5094,7 +5094,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{963ADC1E-6961-40E2-8B9B-709AC1AD34EB}" name="PivotTable4" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{963ADC1E-6961-40E2-8B9B-709AC1AD34EB}" name="PivotTable4" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:U32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -5350,6 +5350,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}" name="Table13" displayName="Table13" ref="A1:AP96" totalsRowShown="0" headerRowDxfId="45" headerRowBorderDxfId="44" tableBorderDxfId="43" totalsRowBorderDxfId="42" headerRowCellStyle="Normal 2">
+  <autoFilter ref="A1:AP96" xr:uid="{227E27DD-A399-428B-89D5-9E5CE9864EEC}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="GTM"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="42">
     <tableColumn id="1" xr3:uid="{6B064E87-3A0D-4584-8192-35267E66F273}" name="País" dataDxfId="41" dataCellStyle="Normal 2"/>
     <tableColumn id="2" xr3:uid="{56390F1F-7512-4FEB-8AF3-898CDB1A9830}" name="Encuesta" dataDxfId="40"/>
@@ -5711,44 +5718,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:75" ht="15" x14ac:dyDescent="0.2">
-      <c r="B1" s="191" t="s">
+      <c r="B1" s="186" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="191"/>
-      <c r="D1" s="191"/>
-      <c r="E1" s="191"/>
-      <c r="F1" s="191"/>
-      <c r="G1" s="191"/>
-      <c r="H1" s="191"/>
-      <c r="I1" s="191"/>
-      <c r="J1" s="191"/>
-      <c r="K1" s="191"/>
-      <c r="L1" s="191"/>
-      <c r="M1" s="191"/>
-      <c r="N1" s="191"/>
-      <c r="O1" s="191"/>
-      <c r="P1" s="191"/>
-      <c r="Q1" s="191"/>
-      <c r="R1" s="191"/>
-      <c r="S1" s="191"/>
-      <c r="T1" s="191"/>
-      <c r="U1" s="191"/>
-      <c r="V1" s="191"/>
-      <c r="W1" s="191"/>
-      <c r="X1" s="191"/>
-      <c r="Y1" s="191"/>
-      <c r="Z1" s="191"/>
-      <c r="AA1" s="191"/>
-      <c r="AB1" s="191"/>
-      <c r="AC1" s="191"/>
-      <c r="AD1" s="191"/>
-      <c r="AE1" s="191"/>
-      <c r="AF1" s="191"/>
-      <c r="AG1" s="191"/>
-      <c r="AH1" s="191"/>
-      <c r="AI1" s="191"/>
-      <c r="AJ1" s="191"/>
-      <c r="AK1" s="191"/>
+      <c r="C1" s="186"/>
+      <c r="D1" s="186"/>
+      <c r="E1" s="186"/>
+      <c r="F1" s="186"/>
+      <c r="G1" s="186"/>
+      <c r="H1" s="186"/>
+      <c r="I1" s="186"/>
+      <c r="J1" s="186"/>
+      <c r="K1" s="186"/>
+      <c r="L1" s="186"/>
+      <c r="M1" s="186"/>
+      <c r="N1" s="186"/>
+      <c r="O1" s="186"/>
+      <c r="P1" s="186"/>
+      <c r="Q1" s="186"/>
+      <c r="R1" s="186"/>
+      <c r="S1" s="186"/>
+      <c r="T1" s="186"/>
+      <c r="U1" s="186"/>
+      <c r="V1" s="186"/>
+      <c r="W1" s="186"/>
+      <c r="X1" s="186"/>
+      <c r="Y1" s="186"/>
+      <c r="Z1" s="186"/>
+      <c r="AA1" s="186"/>
+      <c r="AB1" s="186"/>
+      <c r="AC1" s="186"/>
+      <c r="AD1" s="186"/>
+      <c r="AE1" s="186"/>
+      <c r="AF1" s="186"/>
+      <c r="AG1" s="186"/>
+      <c r="AH1" s="186"/>
+      <c r="AI1" s="186"/>
+      <c r="AJ1" s="186"/>
+      <c r="AK1" s="186"/>
       <c r="AL1" s="51"/>
       <c r="AM1" s="83"/>
       <c r="AN1" s="51"/>
@@ -5917,7 +5924,7 @@
       <c r="A3" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="186" t="s">
+      <c r="B3" s="188" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="57" t="s">
@@ -6011,7 +6018,7 @@
     </row>
     <row r="4" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="145"/>
-      <c r="B4" s="187"/>
+      <c r="B4" s="189"/>
       <c r="C4" s="57" t="s">
         <v>14</v>
       </c>
@@ -6247,7 +6254,7 @@
       <c r="A7" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="189" t="s">
+      <c r="B7" s="190" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="57" t="s">
@@ -6343,7 +6350,7 @@
     </row>
     <row r="8" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="145"/>
-      <c r="B8" s="189"/>
+      <c r="B8" s="190"/>
       <c r="C8" s="57" t="s">
         <v>26</v>
       </c>
@@ -6401,7 +6408,7 @@
     </row>
     <row r="9" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="145"/>
-      <c r="B9" s="189"/>
+      <c r="B9" s="190"/>
       <c r="C9" s="57" t="s">
         <v>27</v>
       </c>
@@ -6451,7 +6458,7 @@
     </row>
     <row r="10" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="145"/>
-      <c r="B10" s="189" t="s">
+      <c r="B10" s="190" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="39" t="s">
@@ -6545,7 +6552,7 @@
       <c r="A11" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="189"/>
+      <c r="B11" s="190"/>
       <c r="C11" s="39" t="s">
         <v>30</v>
       </c>
@@ -6781,7 +6788,7 @@
     </row>
     <row r="14" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="145"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="188" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="39" t="s">
@@ -6839,7 +6846,7 @@
     </row>
     <row r="15" spans="1:75" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="145"/>
-      <c r="B15" s="188"/>
+      <c r="B15" s="191"/>
       <c r="C15" s="39" t="s">
         <v>39</v>
       </c>
@@ -6887,7 +6894,7 @@
     </row>
     <row r="16" spans="1:75" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="145"/>
-      <c r="B16" s="188"/>
+      <c r="B16" s="191"/>
       <c r="C16" s="39" t="s">
         <v>40</v>
       </c>
@@ -6959,7 +6966,7 @@
       <c r="A17" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B17" s="187"/>
+      <c r="B17" s="189"/>
       <c r="C17" s="39" t="s">
         <v>41</v>
       </c>
@@ -7045,7 +7052,7 @@
     </row>
     <row r="18" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="145"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="188" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="41" t="s">
@@ -7135,7 +7142,7 @@
       <c r="A19" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B19" s="187"/>
+      <c r="B19" s="189"/>
       <c r="C19" s="57" t="s">
         <v>45</v>
       </c>
@@ -7213,7 +7220,7 @@
     </row>
     <row r="20" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="145"/>
-      <c r="B20" s="186" t="s">
+      <c r="B20" s="188" t="s">
         <v>48</v>
       </c>
       <c r="C20" s="57" t="s">
@@ -7303,7 +7310,7 @@
       <c r="A21" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B21" s="187"/>
+      <c r="B21" s="189"/>
       <c r="C21" s="57" t="s">
         <v>50</v>
       </c>
@@ -7367,7 +7374,7 @@
       <c r="A22" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B22" s="189" t="s">
+      <c r="B22" s="190" t="s">
         <v>53</v>
       </c>
       <c r="C22" s="57" t="s">
@@ -7487,7 +7494,7 @@
     </row>
     <row r="23" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="145"/>
-      <c r="B23" s="189"/>
+      <c r="B23" s="190"/>
       <c r="C23" s="57" t="s">
         <v>57</v>
       </c>
@@ -7541,7 +7548,7 @@
     </row>
     <row r="24" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="145"/>
-      <c r="B24" s="189" t="s">
+      <c r="B24" s="190" t="s">
         <v>58</v>
       </c>
       <c r="C24" s="57" t="s">
@@ -7597,7 +7604,7 @@
       <c r="A25" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="189"/>
+      <c r="B25" s="190"/>
       <c r="C25" s="57" t="s">
         <v>60</v>
       </c>
@@ -7679,7 +7686,7 @@
     </row>
     <row r="26" spans="1:42" ht="12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="145"/>
-      <c r="B26" s="189"/>
+      <c r="B26" s="190"/>
       <c r="C26" s="57" t="s">
         <v>62</v>
       </c>
@@ -7849,7 +7856,7 @@
       <c r="A28" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B28" s="186" t="s">
+      <c r="B28" s="188" t="s">
         <v>65</v>
       </c>
       <c r="C28" s="57" t="s">
@@ -7953,7 +7960,7 @@
     </row>
     <row r="29" spans="1:42" ht="10.9" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="145"/>
-      <c r="B29" s="187"/>
+      <c r="B29" s="189"/>
       <c r="C29" s="57" t="s">
         <v>67</v>
       </c>
@@ -8107,7 +8114,7 @@
     </row>
     <row r="31" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="145"/>
-      <c r="B31" s="186" t="s">
+      <c r="B31" s="188" t="s">
         <v>73</v>
       </c>
       <c r="C31" s="57" t="s">
@@ -8163,7 +8170,7 @@
       <c r="A32" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B32" s="187"/>
+      <c r="B32" s="189"/>
       <c r="C32" s="57" t="s">
         <v>74</v>
       </c>
@@ -8229,7 +8236,7 @@
     </row>
     <row r="33" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="145"/>
-      <c r="B33" s="186" t="s">
+      <c r="B33" s="188" t="s">
         <v>76</v>
       </c>
       <c r="C33" s="57" t="s">
@@ -8313,7 +8320,7 @@
       <c r="A34" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B34" s="187"/>
+      <c r="B34" s="189"/>
       <c r="C34" s="57" t="s">
         <v>44</v>
       </c>
@@ -8387,7 +8394,7 @@
     </row>
     <row r="35" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="145"/>
-      <c r="B35" s="186" t="s">
+      <c r="B35" s="188" t="s">
         <v>79</v>
       </c>
       <c r="C35" s="57" t="s">
@@ -8451,7 +8458,7 @@
     </row>
     <row r="36" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="145"/>
-      <c r="B36" s="188"/>
+      <c r="B36" s="191"/>
       <c r="C36" s="57" t="s">
         <v>26</v>
       </c>
@@ -8465,15 +8472,15 @@
       <c r="K36" s="80"/>
       <c r="L36" s="80"/>
       <c r="M36" s="80"/>
-      <c r="N36" s="192">
-        <v>1</v>
-      </c>
-      <c r="O36" s="192"/>
+      <c r="N36" s="187">
+        <v>1</v>
+      </c>
+      <c r="O36" s="187"/>
       <c r="P36" s="80"/>
-      <c r="Q36" s="192">
-        <v>1</v>
-      </c>
-      <c r="R36" s="192"/>
+      <c r="Q36" s="187">
+        <v>1</v>
+      </c>
+      <c r="R36" s="187"/>
       <c r="S36" s="80"/>
       <c r="T36" s="80"/>
       <c r="U36" s="80"/>
@@ -8503,7 +8510,7 @@
     </row>
     <row r="37" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="145"/>
-      <c r="B37" s="188"/>
+      <c r="B37" s="191"/>
       <c r="C37" s="57" t="s">
         <v>82</v>
       </c>
@@ -8587,7 +8594,7 @@
       <c r="A38" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B38" s="187"/>
+      <c r="B38" s="189"/>
       <c r="C38" s="57" t="s">
         <v>9</v>
       </c>
@@ -8651,7 +8658,7 @@
       <c r="A39" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B39" s="186" t="s">
+      <c r="B39" s="188" t="s">
         <v>83</v>
       </c>
       <c r="C39" s="57" t="s">
@@ -8757,7 +8764,7 @@
     </row>
     <row r="40" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="145"/>
-      <c r="B40" s="187"/>
+      <c r="B40" s="189"/>
       <c r="C40" s="57" t="s">
         <v>84</v>
       </c>
@@ -9047,7 +9054,7 @@
     </row>
     <row r="43" spans="1:42" ht="11.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="145"/>
-      <c r="B43" s="186" t="s">
+      <c r="B43" s="188" t="s">
         <v>87</v>
       </c>
       <c r="C43" s="57" t="s">
@@ -9149,7 +9156,7 @@
       <c r="A44" s="145" t="b">
         <v>1</v>
       </c>
-      <c r="B44" s="187"/>
+      <c r="B44" s="189"/>
       <c r="C44" s="41" t="s">
         <v>59</v>
       </c>
@@ -9661,43 +9668,43 @@
       </c>
     </row>
     <row r="58" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C58" s="190" t="s">
+      <c r="C58" s="192" t="s">
         <v>97</v>
       </c>
-      <c r="D58" s="190"/>
-      <c r="E58" s="190"/>
-      <c r="F58" s="190"/>
-      <c r="G58" s="190"/>
-      <c r="H58" s="190"/>
-      <c r="I58" s="190"/>
-      <c r="J58" s="190"/>
-      <c r="K58" s="190"/>
-      <c r="L58" s="190"/>
-      <c r="M58" s="190"/>
-      <c r="N58" s="190"/>
-      <c r="O58" s="190"/>
-      <c r="P58" s="190"/>
-      <c r="Q58" s="190"/>
-      <c r="R58" s="190"/>
-      <c r="S58" s="190"/>
-      <c r="T58" s="190"/>
-      <c r="U58" s="190"/>
-      <c r="V58" s="190"/>
-      <c r="W58" s="190"/>
-      <c r="X58" s="190"/>
-      <c r="Y58" s="190"/>
-      <c r="Z58" s="190"/>
-      <c r="AA58" s="190"/>
-      <c r="AB58" s="190"/>
-      <c r="AC58" s="190"/>
-      <c r="AD58" s="190"/>
-      <c r="AE58" s="190"/>
-      <c r="AF58" s="190"/>
-      <c r="AG58" s="190"/>
-      <c r="AH58" s="190"/>
-      <c r="AI58" s="190"/>
-      <c r="AJ58" s="190"/>
-      <c r="AK58" s="190"/>
+      <c r="D58" s="192"/>
+      <c r="E58" s="192"/>
+      <c r="F58" s="192"/>
+      <c r="G58" s="192"/>
+      <c r="H58" s="192"/>
+      <c r="I58" s="192"/>
+      <c r="J58" s="192"/>
+      <c r="K58" s="192"/>
+      <c r="L58" s="192"/>
+      <c r="M58" s="192"/>
+      <c r="N58" s="192"/>
+      <c r="O58" s="192"/>
+      <c r="P58" s="192"/>
+      <c r="Q58" s="192"/>
+      <c r="R58" s="192"/>
+      <c r="S58" s="192"/>
+      <c r="T58" s="192"/>
+      <c r="U58" s="192"/>
+      <c r="V58" s="192"/>
+      <c r="W58" s="192"/>
+      <c r="X58" s="192"/>
+      <c r="Y58" s="192"/>
+      <c r="Z58" s="192"/>
+      <c r="AA58" s="192"/>
+      <c r="AB58" s="192"/>
+      <c r="AC58" s="192"/>
+      <c r="AD58" s="192"/>
+      <c r="AE58" s="192"/>
+      <c r="AF58" s="192"/>
+      <c r="AG58" s="192"/>
+      <c r="AH58" s="192"/>
+      <c r="AI58" s="192"/>
+      <c r="AJ58" s="192"/>
+      <c r="AK58" s="192"/>
     </row>
     <row r="59" spans="3:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C59" s="147" t="s">
@@ -9818,6 +9825,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C58:AK58"/>
     <mergeCell ref="B1:AK1"/>
     <mergeCell ref="Q36:R36"/>
     <mergeCell ref="B39:B40"/>
@@ -9834,8 +9843,6 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C58:AK58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" r:id="rId1"/>
@@ -12927,7 +12934,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="157" t="s">
         <v>8</v>
       </c>
@@ -13002,7 +13009,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="157" t="s">
         <v>8</v>
       </c>
@@ -13099,7 +13106,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="157" t="s">
         <v>8</v>
       </c>
@@ -13156,7 +13163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="157" t="s">
         <v>15</v>
       </c>
@@ -13249,7 +13256,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="157" t="s">
         <v>20</v>
       </c>
@@ -13320,7 +13327,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="157" t="s">
         <v>20</v>
       </c>
@@ -13385,7 +13392,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="157" t="s">
         <v>20</v>
       </c>
@@ -13442,7 +13449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="157" t="s">
         <v>22</v>
       </c>
@@ -13503,7 +13510,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="157" t="s">
         <v>22</v>
       </c>
@@ -13558,7 +13565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="157" t="s">
         <v>22</v>
       </c>
@@ -13613,7 +13620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="157" t="s">
         <v>22</v>
       </c>
@@ -13668,7 +13675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="157" t="s">
         <v>22</v>
       </c>
@@ -13723,7 +13730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="157" t="s">
         <v>22</v>
       </c>
@@ -13778,7 +13785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="157" t="s">
         <v>22</v>
       </c>
@@ -13855,7 +13862,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="157" t="s">
         <v>22</v>
       </c>
@@ -13928,7 +13935,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="157" t="s">
         <v>28</v>
       </c>
@@ -14027,7 +14034,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="157" t="s">
         <v>28</v>
       </c>
@@ -14100,7 +14107,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="157" t="s">
         <v>32</v>
       </c>
@@ -14181,7 +14188,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="157" t="s">
         <v>32</v>
       </c>
@@ -14238,7 +14245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="157" t="s">
         <v>32</v>
       </c>
@@ -14295,7 +14302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="157" t="s">
         <v>34</v>
       </c>
@@ -14366,7 +14373,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="157" t="s">
         <v>34</v>
       </c>
@@ -14431,7 +14438,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="157" t="s">
         <v>38</v>
       </c>
@@ -14508,7 +14515,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="157" t="s">
         <v>38</v>
       </c>
@@ -14573,7 +14580,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="157" t="s">
         <v>38</v>
       </c>
@@ -14664,7 +14671,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="157" t="s">
         <v>38</v>
       </c>
@@ -14721,7 +14728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="157" t="s">
         <v>43</v>
       </c>
@@ -14816,7 +14823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="157" t="s">
         <v>43</v>
       </c>
@@ -14901,7 +14908,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="157" t="s">
         <v>48</v>
       </c>
@@ -14958,7 +14965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="157" t="s">
         <v>48</v>
       </c>
@@ -15015,7 +15022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="157" t="s">
         <v>48</v>
       </c>
@@ -15072,7 +15079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="157" t="s">
         <v>48</v>
       </c>
@@ -15161,7 +15168,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="157" t="s">
         <v>48</v>
       </c>
@@ -15232,7 +15239,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="157" t="s">
         <v>53</v>
       </c>
@@ -15309,7 +15316,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="157" t="s">
         <v>53</v>
       </c>
@@ -15976,7 +15983,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="157" t="s">
         <v>63</v>
       </c>
@@ -16055,7 +16062,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="157" t="s">
         <v>63</v>
       </c>
@@ -16112,7 +16119,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="157" t="s">
         <v>63</v>
       </c>
@@ -16173,7 +16180,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="157" t="s">
         <v>63</v>
       </c>
@@ -16238,7 +16245,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="157" t="s">
         <v>63</v>
       </c>
@@ -16309,7 +16316,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="157" t="s">
         <v>154</v>
       </c>
@@ -16364,7 +16371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="157" t="s">
         <v>65</v>
       </c>
@@ -16423,7 +16430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="157" t="s">
         <v>65</v>
       </c>
@@ -16520,7 +16527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="157" t="s">
         <v>65</v>
       </c>
@@ -16583,7 +16590,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="157" t="s">
         <v>68</v>
       </c>
@@ -16648,7 +16655,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="157" t="s">
         <v>68</v>
       </c>
@@ -16703,7 +16710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="157" t="s">
         <v>68</v>
       </c>
@@ -16758,7 +16765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="157" t="s">
         <v>68</v>
       </c>
@@ -16831,7 +16838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="157" t="s">
         <v>73</v>
       </c>
@@ -16894,7 +16901,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="157" t="s">
         <v>73</v>
       </c>
@@ -16953,7 +16960,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="157" t="s">
         <v>73</v>
       </c>
@@ -17014,7 +17021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="157" t="s">
         <v>73</v>
       </c>
@@ -17071,7 +17078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="157" t="s">
         <v>76</v>
       </c>
@@ -17160,7 +17167,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="65" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="157" t="s">
         <v>76</v>
       </c>
@@ -17235,7 +17242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="157" t="s">
         <v>76</v>
       </c>
@@ -17292,7 +17299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="157" t="s">
         <v>76</v>
       </c>
@@ -17349,7 +17356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="157" t="s">
         <v>79</v>
       </c>
@@ -17404,7 +17411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="157" t="s">
         <v>79</v>
       </c>
@@ -17459,7 +17466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="157" t="s">
         <v>79</v>
       </c>
@@ -17514,7 +17521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="157" t="s">
         <v>79</v>
       </c>
@@ -17569,7 +17576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="157" t="s">
         <v>79</v>
       </c>
@@ -17624,7 +17631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="157" t="s">
         <v>79</v>
       </c>
@@ -17679,7 +17686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="157" t="s">
         <v>79</v>
       </c>
@@ -17734,7 +17741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="157" t="s">
         <v>79</v>
       </c>
@@ -17789,7 +17796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="157" t="s">
         <v>79</v>
       </c>
@@ -17844,7 +17851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="157" t="s">
         <v>79</v>
       </c>
@@ -17901,7 +17908,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="157" t="s">
         <v>79</v>
       </c>
@@ -17958,7 +17965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="157" t="s">
         <v>79</v>
       </c>
@@ -18013,7 +18020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="157" t="s">
         <v>79</v>
       </c>
@@ -18090,7 +18097,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="157" t="s">
         <v>79</v>
       </c>
@@ -18155,7 +18162,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="157" t="s">
         <v>83</v>
       </c>
@@ -18212,7 +18219,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="157" t="s">
         <v>83</v>
       </c>
@@ -18277,7 +18284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="157" t="s">
         <v>83</v>
       </c>
@@ -18374,7 +18381,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="85" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="157" t="s">
         <v>85</v>
       </c>
@@ -18487,7 +18494,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="86" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="157" t="s">
         <v>86</v>
       </c>
@@ -18552,7 +18559,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="157" t="s">
         <v>86</v>
       </c>
@@ -18663,7 +18670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="157" t="s">
         <v>87</v>
       </c>
@@ -18768,7 +18775,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="157" t="s">
         <v>87</v>
       </c>
@@ -18829,7 +18836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="157" t="s">
         <v>87</v>
       </c>
@@ -18890,7 +18897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="157" t="s">
         <v>88</v>
       </c>
@@ -18979,7 +18986,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="92" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="164" t="s">
         <v>89</v>
       </c>
@@ -19036,7 +19043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="164" t="s">
         <v>89</v>
       </c>
@@ -19093,7 +19100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="164" t="s">
         <v>170</v>
       </c>
@@ -19154,7 +19161,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="164" t="s">
         <v>170</v>
       </c>
@@ -19211,7 +19218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:42" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="167" t="s">
         <v>90</v>
       </c>
@@ -19490,34 +19497,34 @@
       <c r="AG2" s="132"/>
     </row>
     <row r="3" spans="1:33" s="130" customFormat="1" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="195" t="s">
+      <c r="A3" s="198" t="s">
         <v>359</v>
       </c>
-      <c r="B3" s="195" t="s">
+      <c r="B3" s="198" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="197" t="s">
+      <c r="C3" s="200" t="s">
         <v>360</v>
       </c>
       <c r="D3" s="131" t="s">
         <v>361</v>
       </c>
-      <c r="E3" s="197" t="s">
+      <c r="E3" s="200" t="s">
         <v>362</v>
       </c>
-      <c r="F3" s="199" t="s">
+      <c r="F3" s="202" t="s">
         <v>363</v>
       </c>
-      <c r="G3" s="201" t="s">
+      <c r="G3" s="204" t="s">
         <v>364</v>
       </c>
-      <c r="H3" s="199" t="s">
+      <c r="H3" s="202" t="s">
         <v>365</v>
       </c>
-      <c r="I3" s="199" t="s">
+      <c r="I3" s="202" t="s">
         <v>366</v>
       </c>
-      <c r="J3" s="199"/>
+      <c r="J3" s="202"/>
       <c r="K3" s="128" t="s">
         <v>367</v>
       </c>
@@ -19530,57 +19537,57 @@
       <c r="N3" s="127" t="s">
         <v>370</v>
       </c>
-      <c r="O3" s="205" t="s">
+      <c r="O3" s="195" t="s">
         <v>371</v>
       </c>
-      <c r="P3" s="205"/>
-      <c r="Q3" s="205" t="s">
+      <c r="P3" s="195"/>
+      <c r="Q3" s="195" t="s">
         <v>372</v>
       </c>
-      <c r="R3" s="205"/>
-      <c r="S3" s="205" t="s">
+      <c r="R3" s="195"/>
+      <c r="S3" s="195" t="s">
         <v>373</v>
       </c>
-      <c r="T3" s="205"/>
-      <c r="U3" s="204" t="s">
+      <c r="T3" s="195"/>
+      <c r="U3" s="194" t="s">
         <v>374</v>
       </c>
-      <c r="V3" s="204"/>
-      <c r="W3" s="204" t="s">
+      <c r="V3" s="194"/>
+      <c r="W3" s="194" t="s">
         <v>375</v>
       </c>
-      <c r="X3" s="204"/>
-      <c r="Y3" s="204" t="s">
+      <c r="X3" s="194"/>
+      <c r="Y3" s="194" t="s">
         <v>376</v>
       </c>
-      <c r="Z3" s="204"/>
-      <c r="AA3" s="204" t="s">
+      <c r="Z3" s="194"/>
+      <c r="AA3" s="194" t="s">
         <v>377</v>
       </c>
-      <c r="AB3" s="204"/>
-      <c r="AC3" s="204" t="s">
+      <c r="AB3" s="194"/>
+      <c r="AC3" s="194" t="s">
         <v>378</v>
       </c>
-      <c r="AD3" s="204"/>
-      <c r="AE3" s="193" t="s">
+      <c r="AD3" s="194"/>
+      <c r="AE3" s="196" t="s">
         <v>379</v>
       </c>
-      <c r="AF3" s="194"/>
+      <c r="AF3" s="197"/>
       <c r="AG3" s="125" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="4" spans="1:33" s="124" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="196"/>
-      <c r="B4" s="196"/>
-      <c r="C4" s="198"/>
+      <c r="A4" s="199"/>
+      <c r="B4" s="199"/>
+      <c r="C4" s="201"/>
       <c r="D4" s="129"/>
-      <c r="E4" s="198"/>
-      <c r="F4" s="200"/>
-      <c r="G4" s="202"/>
-      <c r="H4" s="200"/>
-      <c r="I4" s="200"/>
-      <c r="J4" s="200"/>
+      <c r="E4" s="201"/>
+      <c r="F4" s="203"/>
+      <c r="G4" s="205"/>
+      <c r="H4" s="203"/>
+      <c r="I4" s="203"/>
+      <c r="J4" s="203"/>
       <c r="K4" s="128"/>
       <c r="L4" s="128"/>
       <c r="M4" s="128"/>
@@ -20664,7 +20671,7 @@
       <c r="E25" s="104" t="s">
         <v>454</v>
       </c>
-      <c r="I25" s="203"/>
+      <c r="I25" s="193"/>
       <c r="J25" s="57"/>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.25">
@@ -20674,7 +20681,7 @@
       <c r="E26" s="103" t="s">
         <v>455</v>
       </c>
-      <c r="I26" s="203"/>
+      <c r="I26" s="193"/>
       <c r="J26" s="57"/>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
@@ -20684,7 +20691,7 @@
       <c r="E27" s="104" t="s">
         <v>457</v>
       </c>
-      <c r="I27" s="203"/>
+      <c r="I27" s="193"/>
       <c r="J27" s="57"/>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
@@ -20694,7 +20701,7 @@
       <c r="E28" s="104" t="s">
         <v>458</v>
       </c>
-      <c r="I28" s="203"/>
+      <c r="I28" s="193"/>
       <c r="J28" s="57"/>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
@@ -20728,15 +20735,6 @@
     <filterColumn colId="28" showButton="0"/>
   </autoFilter>
   <mergeCells count="19">
-    <mergeCell ref="I25:I28"/>
-    <mergeCell ref="AC3:AD3"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="W3:X3"/>
-    <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="AA3:AB3"/>
     <mergeCell ref="AE3:AF3"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -20747,6 +20745,15 @@
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
+    <mergeCell ref="I25:I28"/>
+    <mergeCell ref="AC3:AD3"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="Y3:Z3"/>
+    <mergeCell ref="AA3:AB3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -21097,7 +21104,7 @@
       </c>
       <c r="E26" s="28"/>
     </row>
-    <row r="27" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" s="26" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="92"/>
       <c r="B27" s="90"/>
       <c r="C27" s="88" t="s">
@@ -21295,18 +21302,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="222" t="s">
+      <c r="B1" s="215" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="222"/>
-      <c r="D1" s="222"/>
-      <c r="E1" s="222"/>
-      <c r="F1" s="222"/>
-      <c r="G1" s="222"/>
-      <c r="H1" s="222"/>
-      <c r="I1" s="222"/>
-      <c r="J1" s="222"/>
-      <c r="K1" s="222"/>
+      <c r="C1" s="215"/>
+      <c r="D1" s="215"/>
+      <c r="E1" s="215"/>
+      <c r="F1" s="215"/>
+      <c r="G1" s="215"/>
+      <c r="H1" s="215"/>
+      <c r="I1" s="215"/>
+      <c r="J1" s="215"/>
+      <c r="K1" s="215"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" spans="2:12" ht="36" x14ac:dyDescent="0.25">
@@ -21332,7 +21339,7 @@
       <c r="L2" s="44"/>
     </row>
     <row r="3" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="218" t="s">
+      <c r="B3" s="216" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="97" t="s">
@@ -21349,7 +21356,7 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="215"/>
+      <c r="B4" s="217"/>
       <c r="C4" s="97" t="s">
         <v>14</v>
       </c>
@@ -21364,7 +21371,7 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="215"/>
+      <c r="B5" s="217"/>
       <c r="C5" s="97" t="s">
         <v>257</v>
       </c>
@@ -21379,7 +21386,7 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="219"/>
+      <c r="B6" s="218"/>
       <c r="C6" s="97" t="s">
         <v>259</v>
       </c>
@@ -21411,7 +21418,7 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="215" t="s">
+      <c r="B8" s="217" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="94" t="s">
@@ -21428,7 +21435,7 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="215"/>
+      <c r="B9" s="217"/>
       <c r="C9" s="93" t="s">
         <v>67</v>
       </c>
@@ -21443,7 +21450,7 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="223" t="s">
+      <c r="B10" s="219" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="98" t="s">
@@ -21460,7 +21467,7 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="224"/>
+      <c r="B11" s="220"/>
       <c r="C11" s="98" t="s">
         <v>26</v>
       </c>
@@ -21475,7 +21482,7 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="224"/>
+      <c r="B12" s="220"/>
       <c r="C12" s="98" t="s">
         <v>27</v>
       </c>
@@ -21490,7 +21497,7 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="225"/>
+      <c r="B13" s="221"/>
       <c r="C13" s="98" t="s">
         <v>267</v>
       </c>
@@ -21505,7 +21512,7 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="218" t="s">
+      <c r="B14" s="216" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="60" t="s">
@@ -21522,7 +21529,7 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="215"/>
+      <c r="B15" s="217"/>
       <c r="C15" s="60" t="s">
         <v>29</v>
       </c>
@@ -21537,7 +21544,7 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="215"/>
+      <c r="B16" s="217"/>
       <c r="C16" s="60" t="s">
         <v>271</v>
       </c>
@@ -21552,7 +21559,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="219"/>
+      <c r="B17" s="218"/>
       <c r="C17" s="61" t="s">
         <v>267</v>
       </c>
@@ -21567,7 +21574,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="216" t="s">
+      <c r="B18" s="223" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="59" t="s">
@@ -21584,7 +21591,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="217"/>
+      <c r="B19" s="224"/>
       <c r="C19" s="2" t="s">
         <v>67</v>
       </c>
@@ -21599,7 +21606,7 @@
       </c>
     </row>
     <row r="20" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="215" t="s">
+      <c r="B20" s="217" t="s">
         <v>34</v>
       </c>
       <c r="C20" s="62" t="s">
@@ -21616,7 +21623,7 @@
       </c>
     </row>
     <row r="21" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="215"/>
+      <c r="B21" s="217"/>
       <c r="C21" s="60" t="s">
         <v>27</v>
       </c>
@@ -21631,7 +21638,7 @@
       </c>
     </row>
     <row r="22" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="215"/>
+      <c r="B22" s="217"/>
       <c r="C22" s="60" t="s">
         <v>277</v>
       </c>
@@ -21646,7 +21653,7 @@
       </c>
     </row>
     <row r="23" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="215"/>
+      <c r="B23" s="217"/>
       <c r="C23" s="61" t="s">
         <v>279</v>
       </c>
@@ -21661,7 +21668,7 @@
       </c>
     </row>
     <row r="24" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="223" t="s">
+      <c r="B24" s="219" t="s">
         <v>38</v>
       </c>
       <c r="C24" s="63" t="s">
@@ -21678,7 +21685,7 @@
       </c>
     </row>
     <row r="25" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="224"/>
+      <c r="B25" s="220"/>
       <c r="C25" s="63" t="s">
         <v>39</v>
       </c>
@@ -21693,7 +21700,7 @@
       </c>
     </row>
     <row r="26" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="224"/>
+      <c r="B26" s="220"/>
       <c r="C26" s="63" t="s">
         <v>40</v>
       </c>
@@ -21708,7 +21715,7 @@
       </c>
     </row>
     <row r="27" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="224"/>
+      <c r="B27" s="220"/>
       <c r="C27" s="63" t="s">
         <v>41</v>
       </c>
@@ -21723,7 +21730,7 @@
       </c>
     </row>
     <row r="28" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="224"/>
+      <c r="B28" s="220"/>
       <c r="C28" s="63" t="s">
         <v>285</v>
       </c>
@@ -21738,7 +21745,7 @@
       </c>
     </row>
     <row r="29" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="224"/>
+      <c r="B29" s="220"/>
       <c r="C29" s="63" t="s">
         <v>267</v>
       </c>
@@ -21753,7 +21760,7 @@
       </c>
     </row>
     <row r="30" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="225"/>
+      <c r="B30" s="221"/>
       <c r="C30" s="63" t="s">
         <v>279</v>
       </c>
@@ -21768,7 +21775,7 @@
       </c>
     </row>
     <row r="31" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="215" t="s">
+      <c r="B31" s="217" t="s">
         <v>43</v>
       </c>
       <c r="C31" s="12" t="s">
@@ -21785,7 +21792,7 @@
       </c>
     </row>
     <row r="32" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="215"/>
+      <c r="B32" s="217"/>
       <c r="C32" s="97" t="s">
         <v>45</v>
       </c>
@@ -21800,7 +21807,7 @@
       </c>
     </row>
     <row r="33" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="215"/>
+      <c r="B33" s="217"/>
       <c r="C33" s="97" t="s">
         <v>40</v>
       </c>
@@ -21815,7 +21822,7 @@
       </c>
     </row>
     <row r="34" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="215"/>
+      <c r="B34" s="217"/>
       <c r="C34" s="93" t="s">
         <v>259</v>
       </c>
@@ -21830,7 +21837,7 @@
       </c>
     </row>
     <row r="35" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="220" t="s">
+      <c r="B35" s="225" t="s">
         <v>48</v>
       </c>
       <c r="C35" s="98" t="s">
@@ -21847,7 +21854,7 @@
       </c>
     </row>
     <row r="36" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="220"/>
+      <c r="B36" s="225"/>
       <c r="C36" s="98" t="s">
         <v>49</v>
       </c>
@@ -21862,7 +21869,7 @@
       </c>
     </row>
     <row r="37" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="220"/>
+      <c r="B37" s="225"/>
       <c r="C37" s="98" t="s">
         <v>293</v>
       </c>
@@ -21877,7 +21884,7 @@
       </c>
     </row>
     <row r="38" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="220"/>
+      <c r="B38" s="225"/>
       <c r="C38" s="98" t="s">
         <v>267</v>
       </c>
@@ -21892,7 +21899,7 @@
       </c>
     </row>
     <row r="39" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="219" t="s">
+      <c r="B39" s="218" t="s">
         <v>53</v>
       </c>
       <c r="C39" s="94" t="s">
@@ -21909,7 +21916,7 @@
       </c>
     </row>
     <row r="40" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="218"/>
+      <c r="B40" s="216"/>
       <c r="C40" s="93" t="s">
         <v>57</v>
       </c>
@@ -21924,7 +21931,7 @@
       </c>
     </row>
     <row r="41" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="223" t="s">
+      <c r="B41" s="219" t="s">
         <v>58</v>
       </c>
       <c r="C41" s="98" t="s">
@@ -21941,7 +21948,7 @@
       </c>
     </row>
     <row r="42" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="224"/>
+      <c r="B42" s="220"/>
       <c r="C42" s="98" t="s">
         <v>60</v>
       </c>
@@ -21956,7 +21963,7 @@
       </c>
     </row>
     <row r="43" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="224"/>
+      <c r="B43" s="220"/>
       <c r="C43" s="98" t="s">
         <v>62</v>
       </c>
@@ -21971,7 +21978,7 @@
       </c>
     </row>
     <row r="44" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="224"/>
+      <c r="B44" s="220"/>
       <c r="C44" s="98" t="s">
         <v>300</v>
       </c>
@@ -21986,7 +21993,7 @@
       </c>
     </row>
     <row r="45" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="225"/>
+      <c r="B45" s="221"/>
       <c r="C45" s="98" t="s">
         <v>267</v>
       </c>
@@ -22001,7 +22008,7 @@
       </c>
     </row>
     <row r="46" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="218" t="s">
+      <c r="B46" s="216" t="s">
         <v>170</v>
       </c>
       <c r="C46" s="64" t="s">
@@ -22018,7 +22025,7 @@
       </c>
     </row>
     <row r="47" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="215"/>
+      <c r="B47" s="217"/>
       <c r="C47" s="64" t="s">
         <v>259</v>
       </c>
@@ -22033,7 +22040,7 @@
       </c>
     </row>
     <row r="48" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="215"/>
+      <c r="B48" s="217"/>
       <c r="C48" s="64" t="s">
         <v>267</v>
       </c>
@@ -22048,7 +22055,7 @@
       </c>
     </row>
     <row r="49" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="219"/>
+      <c r="B49" s="218"/>
       <c r="C49" s="64" t="s">
         <v>16</v>
       </c>
@@ -22063,7 +22070,7 @@
       </c>
     </row>
     <row r="50" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="218" t="s">
+      <c r="B50" s="216" t="s">
         <v>63</v>
       </c>
       <c r="C50" s="64" t="s">
@@ -22080,7 +22087,7 @@
       </c>
     </row>
     <row r="51" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="215"/>
+      <c r="B51" s="217"/>
       <c r="C51" s="64" t="s">
         <v>59</v>
       </c>
@@ -22095,7 +22102,7 @@
       </c>
     </row>
     <row r="52" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="219"/>
+      <c r="B52" s="218"/>
       <c r="C52" s="64" t="s">
         <v>267</v>
       </c>
@@ -22110,7 +22117,7 @@
       </c>
     </row>
     <row r="53" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="224" t="s">
+      <c r="B53" s="220" t="s">
         <v>154</v>
       </c>
       <c r="C53" s="96" t="s">
@@ -22127,7 +22134,7 @@
       </c>
     </row>
     <row r="54" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="224"/>
+      <c r="B54" s="220"/>
       <c r="C54" s="98" t="s">
         <v>155</v>
       </c>
@@ -22142,7 +22149,7 @@
       </c>
     </row>
     <row r="55" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="224"/>
+      <c r="B55" s="220"/>
       <c r="C55" s="95" t="s">
         <v>267</v>
       </c>
@@ -22157,7 +22164,7 @@
       </c>
     </row>
     <row r="56" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="218" t="s">
+      <c r="B56" s="216" t="s">
         <v>65</v>
       </c>
       <c r="C56" s="97" t="s">
@@ -22174,7 +22181,7 @@
       </c>
     </row>
     <row r="57" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="215"/>
+      <c r="B57" s="217"/>
       <c r="C57" s="97" t="s">
         <v>67</v>
       </c>
@@ -22189,7 +22196,7 @@
       </c>
     </row>
     <row r="58" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="219"/>
+      <c r="B58" s="218"/>
       <c r="C58" s="97" t="s">
         <v>259</v>
       </c>
@@ -22204,7 +22211,7 @@
       </c>
     </row>
     <row r="59" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="223" t="s">
+      <c r="B59" s="219" t="s">
         <v>68</v>
       </c>
       <c r="C59" s="98" t="s">
@@ -22221,7 +22228,7 @@
       </c>
     </row>
     <row r="60" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="224"/>
+      <c r="B60" s="220"/>
       <c r="C60" s="98" t="s">
         <v>27</v>
       </c>
@@ -22236,7 +22243,7 @@
       </c>
     </row>
     <row r="61" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="224"/>
+      <c r="B61" s="220"/>
       <c r="C61" s="98" t="s">
         <v>316</v>
       </c>
@@ -22251,7 +22258,7 @@
       </c>
     </row>
     <row r="62" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="224"/>
+      <c r="B62" s="220"/>
       <c r="C62" s="98" t="s">
         <v>318</v>
       </c>
@@ -22266,7 +22273,7 @@
       </c>
     </row>
     <row r="63" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="224"/>
+      <c r="B63" s="220"/>
       <c r="C63" s="98" t="s">
         <v>320</v>
       </c>
@@ -22281,7 +22288,7 @@
       </c>
     </row>
     <row r="64" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="224"/>
+      <c r="B64" s="220"/>
       <c r="C64" s="98" t="s">
         <v>322</v>
       </c>
@@ -22296,7 +22303,7 @@
       </c>
     </row>
     <row r="65" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="225"/>
+      <c r="B65" s="221"/>
       <c r="C65" s="98" t="s">
         <v>324</v>
       </c>
@@ -22311,7 +22318,7 @@
       </c>
     </row>
     <row r="66" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="218" t="s">
+      <c r="B66" s="216" t="s">
         <v>73</v>
       </c>
       <c r="C66" s="94" t="s">
@@ -22328,7 +22335,7 @@
       </c>
     </row>
     <row r="67" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="215"/>
+      <c r="B67" s="217"/>
       <c r="C67" s="97" t="s">
         <v>74</v>
       </c>
@@ -22343,7 +22350,7 @@
       </c>
     </row>
     <row r="68" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="215"/>
+      <c r="B68" s="217"/>
       <c r="C68" s="97" t="s">
         <v>327</v>
       </c>
@@ -22358,7 +22365,7 @@
       </c>
     </row>
     <row r="69" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="219"/>
+      <c r="B69" s="218"/>
       <c r="C69" s="93" t="s">
         <v>267</v>
       </c>
@@ -22373,7 +22380,7 @@
       </c>
     </row>
     <row r="70" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="223" t="s">
+      <c r="B70" s="219" t="s">
         <v>76</v>
       </c>
       <c r="C70" s="98" t="s">
@@ -22390,7 +22397,7 @@
       </c>
     </row>
     <row r="71" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="224"/>
+      <c r="B71" s="220"/>
       <c r="C71" s="98" t="s">
         <v>44</v>
       </c>
@@ -22405,7 +22412,7 @@
       </c>
     </row>
     <row r="72" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="224"/>
+      <c r="B72" s="220"/>
       <c r="C72" s="98" t="s">
         <v>332</v>
       </c>
@@ -22420,7 +22427,7 @@
       </c>
     </row>
     <row r="73" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="224"/>
+      <c r="B73" s="220"/>
       <c r="C73" s="98" t="s">
         <v>334</v>
       </c>
@@ -22435,7 +22442,7 @@
       </c>
     </row>
     <row r="74" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="225"/>
+      <c r="B74" s="221"/>
       <c r="C74" s="98" t="s">
         <v>82</v>
       </c>
@@ -22450,7 +22457,7 @@
       </c>
     </row>
     <row r="75" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="219" t="s">
+      <c r="B75" s="218" t="s">
         <v>79</v>
       </c>
       <c r="C75" s="94" t="s">
@@ -22467,7 +22474,7 @@
       </c>
     </row>
     <row r="76" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="221"/>
+      <c r="B76" s="222"/>
       <c r="C76" s="97" t="s">
         <v>26</v>
       </c>
@@ -22482,7 +22489,7 @@
       </c>
     </row>
     <row r="77" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="218"/>
+      <c r="B77" s="216"/>
       <c r="C77" s="93" t="s">
         <v>9</v>
       </c>
@@ -22497,7 +22504,7 @@
       </c>
     </row>
     <row r="78" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="218"/>
+      <c r="B78" s="216"/>
       <c r="C78" s="93" t="s">
         <v>82</v>
       </c>
@@ -22512,7 +22519,7 @@
       </c>
     </row>
     <row r="79" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="223" t="s">
+      <c r="B79" s="219" t="s">
         <v>83</v>
       </c>
       <c r="C79" s="98" t="s">
@@ -22529,7 +22536,7 @@
       </c>
     </row>
     <row r="80" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="224"/>
+      <c r="B80" s="220"/>
       <c r="C80" s="98" t="s">
         <v>84</v>
       </c>
@@ -22544,7 +22551,7 @@
       </c>
     </row>
     <row r="81" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="224"/>
+      <c r="B81" s="220"/>
       <c r="C81" s="98" t="s">
         <v>342</v>
       </c>
@@ -22559,7 +22566,7 @@
       </c>
     </row>
     <row r="82" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="225"/>
+      <c r="B82" s="221"/>
       <c r="C82" s="98" t="s">
         <v>267</v>
       </c>
@@ -22574,7 +22581,7 @@
       </c>
     </row>
     <row r="83" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="215" t="s">
+      <c r="B83" s="217" t="s">
         <v>85</v>
       </c>
       <c r="C83" s="94" t="s">
@@ -22591,7 +22598,7 @@
       </c>
     </row>
     <row r="84" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="215"/>
+      <c r="B84" s="217"/>
       <c r="C84" s="93" t="s">
         <v>345</v>
       </c>
@@ -22606,7 +22613,7 @@
       </c>
     </row>
     <row r="85" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="216" t="s">
+      <c r="B85" s="223" t="s">
         <v>89</v>
       </c>
       <c r="C85" s="98" t="s">
@@ -22623,7 +22630,7 @@
       </c>
     </row>
     <row r="86" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="217"/>
+      <c r="B86" s="224"/>
       <c r="C86" s="2" t="s">
         <v>67</v>
       </c>
@@ -22638,7 +22645,7 @@
       </c>
     </row>
     <row r="87" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="215" t="s">
+      <c r="B87" s="217" t="s">
         <v>88</v>
       </c>
       <c r="C87" s="94" t="s">
@@ -22655,7 +22662,7 @@
       </c>
     </row>
     <row r="88" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B88" s="215"/>
+      <c r="B88" s="217"/>
       <c r="C88" s="97" t="s">
         <v>349</v>
       </c>
@@ -22670,7 +22677,7 @@
       </c>
     </row>
     <row r="89" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B89" s="215"/>
+      <c r="B89" s="217"/>
       <c r="C89" s="97" t="s">
         <v>259</v>
       </c>
@@ -22685,7 +22692,7 @@
       </c>
     </row>
     <row r="90" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="215"/>
+      <c r="B90" s="217"/>
       <c r="C90" s="93" t="s">
         <v>67</v>
       </c>
@@ -22717,7 +22724,7 @@
       </c>
     </row>
     <row r="92" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="221" t="s">
+      <c r="B92" s="222" t="s">
         <v>87</v>
       </c>
       <c r="C92" s="94" t="s">
@@ -22734,7 +22741,7 @@
       </c>
     </row>
     <row r="93" spans="2:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B93" s="221"/>
+      <c r="B93" s="222"/>
       <c r="C93" s="94" t="s">
         <v>59</v>
       </c>
@@ -22750,6 +22757,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B87:B90"/>
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="B66:B69"/>
     <mergeCell ref="B70:B74"/>
@@ -22766,15 +22782,6 @@
     <mergeCell ref="B24:B30"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B35:B38"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B87:B90"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
@@ -22820,15 +22827,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100498A226200FBA747BF499A3F16BD9306" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a802e24b83766cc1d8af855be1bd7937">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f" xmlns:ns3="c84b764c-50f3-4666-981f-a21c15460b9f" xmlns:ns4="cdc7663a-08f0-4737-9e8c-148ce897a09c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6e8a154215ca5c893126bc8f6b108500" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="c41eb0e2-a8ee-4193-9a69-ff6e1e787a8f"/>
@@ -23076,6 +23074,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{283029C9-A5AB-4AAC-9B8A-368CAB8C733A}">
   <ds:schemaRefs>
@@ -23089,14 +23096,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5341BEEE-99C0-4ED9-8E19-6F685D668845}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8D9694B-F156-44C8-A40A-23B2416BDA15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23114,4 +23113,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5341BEEE-99C0-4ED9-8E19-6F685D668845}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>